<commit_message>
SOCO: Feature: Control calibration state machine via modbus
Now, it's possible to do automatated calibration via controlling
calibration state machine over modbus.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2535" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2547" uniqueCount="365">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -1016,6 +1016,66 @@
 If set to non-zero, indicates product was calibrated during production</t>
   </si>
   <si>
+    <t xml:space="preserve">Calibration State</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50013</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Internal Only. Not visible to customer. 
+Indicates the state machine of calibration
+0: Calibration Not Initiated. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 20A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. Set Fan 1 Current and Fan 2 current to 0.1A each. And then s</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">et Advance Calibration Flag.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+16,17,18,19: High Point Calibration In Progress
+20: High Point Calibration Done. </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
+21,22,23: Mid Point Calibration In Progress
+24: Mid Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 0.4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
+25,26,27: Low Point Calibration In Progress
+127: Calibration Completed Successfully
+126: Error occured during calibration. Please restart controller</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">READ COIL STATUS (Function Code: 0x01)</t>
   </si>
   <si>
@@ -1097,10 +1157,90 @@
     <t xml:space="preserve">WRITE SINGLE COIL STATUS (Function Code: 0x05)</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Internal Only. Not visible to customer.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Only writtable when test mode enabled.</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Restart Controller</t>
   </si>
   <si>
-    <t xml:space="preserve">Internal Only. Not visible to customer. </t>
+    <t xml:space="preserve">Internal Only. Not visible to customer. 
+Only writtable when test mode enabled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal Only. Not visible to customer. 
+If set to non-zero, indicates product was tested functionally during production. Only writtable when test mode enabled.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Internal Only. Not visible to customer. 
+If set to non-zero, indicates product was calibrated during production. </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Only writtable when test mode enabled.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Advance Calibration State</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Internal Only. Not visible to customer. 
+If set to non-zero, it advances the calibration state machine when it is waiting for external input. </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Only writtable when test mode enabled.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -7226,7 +7366,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I259"/>
+  <dimension ref="A1:I261"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.94"/>
@@ -10223,99 +10363,101 @@
         <v>327</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A114" s="3" t="s">
+    <row r="114" customFormat="false" ht="236.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="B114" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C114" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D114" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E114" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G114" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="H114" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I114" s="12" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B114" s="4" t="s">
+      <c r="B115" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C114" s="4" t="s">
+      <c r="C115" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D114" s="3" t="s">
+      <c r="D115" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E114" s="4" t="s">
+      <c r="E115" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F114" s="3" t="s">
+      <c r="F115" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G114" s="4" t="s">
+      <c r="G115" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H114" s="4" t="s">
+      <c r="H115" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I114" s="3" t="s">
+      <c r="I115" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="3"/>
-      <c r="B115" s="4" t="s">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3"/>
+      <c r="B116" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C115" s="4" t="s">
+      <c r="C116" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D115" s="3"/>
-      <c r="E115" s="4" t="s">
+      <c r="D116" s="3"/>
+      <c r="E116" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F115" s="3"/>
-      <c r="G115" s="4" t="s">
+      <c r="F116" s="3"/>
+      <c r="G116" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H115" s="4" t="s">
+      <c r="H116" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I115" s="3"/>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="5" t="s">
+      <c r="I116" s="3"/>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="B116" s="5"/>
-      <c r="C116" s="5"/>
-      <c r="D116" s="5"/>
-      <c r="E116" s="5"/>
-      <c r="F116" s="5"/>
-      <c r="G116" s="5"/>
-      <c r="H116" s="5"/>
-      <c r="I116" s="5"/>
-    </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="7" t="s">
-        <v>246</v>
-      </c>
-      <c r="B117" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C117" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D117" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E117" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F117" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G117" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H117" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I117" s="7"/>
+      <c r="B117" s="5"/>
+      <c r="C117" s="5"/>
+      <c r="D117" s="5"/>
+      <c r="E117" s="5"/>
+      <c r="F117" s="5"/>
+      <c r="G117" s="5"/>
+      <c r="H117" s="5"/>
+      <c r="I117" s="5"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="7" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B118" s="7" t="s">
         <v>75</v>
@@ -10333,7 +10475,7 @@
         <v>248</v>
       </c>
       <c r="G118" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H118" s="7" t="n">
         <v>1</v>
@@ -10342,7 +10484,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="7" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B119" s="7" t="s">
         <v>75</v>
@@ -10360,7 +10502,7 @@
         <v>248</v>
       </c>
       <c r="G119" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H119" s="7" t="n">
         <v>1</v>
@@ -10369,7 +10511,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B120" s="7" t="s">
         <v>75</v>
@@ -10387,7 +10529,7 @@
         <v>248</v>
       </c>
       <c r="G120" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H120" s="7" t="n">
         <v>1</v>
@@ -10396,7 +10538,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B121" s="7" t="s">
         <v>75</v>
@@ -10414,7 +10556,7 @@
         <v>248</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H121" s="7" t="n">
         <v>1</v>
@@ -10423,7 +10565,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B122" s="7" t="s">
         <v>75</v>
@@ -10441,7 +10583,7 @@
         <v>248</v>
       </c>
       <c r="G122" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H122" s="7" t="n">
         <v>1</v>
@@ -10450,7 +10592,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B123" s="7" t="s">
         <v>75</v>
@@ -10468,7 +10610,7 @@
         <v>248</v>
       </c>
       <c r="G123" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H123" s="7" t="n">
         <v>1</v>
@@ -10477,7 +10619,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B124" s="7" t="s">
         <v>75</v>
@@ -10495,7 +10637,7 @@
         <v>248</v>
       </c>
       <c r="G124" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H124" s="7" t="n">
         <v>1</v>
@@ -10504,7 +10646,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B125" s="7" t="s">
         <v>75</v>
@@ -10522,7 +10664,7 @@
         <v>248</v>
       </c>
       <c r="G125" s="7" t="n">
-        <v>201</v>
+        <v>8</v>
       </c>
       <c r="H125" s="7" t="n">
         <v>1</v>
@@ -10531,7 +10673,7 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B126" s="7" t="s">
         <v>75</v>
@@ -10549,7 +10691,7 @@
         <v>248</v>
       </c>
       <c r="G126" s="7" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H126" s="7" t="n">
         <v>1</v>
@@ -10558,7 +10700,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B127" s="7" t="s">
         <v>75</v>
@@ -10576,7 +10718,7 @@
         <v>248</v>
       </c>
       <c r="G127" s="7" t="n">
-        <v>301</v>
+        <v>202</v>
       </c>
       <c r="H127" s="7" t="n">
         <v>1</v>
@@ -10585,7 +10727,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B128" s="7" t="s">
         <v>75</v>
@@ -10603,7 +10745,7 @@
         <v>248</v>
       </c>
       <c r="G128" s="7" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H128" s="7" t="n">
         <v>1</v>
@@ -10612,7 +10754,7 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B129" s="7" t="s">
         <v>75</v>
@@ -10630,7 +10772,7 @@
         <v>248</v>
       </c>
       <c r="G129" s="7" t="n">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H129" s="7" t="n">
         <v>1</v>
@@ -10639,7 +10781,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B130" s="7" t="s">
         <v>75</v>
@@ -10657,7 +10799,7 @@
         <v>248</v>
       </c>
       <c r="G130" s="7" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H130" s="7" t="n">
         <v>1</v>
@@ -10666,7 +10808,7 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B131" s="7" t="s">
         <v>75</v>
@@ -10684,7 +10826,7 @@
         <v>248</v>
       </c>
       <c r="G131" s="7" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H131" s="7" t="n">
         <v>1</v>
@@ -10693,7 +10835,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B132" s="7" t="s">
         <v>75</v>
@@ -10711,7 +10853,7 @@
         <v>248</v>
       </c>
       <c r="G132" s="7" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H132" s="7" t="n">
         <v>1</v>
@@ -10720,7 +10862,7 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B133" s="7" t="s">
         <v>75</v>
@@ -10738,7 +10880,7 @@
         <v>248</v>
       </c>
       <c r="G133" s="7" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H133" s="7" t="n">
         <v>1</v>
@@ -10747,7 +10889,7 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B134" s="7" t="s">
         <v>75</v>
@@ -10765,7 +10907,7 @@
         <v>248</v>
       </c>
       <c r="G134" s="7" t="n">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H134" s="7" t="n">
         <v>1</v>
@@ -10774,7 +10916,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="7" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B135" s="7" t="s">
         <v>75</v>
@@ -10792,7 +10934,7 @@
         <v>248</v>
       </c>
       <c r="G135" s="7" t="n">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H135" s="7" t="n">
         <v>1</v>
@@ -10801,7 +10943,7 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B136" s="7" t="s">
         <v>75</v>
@@ -10819,7 +10961,7 @@
         <v>248</v>
       </c>
       <c r="G136" s="7" t="n">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H136" s="7" t="n">
         <v>1</v>
@@ -10828,7 +10970,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B137" s="7" t="s">
         <v>75</v>
@@ -10846,7 +10988,7 @@
         <v>248</v>
       </c>
       <c r="G137" s="7" t="n">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H137" s="7" t="n">
         <v>1</v>
@@ -10855,7 +10997,7 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B138" s="7" t="s">
         <v>75</v>
@@ -10873,7 +11015,7 @@
         <v>248</v>
       </c>
       <c r="G138" s="7" t="n">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H138" s="7" t="n">
         <v>1</v>
@@ -10882,7 +11024,7 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B139" s="7" t="s">
         <v>75</v>
@@ -10900,7 +11042,7 @@
         <v>248</v>
       </c>
       <c r="G139" s="7" t="n">
-        <v>401</v>
+        <v>312</v>
       </c>
       <c r="H139" s="7" t="n">
         <v>1</v>
@@ -10909,7 +11051,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B140" s="7" t="s">
         <v>75</v>
@@ -10927,7 +11069,7 @@
         <v>248</v>
       </c>
       <c r="G140" s="7" t="n">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H140" s="7" t="n">
         <v>1</v>
@@ -10936,7 +11078,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B141" s="7" t="s">
         <v>75</v>
@@ -10954,7 +11096,7 @@
         <v>248</v>
       </c>
       <c r="G141" s="7" t="n">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H141" s="7" t="n">
         <v>1</v>
@@ -10963,7 +11105,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="7" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B142" s="7" t="s">
         <v>75</v>
@@ -10981,7 +11123,7 @@
         <v>248</v>
       </c>
       <c r="G142" s="7" t="n">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="H142" s="7" t="n">
         <v>1</v>
@@ -10990,7 +11132,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B143" s="7" t="s">
         <v>75</v>
@@ -11008,7 +11150,7 @@
         <v>248</v>
       </c>
       <c r="G143" s="7" t="n">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="H143" s="7" t="n">
         <v>1</v>
@@ -11017,7 +11159,7 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B144" s="7" t="s">
         <v>75</v>
@@ -11035,7 +11177,7 @@
         <v>248</v>
       </c>
       <c r="G144" s="7" t="n">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="H144" s="7" t="n">
         <v>1</v>
@@ -11044,7 +11186,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B145" s="7" t="s">
         <v>75</v>
@@ -11062,7 +11204,7 @@
         <v>248</v>
       </c>
       <c r="G145" s="7" t="n">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="H145" s="7" t="n">
         <v>1</v>
@@ -11071,7 +11213,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B146" s="7" t="s">
         <v>75</v>
@@ -11089,7 +11231,7 @@
         <v>248</v>
       </c>
       <c r="G146" s="7" t="n">
-        <v>501</v>
+        <v>407</v>
       </c>
       <c r="H146" s="7" t="n">
         <v>1</v>
@@ -11098,7 +11240,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B147" s="7" t="s">
         <v>75</v>
@@ -11116,7 +11258,7 @@
         <v>248</v>
       </c>
       <c r="G147" s="7" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="H147" s="7" t="n">
         <v>1</v>
@@ -11125,7 +11267,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B148" s="7" t="s">
         <v>75</v>
@@ -11143,7 +11285,7 @@
         <v>248</v>
       </c>
       <c r="G148" s="7" t="n">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="H148" s="7" t="n">
         <v>1</v>
@@ -11152,7 +11294,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B149" s="7" t="s">
         <v>75</v>
@@ -11170,7 +11312,7 @@
         <v>248</v>
       </c>
       <c r="G149" s="7" t="n">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="H149" s="7" t="n">
         <v>1</v>
@@ -11179,7 +11321,7 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="7" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B150" s="7" t="s">
         <v>75</v>
@@ -11197,7 +11339,7 @@
         <v>248</v>
       </c>
       <c r="G150" s="7" t="n">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="H150" s="7" t="n">
         <v>1</v>
@@ -11206,7 +11348,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="7" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B151" s="7" t="s">
         <v>75</v>
@@ -11224,7 +11366,7 @@
         <v>248</v>
       </c>
       <c r="G151" s="7" t="n">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="H151" s="7" t="n">
         <v>1</v>
@@ -11233,7 +11375,7 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B152" s="7" t="s">
         <v>75</v>
@@ -11251,7 +11393,7 @@
         <v>248</v>
       </c>
       <c r="G152" s="7" t="n">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="H152" s="7" t="n">
         <v>1</v>
@@ -11260,7 +11402,7 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B153" s="7" t="s">
         <v>75</v>
@@ -11278,7 +11420,7 @@
         <v>248</v>
       </c>
       <c r="G153" s="7" t="n">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="H153" s="7" t="n">
         <v>1</v>
@@ -11287,7 +11429,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="7" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B154" s="7" t="s">
         <v>75</v>
@@ -11305,7 +11447,7 @@
         <v>248</v>
       </c>
       <c r="G154" s="7" t="n">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="H154" s="7" t="n">
         <v>1</v>
@@ -11314,7 +11456,7 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B155" s="7" t="s">
         <v>75</v>
@@ -11332,7 +11474,7 @@
         <v>248</v>
       </c>
       <c r="G155" s="7" t="n">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H155" s="7" t="n">
         <v>1</v>
@@ -11341,7 +11483,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B156" s="7" t="s">
         <v>75</v>
@@ -11359,7 +11501,7 @@
         <v>248</v>
       </c>
       <c r="G156" s="7" t="n">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H156" s="7" t="n">
         <v>1</v>
@@ -11368,7 +11510,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="7" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B157" s="7" t="s">
         <v>75</v>
@@ -11386,7 +11528,7 @@
         <v>248</v>
       </c>
       <c r="G157" s="7" t="n">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H157" s="7" t="n">
         <v>1</v>
@@ -11395,7 +11537,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B158" s="7" t="s">
         <v>75</v>
@@ -11413,7 +11555,7 @@
         <v>248</v>
       </c>
       <c r="G158" s="7" t="n">
-        <v>601</v>
+        <v>512</v>
       </c>
       <c r="H158" s="7" t="n">
         <v>1</v>
@@ -11422,7 +11564,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B159" s="7" t="s">
         <v>75</v>
@@ -11440,7 +11582,7 @@
         <v>248</v>
       </c>
       <c r="G159" s="7" t="n">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="H159" s="7" t="n">
         <v>1</v>
@@ -11449,7 +11591,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B160" s="7" t="s">
         <v>75</v>
@@ -11467,7 +11609,7 @@
         <v>248</v>
       </c>
       <c r="G160" s="7" t="n">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="H160" s="7" t="n">
         <v>1</v>
@@ -11476,7 +11618,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="7" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B161" s="7" t="s">
         <v>75</v>
@@ -11494,7 +11636,7 @@
         <v>248</v>
       </c>
       <c r="G161" s="7" t="n">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="H161" s="7" t="n">
         <v>1</v>
@@ -11503,7 +11645,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B162" s="7" t="s">
         <v>75</v>
@@ -11521,7 +11663,7 @@
         <v>248</v>
       </c>
       <c r="G162" s="7" t="n">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="H162" s="7" t="n">
         <v>1</v>
@@ -11530,7 +11672,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B163" s="7" t="s">
         <v>75</v>
@@ -11548,7 +11690,7 @@
         <v>248</v>
       </c>
       <c r="G163" s="7" t="n">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="H163" s="7" t="n">
         <v>1</v>
@@ -11557,7 +11699,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B164" s="7" t="s">
         <v>75</v>
@@ -11575,7 +11717,7 @@
         <v>248</v>
       </c>
       <c r="G164" s="7" t="n">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="H164" s="7" t="n">
         <v>1</v>
@@ -11584,7 +11726,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B165" s="7" t="s">
         <v>75</v>
@@ -11602,7 +11744,7 @@
         <v>248</v>
       </c>
       <c r="G165" s="7" t="n">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H165" s="7" t="n">
         <v>1</v>
@@ -11611,7 +11753,7 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B166" s="7" t="s">
         <v>75</v>
@@ -11629,7 +11771,7 @@
         <v>248</v>
       </c>
       <c r="G166" s="7" t="n">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="H166" s="7" t="n">
         <v>1</v>
@@ -11638,7 +11780,7 @@
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B167" s="7" t="s">
         <v>75</v>
@@ -11656,7 +11798,7 @@
         <v>248</v>
       </c>
       <c r="G167" s="7" t="n">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="H167" s="7" t="n">
         <v>1</v>
@@ -11665,7 +11807,7 @@
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="7" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B168" s="7" t="s">
         <v>75</v>
@@ -11683,7 +11825,7 @@
         <v>248</v>
       </c>
       <c r="G168" s="7" t="n">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="H168" s="7" t="n">
         <v>1</v>
@@ -11692,7 +11834,7 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="7" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B169" s="7" t="s">
         <v>75</v>
@@ -11710,7 +11852,7 @@
         <v>248</v>
       </c>
       <c r="G169" s="7" t="n">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="H169" s="7" t="n">
         <v>1</v>
@@ -11719,7 +11861,7 @@
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B170" s="7" t="s">
         <v>75</v>
@@ -11737,7 +11879,7 @@
         <v>248</v>
       </c>
       <c r="G170" s="7" t="n">
-        <v>701</v>
+        <v>612</v>
       </c>
       <c r="H170" s="7" t="n">
         <v>1</v>
@@ -11746,7 +11888,7 @@
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B171" s="7" t="s">
         <v>75</v>
@@ -11764,7 +11906,7 @@
         <v>248</v>
       </c>
       <c r="G171" s="7" t="n">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="H171" s="7" t="n">
         <v>1</v>
@@ -11773,7 +11915,7 @@
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="7" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B172" s="7" t="s">
         <v>75</v>
@@ -11791,7 +11933,7 @@
         <v>248</v>
       </c>
       <c r="G172" s="7" t="n">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H172" s="7" t="n">
         <v>1</v>
@@ -11800,7 +11942,7 @@
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="7" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B173" s="7" t="s">
         <v>75</v>
@@ -11818,7 +11960,7 @@
         <v>248</v>
       </c>
       <c r="G173" s="7" t="n">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H173" s="7" t="n">
         <v>1</v>
@@ -11827,7 +11969,7 @@
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="7" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B174" s="7" t="s">
         <v>75</v>
@@ -11845,7 +11987,7 @@
         <v>248</v>
       </c>
       <c r="G174" s="7" t="n">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="H174" s="7" t="n">
         <v>1</v>
@@ -11854,7 +11996,7 @@
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="7" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B175" s="7" t="s">
         <v>75</v>
@@ -11872,7 +12014,7 @@
         <v>248</v>
       </c>
       <c r="G175" s="7" t="n">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="H175" s="7" t="n">
         <v>1</v>
@@ -11881,7 +12023,7 @@
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B176" s="7" t="s">
         <v>75</v>
@@ -11899,7 +12041,7 @@
         <v>248</v>
       </c>
       <c r="G176" s="7" t="n">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="H176" s="7" t="n">
         <v>1</v>
@@ -11908,7 +12050,7 @@
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="7" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B177" s="7" t="s">
         <v>75</v>
@@ -11926,7 +12068,7 @@
         <v>248</v>
       </c>
       <c r="G177" s="7" t="n">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="H177" s="7" t="n">
         <v>1</v>
@@ -11935,7 +12077,7 @@
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B178" s="7" t="s">
         <v>75</v>
@@ -11953,7 +12095,7 @@
         <v>248</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="H178" s="7" t="n">
         <v>1</v>
@@ -11962,7 +12104,7 @@
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B179" s="7" t="s">
         <v>75</v>
@@ -11980,7 +12122,7 @@
         <v>248</v>
       </c>
       <c r="G179" s="7" t="n">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="H179" s="7" t="n">
         <v>1</v>
@@ -11989,7 +12131,7 @@
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="7" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B180" s="7" t="s">
         <v>75</v>
@@ -12007,7 +12149,7 @@
         <v>248</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="H180" s="7" t="n">
         <v>1</v>
@@ -12016,7 +12158,7 @@
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="7" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B181" s="7" t="s">
         <v>75</v>
@@ -12034,7 +12176,7 @@
         <v>248</v>
       </c>
       <c r="G181" s="7" t="n">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="H181" s="7" t="n">
         <v>1</v>
@@ -12043,7 +12185,7 @@
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B182" s="7" t="s">
         <v>75</v>
@@ -12061,7 +12203,7 @@
         <v>248</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>801</v>
+        <v>712</v>
       </c>
       <c r="H182" s="7" t="n">
         <v>1</v>
@@ -12070,7 +12212,7 @@
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="7" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B183" s="7" t="s">
         <v>75</v>
@@ -12088,7 +12230,7 @@
         <v>248</v>
       </c>
       <c r="G183" s="7" t="n">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="H183" s="7" t="n">
         <v>1</v>
@@ -12097,7 +12239,7 @@
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="7" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B184" s="7" t="s">
         <v>75</v>
@@ -12115,7 +12257,7 @@
         <v>248</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="H184" s="7" t="n">
         <v>1</v>
@@ -12124,7 +12266,7 @@
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="7" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B185" s="7" t="s">
         <v>75</v>
@@ -12142,104 +12284,102 @@
         <v>248</v>
       </c>
       <c r="G185" s="7" t="n">
+        <v>803</v>
+      </c>
+      <c r="H185" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I185" s="7"/>
+    </row>
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="B186" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C186" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D186" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E186" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F186" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="G186" s="7" t="n">
         <v>804</v>
       </c>
-      <c r="H185" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I185" s="7"/>
-    </row>
-    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A186" s="3" t="s">
+      <c r="H186" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I186" s="7"/>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A187" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B186" s="4" t="s">
+      <c r="B187" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C186" s="4" t="s">
+      <c r="C187" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D186" s="3" t="s">
+      <c r="D187" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E186" s="4" t="s">
+      <c r="E187" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F186" s="3" t="s">
+      <c r="F187" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G186" s="4" t="s">
+      <c r="G187" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H186" s="4" t="s">
+      <c r="H187" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I186" s="3" t="s">
+      <c r="I187" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A187" s="3"/>
-      <c r="B187" s="4" t="s">
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="3"/>
+      <c r="B188" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C187" s="4" t="s">
+      <c r="C188" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D187" s="3"/>
-      <c r="E187" s="4" t="s">
+      <c r="D188" s="3"/>
+      <c r="E188" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F187" s="3"/>
-      <c r="G187" s="4" t="s">
+      <c r="F188" s="3"/>
+      <c r="G188" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H187" s="4" t="s">
+      <c r="H188" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I187" s="3"/>
-    </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A188" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="B188" s="5"/>
-      <c r="C188" s="5"/>
-      <c r="D188" s="5"/>
-      <c r="E188" s="5"/>
-      <c r="F188" s="5"/>
-      <c r="G188" s="5"/>
-      <c r="H188" s="5"/>
-      <c r="I188" s="5"/>
-    </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A189" s="12" t="s">
-        <v>329</v>
-      </c>
-      <c r="B189" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C189" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D189" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E189" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F189" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G189" s="12" t="n">
-        <v>20001</v>
-      </c>
-      <c r="H189" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I189" s="12" t="s">
+      <c r="I188" s="3"/>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A189" s="5" t="s">
         <v>331</v>
       </c>
+      <c r="B189" s="5"/>
+      <c r="C189" s="5"/>
+      <c r="D189" s="5"/>
+      <c r="E189" s="5"/>
+      <c r="F189" s="5"/>
+      <c r="G189" s="5"/>
+      <c r="H189" s="5"/>
+      <c r="I189" s="5"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="12" t="s">
@@ -12258,79 +12398,79 @@
         <v>75</v>
       </c>
       <c r="F190" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G190" s="12" t="n">
-        <v>20002</v>
+        <v>20001</v>
       </c>
       <c r="H190" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I190" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="12" t="s">
+        <v>335</v>
+      </c>
+      <c r="B191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C191" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F191" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="B191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C191" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F191" s="12" t="s">
-        <v>330</v>
-      </c>
       <c r="G191" s="12" t="n">
-        <v>20003</v>
+        <v>20002</v>
       </c>
       <c r="H191" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I191" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="B192" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C192" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D192" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E192" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F192" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G192" s="12" t="n">
+        <v>20003</v>
+      </c>
+      <c r="H192" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I192" s="12" t="s">
         <v>334</v>
-      </c>
-      <c r="B192" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C192" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D192" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E192" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F192" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G192" s="12" t="n">
-        <v>20004</v>
-      </c>
-      <c r="H192" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I192" s="12" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="12" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B193" s="12" t="s">
         <v>75</v>
@@ -12345,21 +12485,21 @@
         <v>75</v>
       </c>
       <c r="F193" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G193" s="12" t="n">
-        <v>20005</v>
+        <v>20004</v>
       </c>
       <c r="H193" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I193" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="12" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B194" s="12" t="s">
         <v>75</v>
@@ -12374,21 +12514,21 @@
         <v>75</v>
       </c>
       <c r="F194" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G194" s="12" t="n">
-        <v>20006</v>
+        <v>20005</v>
       </c>
       <c r="H194" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I194" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="12" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B195" s="12" t="s">
         <v>75</v>
@@ -12403,21 +12543,21 @@
         <v>75</v>
       </c>
       <c r="F195" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G195" s="12" t="n">
-        <v>20007</v>
+        <v>20006</v>
       </c>
       <c r="H195" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I195" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="12" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B196" s="12" t="s">
         <v>75</v>
@@ -12432,21 +12572,21 @@
         <v>75</v>
       </c>
       <c r="F196" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G196" s="12" t="n">
-        <v>20008</v>
+        <v>20007</v>
       </c>
       <c r="H196" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I196" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="12" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B197" s="12" t="s">
         <v>75</v>
@@ -12461,21 +12601,21 @@
         <v>75</v>
       </c>
       <c r="F197" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G197" s="12" t="n">
-        <v>30001</v>
+        <v>20008</v>
       </c>
       <c r="H197" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I197" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B198" s="12" t="s">
         <v>75</v>
@@ -12490,21 +12630,21 @@
         <v>75</v>
       </c>
       <c r="F198" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G198" s="12" t="n">
-        <v>30002</v>
+        <v>30001</v>
       </c>
       <c r="H198" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I198" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B199" s="12" t="s">
         <v>75</v>
@@ -12519,21 +12659,21 @@
         <v>75</v>
       </c>
       <c r="F199" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G199" s="12" t="n">
-        <v>30003</v>
+        <v>30002</v>
       </c>
       <c r="H199" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I199" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B200" s="12" t="s">
         <v>75</v>
@@ -12548,21 +12688,21 @@
         <v>75</v>
       </c>
       <c r="F200" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G200" s="12" t="n">
-        <v>30004</v>
+        <v>30003</v>
       </c>
       <c r="H200" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I200" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="12" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B201" s="12" t="s">
         <v>75</v>
@@ -12577,21 +12717,21 @@
         <v>75</v>
       </c>
       <c r="F201" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G201" s="12" t="n">
-        <v>30005</v>
+        <v>30004</v>
       </c>
       <c r="H201" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I201" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="12" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B202" s="12" t="s">
         <v>75</v>
@@ -12606,21 +12746,21 @@
         <v>75</v>
       </c>
       <c r="F202" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G202" s="12" t="n">
-        <v>30006</v>
+        <v>30005</v>
       </c>
       <c r="H202" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I202" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="12" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B203" s="12" t="s">
         <v>75</v>
@@ -12635,21 +12775,21 @@
         <v>75</v>
       </c>
       <c r="F203" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G203" s="12" t="n">
-        <v>40001</v>
+        <v>30006</v>
       </c>
       <c r="H203" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I203" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="12" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B204" s="12" t="s">
         <v>75</v>
@@ -12664,21 +12804,21 @@
         <v>75</v>
       </c>
       <c r="F204" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G204" s="12" t="n">
-        <v>60001</v>
+        <v>40001</v>
       </c>
       <c r="H204" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I204" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="12" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B205" s="12" t="s">
         <v>75</v>
@@ -12693,21 +12833,21 @@
         <v>75</v>
       </c>
       <c r="F205" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G205" s="12" t="n">
-        <v>60002</v>
+        <v>60001</v>
       </c>
       <c r="H205" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I205" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="12" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B206" s="12" t="s">
         <v>75</v>
@@ -12722,21 +12862,21 @@
         <v>75</v>
       </c>
       <c r="F206" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G206" s="12" t="n">
-        <v>60003</v>
+        <v>60002</v>
       </c>
       <c r="H206" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I206" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="12" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B207" s="12" t="s">
         <v>75</v>
@@ -12751,21 +12891,21 @@
         <v>75</v>
       </c>
       <c r="F207" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G207" s="12" t="n">
-        <v>60004</v>
+        <v>60003</v>
       </c>
       <c r="H207" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I207" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B208" s="12" t="s">
         <v>75</v>
@@ -12780,21 +12920,21 @@
         <v>75</v>
       </c>
       <c r="F208" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G208" s="12" t="n">
-        <v>60005</v>
+        <v>60004</v>
       </c>
       <c r="H208" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I208" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B209" s="12" t="s">
         <v>75</v>
@@ -12809,21 +12949,21 @@
         <v>75</v>
       </c>
       <c r="F209" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G209" s="12" t="n">
-        <v>60006</v>
+        <v>60005</v>
       </c>
       <c r="H209" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I209" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B210" s="12" t="s">
         <v>75</v>
@@ -12838,669 +12978,669 @@
         <v>75</v>
       </c>
       <c r="F210" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G210" s="12" t="n">
-        <v>60007</v>
+        <v>60006</v>
       </c>
       <c r="H210" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
+        <v>355</v>
+      </c>
+      <c r="B211" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C211" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D211" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E211" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F211" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G211" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H211" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I211" s="12" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="12" t="s">
+        <v>356</v>
+      </c>
+      <c r="B212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C212" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F212" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G212" s="12" t="n">
+        <v>60008</v>
+      </c>
+      <c r="H212" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I212" s="12" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A213" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B213" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C213" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D213" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E213" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F213" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G213" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H213" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I213" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="3"/>
+      <c r="B214" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C214" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D214" s="3"/>
+      <c r="E214" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F214" s="3"/>
+      <c r="G214" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H214" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I214" s="3"/>
+    </row>
+    <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A215" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="B215" s="5"/>
+      <c r="C215" s="5"/>
+      <c r="D215" s="5"/>
+      <c r="E215" s="5"/>
+      <c r="F215" s="5"/>
+      <c r="G215" s="5"/>
+      <c r="H215" s="5"/>
+      <c r="I215" s="5"/>
+    </row>
+    <row r="216" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="12" t="s">
+        <v>342</v>
+      </c>
+      <c r="B216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C216" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F216" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G216" s="12" t="n">
+        <v>30001</v>
+      </c>
+      <c r="H216" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I216" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="B217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C217" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F217" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G217" s="12" t="n">
+        <v>30002</v>
+      </c>
+      <c r="H217" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I217" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="12" t="s">
+        <v>344</v>
+      </c>
+      <c r="B218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C218" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F218" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G218" s="12" t="n">
+        <v>30003</v>
+      </c>
+      <c r="H218" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I218" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="B219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C219" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F219" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G219" s="12" t="n">
+        <v>30004</v>
+      </c>
+      <c r="H219" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I219" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="12" t="s">
+        <v>346</v>
+      </c>
+      <c r="B220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C220" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F220" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G220" s="12" t="n">
+        <v>30005</v>
+      </c>
+      <c r="H220" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I220" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="B221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C221" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F221" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G221" s="12" t="n">
+        <v>30006</v>
+      </c>
+      <c r="H221" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I221" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="B222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C222" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F222" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G222" s="12" t="n">
+        <v>40001</v>
+      </c>
+      <c r="H222" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I222" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="12" t="s">
+        <v>359</v>
+      </c>
+      <c r="B223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C223" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F223" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G223" s="12" t="n">
+        <v>45001</v>
+      </c>
+      <c r="H223" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I223" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="B224" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C224" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D224" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E224" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F224" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G224" s="12" t="n">
+        <v>60001</v>
+      </c>
+      <c r="H224" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I224" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="B225" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C225" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D225" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E225" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F225" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G225" s="12" t="n">
+        <v>60002</v>
+      </c>
+      <c r="H225" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I225" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="B226" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C226" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D226" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E226" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F226" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G226" s="12" t="n">
+        <v>60003</v>
+      </c>
+      <c r="H226" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I226" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="12" t="s">
+        <v>352</v>
+      </c>
+      <c r="B227" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C227" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D227" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E227" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F227" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G227" s="12" t="n">
+        <v>60004</v>
+      </c>
+      <c r="H227" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I227" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="12" t="s">
         <v>353</v>
       </c>
-      <c r="B211" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C211" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D211" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E211" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F211" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G211" s="12" t="n">
+      <c r="B228" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C228" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D228" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E228" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F228" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G228" s="12" t="n">
+        <v>60005</v>
+      </c>
+      <c r="H228" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I228" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="12" t="s">
+        <v>354</v>
+      </c>
+      <c r="B229" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C229" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D229" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E229" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F229" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G229" s="12" t="n">
+        <v>60006</v>
+      </c>
+      <c r="H229" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I229" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="12" t="s">
+        <v>355</v>
+      </c>
+      <c r="B230" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C230" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D230" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E230" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F230" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G230" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H230" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I230" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="12" t="s">
+        <v>356</v>
+      </c>
+      <c r="B231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C231" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F231" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="G231" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H211" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I211" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A212" s="3" t="s">
+      <c r="H231" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I231" s="12" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A232" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B212" s="4" t="s">
+      <c r="B232" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C212" s="4" t="s">
+      <c r="C232" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D212" s="3" t="s">
+      <c r="D232" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E212" s="4" t="s">
+      <c r="E232" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F212" s="3" t="s">
+      <c r="F232" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G212" s="4" t="s">
+      <c r="G232" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H212" s="4" t="s">
+      <c r="H232" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I212" s="3" t="s">
+      <c r="I232" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A213" s="3"/>
-      <c r="B213" s="4" t="s">
+    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="3"/>
+      <c r="B233" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C213" s="4" t="s">
+      <c r="C233" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D213" s="3"/>
-      <c r="E213" s="4" t="s">
+      <c r="D233" s="3"/>
+      <c r="E233" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F213" s="3"/>
-      <c r="G213" s="4" t="s">
+      <c r="F233" s="3"/>
+      <c r="G233" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H213" s="4" t="s">
+      <c r="H233" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I213" s="3"/>
-    </row>
-    <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A214" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="B214" s="5"/>
-      <c r="C214" s="5"/>
-      <c r="D214" s="5"/>
-      <c r="E214" s="5"/>
-      <c r="F214" s="5"/>
-      <c r="G214" s="5"/>
-      <c r="H214" s="5"/>
-      <c r="I214" s="5"/>
-    </row>
-    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A215" s="12" t="s">
-        <v>339</v>
-      </c>
-      <c r="B215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C215" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F215" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G215" s="12" t="n">
-        <v>30001</v>
-      </c>
-      <c r="H215" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I215" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A216" s="12" t="s">
-        <v>340</v>
-      </c>
-      <c r="B216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C216" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F216" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G216" s="12" t="n">
-        <v>30002</v>
-      </c>
-      <c r="H216" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I216" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A217" s="12" t="s">
-        <v>341</v>
-      </c>
-      <c r="B217" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C217" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D217" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E217" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F217" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G217" s="12" t="n">
-        <v>30003</v>
-      </c>
-      <c r="H217" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I217" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A218" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="B218" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C218" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D218" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E218" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F218" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G218" s="12" t="n">
-        <v>30004</v>
-      </c>
-      <c r="H218" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I218" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A219" s="12" t="s">
-        <v>343</v>
-      </c>
-      <c r="B219" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C219" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D219" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E219" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F219" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G219" s="12" t="n">
-        <v>30005</v>
-      </c>
-      <c r="H219" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I219" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A220" s="12" t="s">
-        <v>344</v>
-      </c>
-      <c r="B220" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C220" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D220" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E220" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F220" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G220" s="12" t="n">
-        <v>30006</v>
-      </c>
-      <c r="H220" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I220" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A221" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="B221" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C221" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D221" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E221" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F221" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G221" s="12" t="n">
-        <v>40001</v>
-      </c>
-      <c r="H221" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I221" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A222" s="12" t="s">
-        <v>355</v>
-      </c>
-      <c r="B222" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C222" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D222" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E222" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F222" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G222" s="12" t="n">
-        <v>45001</v>
-      </c>
-      <c r="H222" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I222" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A223" s="12" t="s">
-        <v>346</v>
-      </c>
-      <c r="B223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C223" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F223" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G223" s="12" t="n">
-        <v>60001</v>
-      </c>
-      <c r="H223" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I223" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A224" s="12" t="s">
-        <v>347</v>
-      </c>
-      <c r="B224" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C224" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D224" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E224" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F224" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G224" s="12" t="n">
-        <v>60002</v>
-      </c>
-      <c r="H224" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I224" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A225" s="12" t="s">
-        <v>348</v>
-      </c>
-      <c r="B225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C225" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F225" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G225" s="12" t="n">
-        <v>60003</v>
-      </c>
-      <c r="H225" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I225" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A226" s="12" t="s">
-        <v>349</v>
-      </c>
-      <c r="B226" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C226" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D226" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E226" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F226" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G226" s="12" t="n">
-        <v>60004</v>
-      </c>
-      <c r="H226" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I226" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A227" s="12" t="s">
-        <v>350</v>
-      </c>
-      <c r="B227" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C227" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D227" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E227" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F227" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G227" s="12" t="n">
-        <v>60005</v>
-      </c>
-      <c r="H227" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I227" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A228" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="B228" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C228" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D228" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E228" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F228" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G228" s="12" t="n">
-        <v>60006</v>
-      </c>
-      <c r="H228" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I228" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A229" s="12" t="s">
-        <v>352</v>
-      </c>
-      <c r="B229" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C229" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D229" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E229" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F229" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G229" s="12" t="n">
-        <v>60007</v>
-      </c>
-      <c r="H229" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I229" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A230" s="12" t="s">
-        <v>353</v>
-      </c>
-      <c r="B230" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C230" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D230" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E230" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F230" s="12" t="s">
-        <v>330</v>
-      </c>
-      <c r="G230" s="12" t="n">
-        <v>60008</v>
-      </c>
-      <c r="H230" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I230" s="12" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A231" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B231" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C231" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D231" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E231" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F231" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G231" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H231" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I231" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A232" s="3"/>
-      <c r="B232" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C232" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D232" s="3"/>
-      <c r="E232" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F232" s="3"/>
-      <c r="G232" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H232" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I232" s="3"/>
-    </row>
-    <row r="233" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A233" s="5" t="s">
+      <c r="I233" s="3"/>
+    </row>
+    <row r="234" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A234" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="B233" s="5"/>
-      <c r="C233" s="5"/>
-      <c r="D233" s="5"/>
-      <c r="E233" s="5"/>
-      <c r="F233" s="5"/>
-      <c r="G233" s="5"/>
-      <c r="H233" s="5"/>
-      <c r="I233" s="5"/>
-    </row>
-    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A234" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B234" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C234" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D234" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E234" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F234" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G234" s="10" t="s">
-        <v>318</v>
-      </c>
-      <c r="H234" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I234" s="7" t="s">
-        <v>112</v>
-      </c>
+      <c r="B234" s="5"/>
+      <c r="C234" s="5"/>
+      <c r="D234" s="5"/>
+      <c r="E234" s="5"/>
+      <c r="F234" s="5"/>
+      <c r="G234" s="5"/>
+      <c r="H234" s="5"/>
+      <c r="I234" s="5"/>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="9" t="s">
-        <v>187</v>
+        <v>108</v>
       </c>
       <c r="B235" s="7" t="s">
         <v>109</v>
@@ -13518,21 +13658,21 @@
         <v>26</v>
       </c>
       <c r="G235" s="10" t="s">
-        <v>188</v>
+        <v>318</v>
       </c>
       <c r="H235" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I235" s="7" t="s">
-        <v>189</v>
+        <v>112</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="9" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="B236" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C236" s="7" t="s">
         <v>110</v>
@@ -13547,16 +13687,18 @@
         <v>26</v>
       </c>
       <c r="G236" s="10" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="H236" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I236" s="7"/>
+      <c r="I236" s="7" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B237" s="7" t="s">
         <v>24</v>
@@ -13574,7 +13716,7 @@
         <v>26</v>
       </c>
       <c r="G237" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H237" s="7" t="n">
         <v>2</v>
@@ -13583,7 +13725,7 @@
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="9" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B238" s="7" t="s">
         <v>24</v>
@@ -13601,7 +13743,7 @@
         <v>26</v>
       </c>
       <c r="G238" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H238" s="7" t="n">
         <v>2</v>
@@ -13610,7 +13752,7 @@
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B239" s="7" t="s">
         <v>24</v>
@@ -13628,7 +13770,7 @@
         <v>26</v>
       </c>
       <c r="G239" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H239" s="7" t="n">
         <v>2</v>
@@ -13637,10 +13779,10 @@
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="9" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B240" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C240" s="7" t="s">
         <v>110</v>
@@ -13655,7 +13797,7 @@
         <v>26</v>
       </c>
       <c r="G240" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H240" s="7" t="n">
         <v>2</v>
@@ -13664,7 +13806,7 @@
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="9" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B241" s="7" t="s">
         <v>109</v>
@@ -13682,7 +13824,7 @@
         <v>26</v>
       </c>
       <c r="G241" s="10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H241" s="7" t="n">
         <v>2</v>
@@ -13691,10 +13833,10 @@
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="9" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B242" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C242" s="7" t="s">
         <v>110</v>
@@ -13709,7 +13851,7 @@
         <v>26</v>
       </c>
       <c r="G242" s="10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H242" s="7" t="n">
         <v>2</v>
@@ -13718,7 +13860,7 @@
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B243" s="7" t="s">
         <v>24</v>
@@ -13736,7 +13878,7 @@
         <v>26</v>
       </c>
       <c r="G243" s="10" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H243" s="7" t="n">
         <v>2</v>
@@ -13745,7 +13887,7 @@
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B244" s="7" t="s">
         <v>24</v>
@@ -13763,7 +13905,7 @@
         <v>26</v>
       </c>
       <c r="G244" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H244" s="7" t="n">
         <v>2</v>
@@ -13772,7 +13914,7 @@
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B245" s="7" t="s">
         <v>24</v>
@@ -13790,7 +13932,7 @@
         <v>26</v>
       </c>
       <c r="G245" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H245" s="7" t="n">
         <v>2</v>
@@ -13799,10 +13941,10 @@
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="9" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B246" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C246" s="7" t="s">
         <v>110</v>
@@ -13817,7 +13959,7 @@
         <v>26</v>
       </c>
       <c r="G246" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="H246" s="7" t="n">
         <v>2</v>
@@ -13826,7 +13968,7 @@
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B247" s="7" t="s">
         <v>109</v>
@@ -13844,7 +13986,7 @@
         <v>26</v>
       </c>
       <c r="G247" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H247" s="7" t="n">
         <v>2</v>
@@ -13853,10 +13995,10 @@
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B248" s="7" t="s">
-        <v>222</v>
+        <v>109</v>
       </c>
       <c r="C248" s="7" t="s">
         <v>110</v>
@@ -13871,7 +14013,7 @@
         <v>26</v>
       </c>
       <c r="G248" s="10" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H248" s="7" t="n">
         <v>2</v>
@@ -13880,7 +14022,7 @@
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B249" s="7" t="s">
         <v>222</v>
@@ -13898,7 +14040,7 @@
         <v>26</v>
       </c>
       <c r="G249" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H249" s="7" t="n">
         <v>2</v>
@@ -13907,10 +14049,10 @@
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="9" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B250" s="7" t="s">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="C250" s="7" t="s">
         <v>110</v>
@@ -13925,7 +14067,7 @@
         <v>26</v>
       </c>
       <c r="G250" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H250" s="7" t="n">
         <v>2</v>
@@ -13934,7 +14076,7 @@
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="9" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B251" s="7" t="s">
         <v>195</v>
@@ -13952,7 +14094,7 @@
         <v>26</v>
       </c>
       <c r="G251" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H251" s="7" t="n">
         <v>2</v>
@@ -13961,10 +14103,10 @@
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="9" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B252" s="7" t="s">
-        <v>109</v>
+        <v>195</v>
       </c>
       <c r="C252" s="7" t="s">
         <v>110</v>
@@ -13979,7 +14121,7 @@
         <v>26</v>
       </c>
       <c r="G252" s="10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H252" s="7" t="n">
         <v>2</v>
@@ -13988,7 +14130,7 @@
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="9" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B253" s="7" t="s">
         <v>109</v>
@@ -14006,7 +14148,7 @@
         <v>26</v>
       </c>
       <c r="G253" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H253" s="7" t="n">
         <v>2</v>
@@ -14014,11 +14156,11 @@
       <c r="I253" s="7"/>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A254" s="7" t="s">
-        <v>234</v>
+      <c r="A254" s="9" t="s">
+        <v>232</v>
       </c>
       <c r="B254" s="7" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C254" s="7" t="s">
         <v>110</v>
@@ -14033,18 +14175,16 @@
         <v>26</v>
       </c>
       <c r="G254" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H254" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I254" s="7" t="s">
-        <v>236</v>
-      </c>
+      <c r="I254" s="7"/>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="7" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B255" s="7" t="s">
         <v>75</v>
@@ -14062,7 +14202,7 @@
         <v>26</v>
       </c>
       <c r="G255" s="10" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H255" s="7" t="n">
         <v>2</v>
@@ -14072,37 +14212,37 @@
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A256" s="12" t="s">
+      <c r="A256" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B256" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C256" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D256" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E256" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F256" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G256" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="H256" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I256" s="7" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="257" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A257" s="12" t="s">
         <v>239</v>
-      </c>
-      <c r="B256" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C256" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D256" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E256" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F256" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G256" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="H256" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I256" s="14" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A257" s="12" t="s">
-        <v>241</v>
       </c>
       <c r="B257" s="12" t="s">
         <v>75</v>
@@ -14120,18 +14260,18 @@
         <v>26</v>
       </c>
       <c r="G257" s="12" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="H257" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I257" s="14" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="258" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A258" s="11" t="s">
-        <v>322</v>
+        <v>360</v>
+      </c>
+    </row>
+    <row r="258" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="12" t="s">
+        <v>241</v>
       </c>
       <c r="B258" s="12" t="s">
         <v>75</v>
@@ -14148,19 +14288,19 @@
       <c r="F258" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="G258" s="13" t="s">
-        <v>323</v>
+      <c r="G258" s="12" t="s">
+        <v>242</v>
       </c>
       <c r="H258" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I258" s="12" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="259" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I258" s="14" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="259" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="11" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B259" s="12" t="s">
         <v>75</v>
@@ -14178,13 +14318,71 @@
         <v>26</v>
       </c>
       <c r="G259" s="13" t="s">
+        <v>323</v>
+      </c>
+      <c r="H259" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I259" s="12" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="260" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="11" t="s">
+        <v>325</v>
+      </c>
+      <c r="B260" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C260" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D260" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E260" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F260" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G260" s="13" t="s">
         <v>326</v>
       </c>
-      <c r="H259" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I259" s="12" t="s">
-        <v>327</v>
+      <c r="H260" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I260" s="12" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="261" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="B261" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C261" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D261" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E261" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F261" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G261" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="H261" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I261" s="12" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>
@@ -14194,26 +14392,26 @@
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A114:A115"/>
-    <mergeCell ref="D114:D115"/>
-    <mergeCell ref="F114:F115"/>
-    <mergeCell ref="I114:I115"/>
-    <mergeCell ref="A116:I116"/>
-    <mergeCell ref="A186:A187"/>
-    <mergeCell ref="D186:D187"/>
-    <mergeCell ref="F186:F187"/>
-    <mergeCell ref="I186:I187"/>
-    <mergeCell ref="A188:I188"/>
-    <mergeCell ref="A212:A213"/>
-    <mergeCell ref="D212:D213"/>
-    <mergeCell ref="F212:F213"/>
-    <mergeCell ref="I212:I213"/>
-    <mergeCell ref="A214:I214"/>
-    <mergeCell ref="A231:A232"/>
-    <mergeCell ref="D231:D232"/>
-    <mergeCell ref="F231:F232"/>
-    <mergeCell ref="I231:I232"/>
-    <mergeCell ref="A233:I233"/>
+    <mergeCell ref="A115:A116"/>
+    <mergeCell ref="D115:D116"/>
+    <mergeCell ref="F115:F116"/>
+    <mergeCell ref="I115:I116"/>
+    <mergeCell ref="A117:I117"/>
+    <mergeCell ref="A187:A188"/>
+    <mergeCell ref="D187:D188"/>
+    <mergeCell ref="F187:F188"/>
+    <mergeCell ref="I187:I188"/>
+    <mergeCell ref="A189:I189"/>
+    <mergeCell ref="A213:A214"/>
+    <mergeCell ref="D213:D214"/>
+    <mergeCell ref="F213:F214"/>
+    <mergeCell ref="I213:I214"/>
+    <mergeCell ref="A215:I215"/>
+    <mergeCell ref="A232:A233"/>
+    <mergeCell ref="D232:D233"/>
+    <mergeCell ref="F232:F233"/>
+    <mergeCell ref="I232:I233"/>
+    <mergeCell ref="A234:I234"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
SOCO: Bugfix: Disallow toggling LEDs/Output via modbus for user
Unless the user puts the controller in test mode, we shouldn't allow the
user to toggle LEDs/Output Relays over modbus.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2547" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2547" uniqueCount="366">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -1157,35 +1157,21 @@
     <t xml:space="preserve">WRITE SINGLE COIL STATUS (Function Code: 0x05)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Internal Only. Not visible to customer.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">Only writtable when test mode enabled.</t>
-    </r>
+    <t xml:space="preserve">Internal Only. Not visible to customer.
+Only settable when test mode enabled</t>
   </si>
   <si>
     <t xml:space="preserve">Restart Controller</t>
   </si>
   <si>
     <t xml:space="preserve">Internal Only. Not visible to customer. 
-Only writtable when test mode enabled.</t>
+Only writtable when test mode enabled.
+Only writtable together with Serial Number Upper Half</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal Only. Not visible to customer. 
+Only writtable when test mode enabled.
+Only writtable together with Serial Number Lower Half</t>
   </si>
   <si>
     <t xml:space="preserve">Internal Only. Not visible to customer. 
@@ -13285,7 +13271,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="12" t="s">
         <v>348</v>
       </c>
@@ -13311,7 +13297,7 @@
         <v>1</v>
       </c>
       <c r="I222" s="12" t="s">
-        <v>358</v>
+        <v>334</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14240,7 +14226,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="257" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="257" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="12" t="s">
         <v>239</v>
       </c>
@@ -14269,7 +14255,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="258" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="258" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="12" t="s">
         <v>241</v>
       </c>
@@ -14295,7 +14281,7 @@
         <v>2</v>
       </c>
       <c r="I258" s="14" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="259" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14324,7 +14310,7 @@
         <v>2</v>
       </c>
       <c r="I259" s="12" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14353,12 +14339,12 @@
         <v>2</v>
       </c>
       <c r="I260" s="12" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="261" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="11" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B261" s="12" t="s">
         <v>75</v>
@@ -14382,7 +14368,7 @@
         <v>2</v>
       </c>
       <c r="I261" s="12" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SOCO: Bugfix: Fix modbus excel table
Removed an entry which didn't exists.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2547" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="367">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -1074,6 +1074,9 @@
 127: Calibration Completed Successfully
 126: Error occured during calibration. Please restart controller</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Load On Grid Contactor &amp; Solar Neutral Earth Contactor Coil</t>
   </si>
   <si>
     <t xml:space="preserve">READ COIL STATUS (Function Code: 0x01)</t>
@@ -7352,7 +7355,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I261"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.94"/>
@@ -11145,7 +11148,7 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="7" t="s">
-        <v>274</v>
+        <v>331</v>
       </c>
       <c r="B144" s="7" t="s">
         <v>75</v>
@@ -11172,7 +11175,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B145" s="7" t="s">
         <v>75</v>
@@ -11199,7 +11202,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="7" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B146" s="7" t="s">
         <v>75</v>
@@ -11217,7 +11220,7 @@
         <v>248</v>
       </c>
       <c r="G146" s="7" t="n">
-        <v>407</v>
+        <v>501</v>
       </c>
       <c r="H146" s="7" t="n">
         <v>1</v>
@@ -11226,7 +11229,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B147" s="7" t="s">
         <v>75</v>
@@ -11244,7 +11247,7 @@
         <v>248</v>
       </c>
       <c r="G147" s="7" t="n">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="H147" s="7" t="n">
         <v>1</v>
@@ -11253,7 +11256,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="7" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B148" s="7" t="s">
         <v>75</v>
@@ -11271,7 +11274,7 @@
         <v>248</v>
       </c>
       <c r="G148" s="7" t="n">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="H148" s="7" t="n">
         <v>1</v>
@@ -11280,7 +11283,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="7" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B149" s="7" t="s">
         <v>75</v>
@@ -11298,7 +11301,7 @@
         <v>248</v>
       </c>
       <c r="G149" s="7" t="n">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="H149" s="7" t="n">
         <v>1</v>
@@ -11307,7 +11310,7 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B150" s="7" t="s">
         <v>75</v>
@@ -11325,7 +11328,7 @@
         <v>248</v>
       </c>
       <c r="G150" s="7" t="n">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="H150" s="7" t="n">
         <v>1</v>
@@ -11334,7 +11337,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B151" s="7" t="s">
         <v>75</v>
@@ -11352,7 +11355,7 @@
         <v>248</v>
       </c>
       <c r="G151" s="7" t="n">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H151" s="7" t="n">
         <v>1</v>
@@ -11361,7 +11364,7 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B152" s="7" t="s">
         <v>75</v>
@@ -11379,7 +11382,7 @@
         <v>248</v>
       </c>
       <c r="G152" s="7" t="n">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="H152" s="7" t="n">
         <v>1</v>
@@ -11388,7 +11391,7 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B153" s="7" t="s">
         <v>75</v>
@@ -11406,7 +11409,7 @@
         <v>248</v>
       </c>
       <c r="G153" s="7" t="n">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="H153" s="7" t="n">
         <v>1</v>
@@ -11415,7 +11418,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="7" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B154" s="7" t="s">
         <v>75</v>
@@ -11433,7 +11436,7 @@
         <v>248</v>
       </c>
       <c r="G154" s="7" t="n">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="H154" s="7" t="n">
         <v>1</v>
@@ -11442,7 +11445,7 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="7" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B155" s="7" t="s">
         <v>75</v>
@@ -11460,7 +11463,7 @@
         <v>248</v>
       </c>
       <c r="G155" s="7" t="n">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="H155" s="7" t="n">
         <v>1</v>
@@ -11469,7 +11472,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B156" s="7" t="s">
         <v>75</v>
@@ -11487,7 +11490,7 @@
         <v>248</v>
       </c>
       <c r="G156" s="7" t="n">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="H156" s="7" t="n">
         <v>1</v>
@@ -11496,7 +11499,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B157" s="7" t="s">
         <v>75</v>
@@ -11514,7 +11517,7 @@
         <v>248</v>
       </c>
       <c r="G157" s="7" t="n">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="H157" s="7" t="n">
         <v>1</v>
@@ -11523,7 +11526,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B158" s="7" t="s">
         <v>75</v>
@@ -11541,7 +11544,7 @@
         <v>248</v>
       </c>
       <c r="G158" s="7" t="n">
-        <v>512</v>
+        <v>601</v>
       </c>
       <c r="H158" s="7" t="n">
         <v>1</v>
@@ -11550,7 +11553,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B159" s="7" t="s">
         <v>75</v>
@@ -11568,7 +11571,7 @@
         <v>248</v>
       </c>
       <c r="G159" s="7" t="n">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="H159" s="7" t="n">
         <v>1</v>
@@ -11577,7 +11580,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B160" s="7" t="s">
         <v>75</v>
@@ -11595,7 +11598,7 @@
         <v>248</v>
       </c>
       <c r="G160" s="7" t="n">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="H160" s="7" t="n">
         <v>1</v>
@@ -11604,7 +11607,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B161" s="7" t="s">
         <v>75</v>
@@ -11622,7 +11625,7 @@
         <v>248</v>
       </c>
       <c r="G161" s="7" t="n">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H161" s="7" t="n">
         <v>1</v>
@@ -11631,7 +11634,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B162" s="7" t="s">
         <v>75</v>
@@ -11649,7 +11652,7 @@
         <v>248</v>
       </c>
       <c r="G162" s="7" t="n">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="H162" s="7" t="n">
         <v>1</v>
@@ -11658,7 +11661,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B163" s="7" t="s">
         <v>75</v>
@@ -11676,7 +11679,7 @@
         <v>248</v>
       </c>
       <c r="G163" s="7" t="n">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="H163" s="7" t="n">
         <v>1</v>
@@ -11685,7 +11688,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="7" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B164" s="7" t="s">
         <v>75</v>
@@ -11703,7 +11706,7 @@
         <v>248</v>
       </c>
       <c r="G164" s="7" t="n">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="H164" s="7" t="n">
         <v>1</v>
@@ -11712,7 +11715,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B165" s="7" t="s">
         <v>75</v>
@@ -11730,7 +11733,7 @@
         <v>248</v>
       </c>
       <c r="G165" s="7" t="n">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="H165" s="7" t="n">
         <v>1</v>
@@ -11739,7 +11742,7 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B166" s="7" t="s">
         <v>75</v>
@@ -11757,7 +11760,7 @@
         <v>248</v>
       </c>
       <c r="G166" s="7" t="n">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="H166" s="7" t="n">
         <v>1</v>
@@ -11766,7 +11769,7 @@
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B167" s="7" t="s">
         <v>75</v>
@@ -11784,7 +11787,7 @@
         <v>248</v>
       </c>
       <c r="G167" s="7" t="n">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="H167" s="7" t="n">
         <v>1</v>
@@ -11793,7 +11796,7 @@
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B168" s="7" t="s">
         <v>75</v>
@@ -11811,7 +11814,7 @@
         <v>248</v>
       </c>
       <c r="G168" s="7" t="n">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="H168" s="7" t="n">
         <v>1</v>
@@ -11820,7 +11823,7 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B169" s="7" t="s">
         <v>75</v>
@@ -11838,7 +11841,7 @@
         <v>248</v>
       </c>
       <c r="G169" s="7" t="n">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="H169" s="7" t="n">
         <v>1</v>
@@ -11847,7 +11850,7 @@
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B170" s="7" t="s">
         <v>75</v>
@@ -11865,7 +11868,7 @@
         <v>248</v>
       </c>
       <c r="G170" s="7" t="n">
-        <v>612</v>
+        <v>701</v>
       </c>
       <c r="H170" s="7" t="n">
         <v>1</v>
@@ -11874,7 +11877,7 @@
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="7" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B171" s="7" t="s">
         <v>75</v>
@@ -11892,7 +11895,7 @@
         <v>248</v>
       </c>
       <c r="G171" s="7" t="n">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="H171" s="7" t="n">
         <v>1</v>
@@ -11901,7 +11904,7 @@
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B172" s="7" t="s">
         <v>75</v>
@@ -11919,7 +11922,7 @@
         <v>248</v>
       </c>
       <c r="G172" s="7" t="n">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="H172" s="7" t="n">
         <v>1</v>
@@ -11928,7 +11931,7 @@
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B173" s="7" t="s">
         <v>75</v>
@@ -11946,7 +11949,7 @@
         <v>248</v>
       </c>
       <c r="G173" s="7" t="n">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="H173" s="7" t="n">
         <v>1</v>
@@ -11955,7 +11958,7 @@
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B174" s="7" t="s">
         <v>75</v>
@@ -11973,7 +11976,7 @@
         <v>248</v>
       </c>
       <c r="G174" s="7" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="H174" s="7" t="n">
         <v>1</v>
@@ -11982,7 +11985,7 @@
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B175" s="7" t="s">
         <v>75</v>
@@ -12000,7 +12003,7 @@
         <v>248</v>
       </c>
       <c r="G175" s="7" t="n">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="H175" s="7" t="n">
         <v>1</v>
@@ -12009,7 +12012,7 @@
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="7" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B176" s="7" t="s">
         <v>75</v>
@@ -12027,7 +12030,7 @@
         <v>248</v>
       </c>
       <c r="G176" s="7" t="n">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="H176" s="7" t="n">
         <v>1</v>
@@ -12036,7 +12039,7 @@
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="7" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B177" s="7" t="s">
         <v>75</v>
@@ -12054,7 +12057,7 @@
         <v>248</v>
       </c>
       <c r="G177" s="7" t="n">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="H177" s="7" t="n">
         <v>1</v>
@@ -12063,7 +12066,7 @@
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B178" s="7" t="s">
         <v>75</v>
@@ -12081,7 +12084,7 @@
         <v>248</v>
       </c>
       <c r="G178" s="7" t="n">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="H178" s="7" t="n">
         <v>1</v>
@@ -12090,7 +12093,7 @@
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="7" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B179" s="7" t="s">
         <v>75</v>
@@ -12108,7 +12111,7 @@
         <v>248</v>
       </c>
       <c r="G179" s="7" t="n">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="H179" s="7" t="n">
         <v>1</v>
@@ -12117,7 +12120,7 @@
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B180" s="7" t="s">
         <v>75</v>
@@ -12135,7 +12138,7 @@
         <v>248</v>
       </c>
       <c r="G180" s="7" t="n">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="H180" s="7" t="n">
         <v>1</v>
@@ -12144,7 +12147,7 @@
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B181" s="7" t="s">
         <v>75</v>
@@ -12162,7 +12165,7 @@
         <v>248</v>
       </c>
       <c r="G181" s="7" t="n">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="H181" s="7" t="n">
         <v>1</v>
@@ -12171,7 +12174,7 @@
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="7" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B182" s="7" t="s">
         <v>75</v>
@@ -12189,7 +12192,7 @@
         <v>248</v>
       </c>
       <c r="G182" s="7" t="n">
-        <v>712</v>
+        <v>801</v>
       </c>
       <c r="H182" s="7" t="n">
         <v>1</v>
@@ -12198,7 +12201,7 @@
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="7" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B183" s="7" t="s">
         <v>75</v>
@@ -12216,7 +12219,7 @@
         <v>248</v>
       </c>
       <c r="G183" s="7" t="n">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="H183" s="7" t="n">
         <v>1</v>
@@ -12225,7 +12228,7 @@
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="7" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B184" s="7" t="s">
         <v>75</v>
@@ -12243,7 +12246,7 @@
         <v>248</v>
       </c>
       <c r="G184" s="7" t="n">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="H184" s="7" t="n">
         <v>1</v>
@@ -12252,7 +12255,7 @@
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B185" s="7" t="s">
         <v>75</v>
@@ -12270,106 +12273,108 @@
         <v>248</v>
       </c>
       <c r="G185" s="7" t="n">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="H185" s="7" t="n">
         <v>1</v>
       </c>
       <c r="I185" s="7"/>
     </row>
-    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A186" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="B186" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C186" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D186" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E186" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F186" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G186" s="7" t="n">
-        <v>804</v>
-      </c>
-      <c r="H186" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I186" s="7"/>
-    </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A187" s="3" t="s">
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A186" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="B186" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C186" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D186" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E186" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F186" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G186" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H186" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I186" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="3"/>
       <c r="B187" s="4" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D187" s="3" t="s">
-        <v>11</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="D187" s="3"/>
       <c r="E187" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F187" s="3" t="s">
-        <v>13</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="F187" s="3"/>
       <c r="G187" s="4" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H187" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I187" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A188" s="3"/>
-      <c r="B188" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C188" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D188" s="3"/>
-      <c r="E188" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F188" s="3"/>
-      <c r="G188" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H188" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I188" s="3"/>
-    </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A189" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="B189" s="5"/>
-      <c r="C189" s="5"/>
-      <c r="D189" s="5"/>
-      <c r="E189" s="5"/>
-      <c r="F189" s="5"/>
-      <c r="G189" s="5"/>
-      <c r="H189" s="5"/>
-      <c r="I189" s="5"/>
+      <c r="I187" s="3"/>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A188" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="B188" s="5"/>
+      <c r="C188" s="5"/>
+      <c r="D188" s="5"/>
+      <c r="E188" s="5"/>
+      <c r="F188" s="5"/>
+      <c r="G188" s="5"/>
+      <c r="H188" s="5"/>
+      <c r="I188" s="5"/>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="B189" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C189" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D189" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E189" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F189" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="G189" s="12" t="n">
+        <v>20001</v>
+      </c>
+      <c r="H189" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I189" s="12" t="s">
+        <v>335</v>
+      </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="12" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B190" s="12" t="s">
         <v>75</v>
@@ -12384,50 +12389,50 @@
         <v>75</v>
       </c>
       <c r="F190" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G190" s="12" t="n">
-        <v>20001</v>
+        <v>20002</v>
       </c>
       <c r="H190" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I190" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="B191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C191" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F191" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="G191" s="12" t="n">
+        <v>20003</v>
+      </c>
+      <c r="H191" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I191" s="12" t="s">
         <v>335</v>
-      </c>
-      <c r="B191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C191" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F191" s="12" t="s">
-        <v>333</v>
-      </c>
-      <c r="G191" s="12" t="n">
-        <v>20002</v>
-      </c>
-      <c r="H191" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I191" s="12" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="12" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B192" s="12" t="s">
         <v>75</v>
@@ -12442,21 +12447,21 @@
         <v>75</v>
       </c>
       <c r="F192" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G192" s="12" t="n">
-        <v>20003</v>
+        <v>20004</v>
       </c>
       <c r="H192" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I192" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="12" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B193" s="12" t="s">
         <v>75</v>
@@ -12471,21 +12476,21 @@
         <v>75</v>
       </c>
       <c r="F193" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G193" s="12" t="n">
-        <v>20004</v>
+        <v>20005</v>
       </c>
       <c r="H193" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I193" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="12" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B194" s="12" t="s">
         <v>75</v>
@@ -12500,21 +12505,21 @@
         <v>75</v>
       </c>
       <c r="F194" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G194" s="12" t="n">
-        <v>20005</v>
+        <v>20006</v>
       </c>
       <c r="H194" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I194" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="12" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B195" s="12" t="s">
         <v>75</v>
@@ -12529,21 +12534,21 @@
         <v>75</v>
       </c>
       <c r="F195" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G195" s="12" t="n">
-        <v>20006</v>
+        <v>20007</v>
       </c>
       <c r="H195" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I195" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B196" s="12" t="s">
         <v>75</v>
@@ -12558,21 +12563,21 @@
         <v>75</v>
       </c>
       <c r="F196" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G196" s="12" t="n">
-        <v>20007</v>
+        <v>20008</v>
       </c>
       <c r="H196" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I196" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B197" s="12" t="s">
         <v>75</v>
@@ -12587,21 +12592,21 @@
         <v>75</v>
       </c>
       <c r="F197" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G197" s="12" t="n">
-        <v>20008</v>
+        <v>30001</v>
       </c>
       <c r="H197" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I197" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B198" s="12" t="s">
         <v>75</v>
@@ -12616,21 +12621,21 @@
         <v>75</v>
       </c>
       <c r="F198" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G198" s="12" t="n">
-        <v>30001</v>
+        <v>30002</v>
       </c>
       <c r="H198" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I198" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="12" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B199" s="12" t="s">
         <v>75</v>
@@ -12645,21 +12650,21 @@
         <v>75</v>
       </c>
       <c r="F199" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G199" s="12" t="n">
-        <v>30002</v>
+        <v>30003</v>
       </c>
       <c r="H199" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I199" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="12" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B200" s="12" t="s">
         <v>75</v>
@@ -12674,21 +12679,21 @@
         <v>75</v>
       </c>
       <c r="F200" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G200" s="12" t="n">
-        <v>30003</v>
+        <v>30004</v>
       </c>
       <c r="H200" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I200" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="12" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B201" s="12" t="s">
         <v>75</v>
@@ -12703,21 +12708,21 @@
         <v>75</v>
       </c>
       <c r="F201" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G201" s="12" t="n">
-        <v>30004</v>
+        <v>30005</v>
       </c>
       <c r="H201" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I201" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="12" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B202" s="12" t="s">
         <v>75</v>
@@ -12732,21 +12737,21 @@
         <v>75</v>
       </c>
       <c r="F202" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G202" s="12" t="n">
-        <v>30005</v>
+        <v>30006</v>
       </c>
       <c r="H202" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I202" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="12" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B203" s="12" t="s">
         <v>75</v>
@@ -12761,21 +12766,21 @@
         <v>75</v>
       </c>
       <c r="F203" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G203" s="12" t="n">
-        <v>30006</v>
+        <v>40001</v>
       </c>
       <c r="H203" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I203" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="12" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B204" s="12" t="s">
         <v>75</v>
@@ -12790,21 +12795,21 @@
         <v>75</v>
       </c>
       <c r="F204" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G204" s="12" t="n">
-        <v>40001</v>
+        <v>60001</v>
       </c>
       <c r="H204" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I204" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="12" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B205" s="12" t="s">
         <v>75</v>
@@ -12819,21 +12824,21 @@
         <v>75</v>
       </c>
       <c r="F205" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G205" s="12" t="n">
-        <v>60001</v>
+        <v>60002</v>
       </c>
       <c r="H205" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I205" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="12" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B206" s="12" t="s">
         <v>75</v>
@@ -12848,21 +12853,21 @@
         <v>75</v>
       </c>
       <c r="F206" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G206" s="12" t="n">
-        <v>60002</v>
+        <v>60003</v>
       </c>
       <c r="H206" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I206" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B207" s="12" t="s">
         <v>75</v>
@@ -12877,21 +12882,21 @@
         <v>75</v>
       </c>
       <c r="F207" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G207" s="12" t="n">
-        <v>60003</v>
+        <v>60004</v>
       </c>
       <c r="H207" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I207" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B208" s="12" t="s">
         <v>75</v>
@@ -12906,21 +12911,21 @@
         <v>75</v>
       </c>
       <c r="F208" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G208" s="12" t="n">
-        <v>60004</v>
+        <v>60005</v>
       </c>
       <c r="H208" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I208" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B209" s="12" t="s">
         <v>75</v>
@@ -12935,21 +12940,21 @@
         <v>75</v>
       </c>
       <c r="F209" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G209" s="12" t="n">
-        <v>60005</v>
+        <v>60006</v>
       </c>
       <c r="H209" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I209" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B210" s="12" t="s">
         <v>75</v>
@@ -12964,21 +12969,21 @@
         <v>75</v>
       </c>
       <c r="F210" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G210" s="12" t="n">
-        <v>60006</v>
+        <v>60007</v>
       </c>
       <c r="H210" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B211" s="12" t="s">
         <v>75</v>
@@ -12993,113 +12998,113 @@
         <v>75</v>
       </c>
       <c r="F211" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G211" s="12" t="n">
-        <v>60007</v>
+        <v>60008</v>
       </c>
       <c r="H211" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I211" s="12" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A212" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B212" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C212" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E212" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F212" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G212" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H212" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I212" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="3"/>
+      <c r="B213" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C213" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D213" s="3"/>
+      <c r="E213" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F213" s="3"/>
+      <c r="G213" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H213" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I213" s="3"/>
+    </row>
+    <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A214" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="B214" s="5"/>
+      <c r="C214" s="5"/>
+      <c r="D214" s="5"/>
+      <c r="E214" s="5"/>
+      <c r="F214" s="5"/>
+      <c r="G214" s="5"/>
+      <c r="H214" s="5"/>
+      <c r="I214" s="5"/>
+    </row>
+    <row r="215" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="B215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C215" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F215" s="12" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A212" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="B212" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C212" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D212" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E212" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F212" s="12" t="s">
-        <v>333</v>
-      </c>
-      <c r="G212" s="12" t="n">
-        <v>60008</v>
-      </c>
-      <c r="H212" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I212" s="12" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A213" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B213" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C213" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D213" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E213" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F213" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G213" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H213" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I213" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A214" s="3"/>
-      <c r="B214" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C214" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D214" s="3"/>
-      <c r="E214" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F214" s="3"/>
-      <c r="G214" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H214" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I214" s="3"/>
-    </row>
-    <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A215" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="B215" s="5"/>
-      <c r="C215" s="5"/>
-      <c r="D215" s="5"/>
-      <c r="E215" s="5"/>
-      <c r="F215" s="5"/>
-      <c r="G215" s="5"/>
-      <c r="H215" s="5"/>
-      <c r="I215" s="5"/>
+      <c r="G215" s="12" t="n">
+        <v>30001</v>
+      </c>
+      <c r="H215" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I215" s="12" t="s">
+        <v>359</v>
+      </c>
     </row>
     <row r="216" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B216" s="12" t="s">
         <v>75</v>
@@ -13114,21 +13119,21 @@
         <v>75</v>
       </c>
       <c r="F216" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G216" s="12" t="n">
-        <v>30001</v>
+        <v>30002</v>
       </c>
       <c r="H216" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I216" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="12" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B217" s="12" t="s">
         <v>75</v>
@@ -13143,21 +13148,21 @@
         <v>75</v>
       </c>
       <c r="F217" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G217" s="12" t="n">
-        <v>30002</v>
+        <v>30003</v>
       </c>
       <c r="H217" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I217" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="12" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B218" s="12" t="s">
         <v>75</v>
@@ -13172,21 +13177,21 @@
         <v>75</v>
       </c>
       <c r="F218" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G218" s="12" t="n">
-        <v>30003</v>
+        <v>30004</v>
       </c>
       <c r="H218" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I218" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="12" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B219" s="12" t="s">
         <v>75</v>
@@ -13201,21 +13206,21 @@
         <v>75</v>
       </c>
       <c r="F219" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G219" s="12" t="n">
-        <v>30004</v>
+        <v>30005</v>
       </c>
       <c r="H219" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I219" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="12" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B220" s="12" t="s">
         <v>75</v>
@@ -13230,21 +13235,21 @@
         <v>75</v>
       </c>
       <c r="F220" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G220" s="12" t="n">
-        <v>30005</v>
+        <v>30006</v>
       </c>
       <c r="H220" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I220" s="12" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="221" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="12" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B221" s="12" t="s">
         <v>75</v>
@@ -13259,21 +13264,21 @@
         <v>75</v>
       </c>
       <c r="F221" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G221" s="12" t="n">
-        <v>30006</v>
+        <v>40001</v>
       </c>
       <c r="H221" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I221" s="12" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="12" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="B222" s="12" t="s">
         <v>75</v>
@@ -13288,50 +13293,50 @@
         <v>75</v>
       </c>
       <c r="F222" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G222" s="12" t="n">
-        <v>40001</v>
+        <v>45001</v>
       </c>
       <c r="H222" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I222" s="12" t="s">
-        <v>334</v>
+        <v>359</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="B223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C223" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F223" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="G223" s="12" t="n">
+        <v>60001</v>
+      </c>
+      <c r="H223" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I223" s="12" t="s">
         <v>359</v>
-      </c>
-      <c r="B223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C223" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F223" s="12" t="s">
-        <v>333</v>
-      </c>
-      <c r="G223" s="12" t="n">
-        <v>45001</v>
-      </c>
-      <c r="H223" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I223" s="12" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="12" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B224" s="12" t="s">
         <v>75</v>
@@ -13346,21 +13351,21 @@
         <v>75</v>
       </c>
       <c r="F224" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G224" s="12" t="n">
-        <v>60001</v>
+        <v>60002</v>
       </c>
       <c r="H224" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I224" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="12" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B225" s="12" t="s">
         <v>75</v>
@@ -13375,21 +13380,21 @@
         <v>75</v>
       </c>
       <c r="F225" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G225" s="12" t="n">
-        <v>60002</v>
+        <v>60003</v>
       </c>
       <c r="H225" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I225" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="12" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B226" s="12" t="s">
         <v>75</v>
@@ -13404,21 +13409,21 @@
         <v>75</v>
       </c>
       <c r="F226" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G226" s="12" t="n">
-        <v>60003</v>
+        <v>60004</v>
       </c>
       <c r="H226" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I226" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="12" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B227" s="12" t="s">
         <v>75</v>
@@ -13433,21 +13438,21 @@
         <v>75</v>
       </c>
       <c r="F227" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G227" s="12" t="n">
-        <v>60004</v>
+        <v>60005</v>
       </c>
       <c r="H227" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I227" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="12" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B228" s="12" t="s">
         <v>75</v>
@@ -13462,21 +13467,21 @@
         <v>75</v>
       </c>
       <c r="F228" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G228" s="12" t="n">
-        <v>60005</v>
+        <v>60006</v>
       </c>
       <c r="H228" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I228" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="12" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B229" s="12" t="s">
         <v>75</v>
@@ -13491,21 +13496,21 @@
         <v>75</v>
       </c>
       <c r="F229" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G229" s="12" t="n">
-        <v>60006</v>
+        <v>60007</v>
       </c>
       <c r="H229" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I229" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="12" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B230" s="12" t="s">
         <v>75</v>
@@ -13520,113 +13525,113 @@
         <v>75</v>
       </c>
       <c r="F230" s="12" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G230" s="12" t="n">
-        <v>60007</v>
+        <v>60008</v>
       </c>
       <c r="H230" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I230" s="12" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="231" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A231" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="B231" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C231" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D231" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E231" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F231" s="12" t="s">
-        <v>333</v>
-      </c>
-      <c r="G231" s="12" t="n">
-        <v>60008</v>
-      </c>
-      <c r="H231" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I231" s="12" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A232" s="3" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A231" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="B231" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C231" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D231" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E231" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F231" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G231" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H231" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I231" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="3"/>
       <c r="B232" s="4" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C232" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D232" s="3" t="s">
-        <v>11</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="D232" s="3"/>
       <c r="E232" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F232" s="3" t="s">
-        <v>13</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="F232" s="3"/>
       <c r="G232" s="4" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H232" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I232" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A233" s="3"/>
-      <c r="B233" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C233" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D233" s="3"/>
-      <c r="E233" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F233" s="3"/>
-      <c r="G233" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H233" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I233" s="3"/>
-    </row>
-    <row r="234" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A234" s="5" t="s">
+      <c r="I232" s="3"/>
+    </row>
+    <row r="233" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A233" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="B234" s="5"/>
-      <c r="C234" s="5"/>
-      <c r="D234" s="5"/>
-      <c r="E234" s="5"/>
-      <c r="F234" s="5"/>
-      <c r="G234" s="5"/>
-      <c r="H234" s="5"/>
-      <c r="I234" s="5"/>
+      <c r="B233" s="5"/>
+      <c r="C233" s="5"/>
+      <c r="D233" s="5"/>
+      <c r="E233" s="5"/>
+      <c r="F233" s="5"/>
+      <c r="G233" s="5"/>
+      <c r="H233" s="5"/>
+      <c r="I233" s="5"/>
+    </row>
+    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B234" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C234" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D234" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E234" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F234" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G234" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="H234" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I234" s="7" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="9" t="s">
-        <v>108</v>
+        <v>187</v>
       </c>
       <c r="B235" s="7" t="s">
         <v>109</v>
@@ -13644,21 +13649,21 @@
         <v>26</v>
       </c>
       <c r="G235" s="10" t="s">
-        <v>318</v>
+        <v>188</v>
       </c>
       <c r="H235" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I235" s="7" t="s">
-        <v>112</v>
+        <v>189</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="9" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="B236" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C236" s="7" t="s">
         <v>110</v>
@@ -13673,18 +13678,16 @@
         <v>26</v>
       </c>
       <c r="G236" s="10" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="H236" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I236" s="7" t="s">
-        <v>189</v>
-      </c>
+      <c r="I236" s="7"/>
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="9" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B237" s="7" t="s">
         <v>24</v>
@@ -13702,7 +13705,7 @@
         <v>26</v>
       </c>
       <c r="G237" s="10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H237" s="7" t="n">
         <v>2</v>
@@ -13711,7 +13714,7 @@
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="9" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B238" s="7" t="s">
         <v>24</v>
@@ -13729,7 +13732,7 @@
         <v>26</v>
       </c>
       <c r="G238" s="10" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H238" s="7" t="n">
         <v>2</v>
@@ -13738,7 +13741,7 @@
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="9" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B239" s="7" t="s">
         <v>24</v>
@@ -13756,7 +13759,7 @@
         <v>26</v>
       </c>
       <c r="G239" s="10" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H239" s="7" t="n">
         <v>2</v>
@@ -13765,10 +13768,10 @@
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="9" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B240" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C240" s="7" t="s">
         <v>110</v>
@@ -13783,7 +13786,7 @@
         <v>26</v>
       </c>
       <c r="G240" s="10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H240" s="7" t="n">
         <v>2</v>
@@ -13792,7 +13795,7 @@
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B241" s="7" t="s">
         <v>109</v>
@@ -13810,7 +13813,7 @@
         <v>26</v>
       </c>
       <c r="G241" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H241" s="7" t="n">
         <v>2</v>
@@ -13819,10 +13822,10 @@
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B242" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C242" s="7" t="s">
         <v>110</v>
@@ -13837,7 +13840,7 @@
         <v>26</v>
       </c>
       <c r="G242" s="10" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="H242" s="7" t="n">
         <v>2</v>
@@ -13846,7 +13849,7 @@
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B243" s="7" t="s">
         <v>24</v>
@@ -13864,7 +13867,7 @@
         <v>26</v>
       </c>
       <c r="G243" s="10" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H243" s="7" t="n">
         <v>2</v>
@@ -13873,7 +13876,7 @@
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="9" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B244" s="7" t="s">
         <v>24</v>
@@ -13891,7 +13894,7 @@
         <v>26</v>
       </c>
       <c r="G244" s="10" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H244" s="7" t="n">
         <v>2</v>
@@ -13900,7 +13903,7 @@
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="9" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B245" s="7" t="s">
         <v>24</v>
@@ -13918,7 +13921,7 @@
         <v>26</v>
       </c>
       <c r="G245" s="10" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="H245" s="7" t="n">
         <v>2</v>
@@ -13927,10 +13930,10 @@
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="9" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B246" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C246" s="7" t="s">
         <v>110</v>
@@ -13945,7 +13948,7 @@
         <v>26</v>
       </c>
       <c r="G246" s="10" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="H246" s="7" t="n">
         <v>2</v>
@@ -13954,7 +13957,7 @@
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="9" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B247" s="7" t="s">
         <v>109</v>
@@ -13972,7 +13975,7 @@
         <v>26</v>
       </c>
       <c r="G247" s="10" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="H247" s="7" t="n">
         <v>2</v>
@@ -13981,10 +13984,10 @@
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="9" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B248" s="7" t="s">
-        <v>109</v>
+        <v>222</v>
       </c>
       <c r="C248" s="7" t="s">
         <v>110</v>
@@ -13999,7 +14002,7 @@
         <v>26</v>
       </c>
       <c r="G248" s="10" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="H248" s="7" t="n">
         <v>2</v>
@@ -14008,7 +14011,7 @@
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="9" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B249" s="7" t="s">
         <v>222</v>
@@ -14026,7 +14029,7 @@
         <v>26</v>
       </c>
       <c r="G249" s="10" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="H249" s="7" t="n">
         <v>2</v>
@@ -14035,10 +14038,10 @@
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="9" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B250" s="7" t="s">
-        <v>222</v>
+        <v>195</v>
       </c>
       <c r="C250" s="7" t="s">
         <v>110</v>
@@ -14053,7 +14056,7 @@
         <v>26</v>
       </c>
       <c r="G250" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="H250" s="7" t="n">
         <v>2</v>
@@ -14062,7 +14065,7 @@
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="9" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B251" s="7" t="s">
         <v>195</v>
@@ -14080,7 +14083,7 @@
         <v>26</v>
       </c>
       <c r="G251" s="10" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="H251" s="7" t="n">
         <v>2</v>
@@ -14089,10 +14092,10 @@
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="9" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B252" s="7" t="s">
-        <v>195</v>
+        <v>109</v>
       </c>
       <c r="C252" s="7" t="s">
         <v>110</v>
@@ -14107,7 +14110,7 @@
         <v>26</v>
       </c>
       <c r="G252" s="10" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="H252" s="7" t="n">
         <v>2</v>
@@ -14116,7 +14119,7 @@
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="9" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B253" s="7" t="s">
         <v>109</v>
@@ -14134,7 +14137,7 @@
         <v>26</v>
       </c>
       <c r="G253" s="10" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H253" s="7" t="n">
         <v>2</v>
@@ -14142,11 +14145,11 @@
       <c r="I253" s="7"/>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A254" s="9" t="s">
-        <v>232</v>
+      <c r="A254" s="7" t="s">
+        <v>234</v>
       </c>
       <c r="B254" s="7" t="s">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="C254" s="7" t="s">
         <v>110</v>
@@ -14161,16 +14164,18 @@
         <v>26</v>
       </c>
       <c r="G254" s="10" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="H254" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I254" s="7"/>
+      <c r="I254" s="7" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="7" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B255" s="7" t="s">
         <v>75</v>
@@ -14188,7 +14193,7 @@
         <v>26</v>
       </c>
       <c r="G255" s="10" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="H255" s="7" t="n">
         <v>2</v>
@@ -14197,38 +14202,38 @@
         <v>236</v>
       </c>
     </row>
-    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A256" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="B256" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C256" s="7" t="s">
+    <row r="256" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A256" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="B256" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C256" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D256" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E256" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F256" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G256" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="H256" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I256" s="7" t="s">
-        <v>236</v>
+      <c r="D256" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E256" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F256" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G256" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="H256" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I256" s="14" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="12" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B257" s="12" t="s">
         <v>75</v>
@@ -14246,18 +14251,18 @@
         <v>26</v>
       </c>
       <c r="G257" s="12" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="H257" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I257" s="14" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="258" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A258" s="12" t="s">
-        <v>241</v>
+        <v>362</v>
+      </c>
+    </row>
+    <row r="258" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="11" t="s">
+        <v>322</v>
       </c>
       <c r="B258" s="12" t="s">
         <v>75</v>
@@ -14274,19 +14279,19 @@
       <c r="F258" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="G258" s="12" t="s">
-        <v>242</v>
+      <c r="G258" s="13" t="s">
+        <v>323</v>
       </c>
       <c r="H258" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I258" s="14" t="s">
-        <v>361</v>
+      <c r="I258" s="12" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="259" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="11" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B259" s="12" t="s">
         <v>75</v>
@@ -14304,18 +14309,18 @@
         <v>26</v>
       </c>
       <c r="G259" s="13" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="H259" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I259" s="12" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="260" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="260" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="11" t="s">
-        <v>325</v>
+        <v>365</v>
       </c>
       <c r="B260" s="12" t="s">
         <v>75</v>
@@ -14333,44 +14338,16 @@
         <v>26</v>
       </c>
       <c r="G260" s="13" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="H260" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I260" s="12" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="261" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A261" s="11" t="s">
-        <v>364</v>
-      </c>
-      <c r="B261" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C261" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D261" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E261" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F261" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G261" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="H261" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I261" s="12" t="s">
-        <v>365</v>
-      </c>
-    </row>
+        <v>366</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="25">
     <mergeCell ref="A6:A7"/>
@@ -14383,21 +14360,21 @@
     <mergeCell ref="F115:F116"/>
     <mergeCell ref="I115:I116"/>
     <mergeCell ref="A117:I117"/>
-    <mergeCell ref="A187:A188"/>
-    <mergeCell ref="D187:D188"/>
-    <mergeCell ref="F187:F188"/>
-    <mergeCell ref="I187:I188"/>
-    <mergeCell ref="A189:I189"/>
-    <mergeCell ref="A213:A214"/>
-    <mergeCell ref="D213:D214"/>
-    <mergeCell ref="F213:F214"/>
-    <mergeCell ref="I213:I214"/>
-    <mergeCell ref="A215:I215"/>
-    <mergeCell ref="A232:A233"/>
-    <mergeCell ref="D232:D233"/>
-    <mergeCell ref="F232:F233"/>
-    <mergeCell ref="I232:I233"/>
-    <mergeCell ref="A234:I234"/>
+    <mergeCell ref="A186:A187"/>
+    <mergeCell ref="D186:D187"/>
+    <mergeCell ref="F186:F187"/>
+    <mergeCell ref="I186:I187"/>
+    <mergeCell ref="A188:I188"/>
+    <mergeCell ref="A212:A213"/>
+    <mergeCell ref="D212:D213"/>
+    <mergeCell ref="F212:F213"/>
+    <mergeCell ref="I212:I213"/>
+    <mergeCell ref="A214:I214"/>
+    <mergeCell ref="A231:A232"/>
+    <mergeCell ref="D231:D232"/>
+    <mergeCell ref="F231:F232"/>
+    <mergeCell ref="I231:I232"/>
+    <mergeCell ref="A233:I233"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
SOCO: Bugfix: Check RELAY 6 also during manual self-test
Relay 6 wasn't being used earlier. Now it's in used so should test it in
manual self-test also.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -1022,58 +1022,16 @@
     <t xml:space="preserve">50013</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Internal Only. Not visible to customer. 
+    <t xml:space="preserve">Internal Only. Not visible to customer. 
 Indicates the state machine of calibration
-0: Calibration Not Initiated. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 20A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. Set Fan 1 Current and Fan 2 current to 0.1A each. And then s</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">et Advance Calibration Flag.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-16,17,18,19: High Point Calibration In Progress
-20: High Point Calibration Done. </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
-21,22,23: Mid Point Calibration In Progress
-24: Mid Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 0.4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
-25,26,27: Low Point Calibration In Progress
+0: Calibration Not Initiated. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 20A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. Set Fan 1 Current and Fan 2 current to 0.1A each. And then set Advance Calibration Flag.
+17,18,19,20: High Point Calibration In Progress
+21: High Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
+22,23,24: Mid Point Calibration In Progress
+25: Mid Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 0.4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
+26,27,28: Low Point Calibration In Progress
 127: Calibration Completed Successfully
 126: Error occured during calibration. Please restart controller</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">Load On Grid Contactor &amp; Solar Neutral Earth Contactor Coil</t>
@@ -1181,55 +1139,15 @@
 If set to non-zero, indicates product was tested functionally during production. Only writtable when test mode enabled.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Internal Only. Not visible to customer. 
-If set to non-zero, indicates product was calibrated during production. </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">Only writtable when test mode enabled.</t>
-    </r>
+    <t xml:space="preserve">Internal Only. Not visible to customer. 
+If set to non-zero, indicates product was calibrated during production. Only writtable when test mode enabled.</t>
   </si>
   <si>
     <t xml:space="preserve">Advance Calibration State</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Internal Only. Not visible to customer. 
-If set to non-zero, it advances the calibration state machine when it is waiting for external input. </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="8"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">Only writtable when test mode enabled.</t>
-    </r>
+    <t xml:space="preserve">Internal Only. Not visible to customer. 
+If set to non-zero, it advances the calibration state machine when it is waiting for external input. Only writtable when test mode enabled.</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1157,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1291,13 +1209,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1419,7 +1330,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1474,10 +1385,6 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -13073,7 +12980,7 @@
       <c r="H214" s="5"/>
       <c r="I214" s="5"/>
     </row>
-    <row r="215" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="12" t="s">
         <v>343</v>
       </c>
@@ -13102,7 +13009,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="12" t="s">
         <v>344</v>
       </c>
@@ -13131,7 +13038,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="12" t="s">
         <v>345</v>
       </c>
@@ -13160,7 +13067,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="12" t="s">
         <v>346</v>
       </c>
@@ -13189,7 +13096,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="12" t="s">
         <v>347</v>
       </c>
@@ -13218,7 +13125,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="12" t="s">
         <v>348</v>
       </c>
@@ -13276,7 +13183,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="12" t="s">
         <v>360</v>
       </c>
@@ -13305,7 +13212,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="12" t="s">
         <v>350</v>
       </c>
@@ -13334,7 +13241,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="12" t="s">
         <v>351</v>
       </c>
@@ -13363,7 +13270,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="12" t="s">
         <v>352</v>
       </c>
@@ -13392,7 +13299,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="12" t="s">
         <v>353</v>
       </c>
@@ -13421,7 +13328,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="12" t="s">
         <v>354</v>
       </c>
@@ -13450,7 +13357,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="12" t="s">
         <v>355</v>
       </c>
@@ -13479,7 +13386,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="12" t="s">
         <v>356</v>
       </c>
@@ -13508,7 +13415,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="19.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="12" t="s">
         <v>357</v>
       </c>
@@ -14202,7 +14109,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="256" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="256" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="12" t="s">
         <v>239</v>
       </c>
@@ -14227,11 +14134,11 @@
       <c r="H256" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I256" s="14" t="s">
+      <c r="I256" s="12" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="257" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="257" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="12" t="s">
         <v>241</v>
       </c>
@@ -14256,7 +14163,7 @@
       <c r="H257" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="I257" s="14" t="s">
+      <c r="I257" s="12" t="s">
         <v>362</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SOCO: Improvement: Allow "Calibration Done" flag to be selectively set
Allow this flag to be only set when calibration is truely set.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -1136,11 +1136,11 @@
   </si>
   <si>
     <t xml:space="preserve">Internal Only. Not visible to customer. 
-If set to non-zero, indicates product was tested functionally during production. Only writtable when test mode enabled.</t>
+If set to non-zero, indicates product was tested functionally during production. Only writtable when test mode enabled. Suggested to write the Unix Timestamp for the time when the product was functionally tested.</t>
   </si>
   <si>
     <t xml:space="preserve">Internal Only. Not visible to customer. 
-If set to non-zero, indicates product was calibrated during production. Only writtable when test mode enabled.</t>
+If set to non-zero, indicates product was calibrated during production. Only writtable when test mode enabled. Suggested to write Unix Epoch Timestamp of the time when calibration took place</t>
   </si>
   <si>
     <t xml:space="preserve">Advance Calibration State</t>
@@ -14167,7 +14167,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="258" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="258" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="11" t="s">
         <v>322</v>
       </c>
@@ -14196,7 +14196,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="259" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="259" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="11" t="s">
         <v>325</v>
       </c>

</xml_diff>

<commit_message>
SOCO: Feature: Expose under-volt/over-volt flags over modbus
Added these flags as per modbus table
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="375">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -978,6 +978,15 @@
   </si>
   <si>
     <t xml:space="preserve">6001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DG Detection Disable Setting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0: OFF (DG Detection Enabled), 1: ON (DG Detection Disabled)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0: OFF (Fans Enabled), 1: ON (Fans Disabled)</t>
   </si>
   <si>
     <t xml:space="preserve">Switch Pressed</t>
@@ -1034,7 +1043,22 @@
 126: Error occured during calibration. Please restart controller</t>
   </si>
   <si>
-    <t xml:space="preserve">Load On Grid Contactor &amp; Solar Neutral Earth Contactor Coil</t>
+    <t xml:space="preserve">Grid R Phase Contactor Coil Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grid Y Phase Contactor Coil Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grid B Phase Contactor Coil Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load On Solar Contactor Coil Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load On Grid Contactor &amp; Solar Neutral Earth Contactor Coil Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fans Output</t>
   </si>
   <si>
     <t xml:space="preserve">READ COIL STATUS (Function Code: 0x01)</t>
@@ -10035,7 +10059,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="s">
-        <v>234</v>
+        <v>319</v>
       </c>
       <c r="B106" s="7" t="s">
         <v>75</v>
@@ -10059,7 +10083,7 @@
         <v>2</v>
       </c>
       <c r="I106" s="7" t="s">
-        <v>236</v>
+        <v>320</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10088,12 +10112,12 @@
         <v>2</v>
       </c>
       <c r="I107" s="7" t="s">
-        <v>236</v>
+        <v>321</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="86.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="11" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B108" s="12" t="s">
         <v>75</v>
@@ -10111,13 +10135,13 @@
         <v>26</v>
       </c>
       <c r="G108" s="13" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="H108" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I108" s="12" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10203,7 +10227,7 @@
     </row>
     <row r="112" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="11" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B112" s="12" t="s">
         <v>75</v>
@@ -10221,18 +10245,18 @@
         <v>26</v>
       </c>
       <c r="G112" s="13" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="H112" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I112" s="12" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B113" s="12" t="s">
         <v>75</v>
@@ -10250,18 +10274,18 @@
         <v>26</v>
       </c>
       <c r="G113" s="13" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="H113" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I113" s="12" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="236.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="11" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B114" s="12" t="s">
         <v>75</v>
@@ -10279,13 +10303,13 @@
         <v>26</v>
       </c>
       <c r="G114" s="13" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="H114" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I114" s="12" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10947,7 +10971,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="7" t="s">
-        <v>270</v>
+        <v>334</v>
       </c>
       <c r="B140" s="7" t="s">
         <v>75</v>
@@ -10974,7 +10998,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="7" t="s">
-        <v>271</v>
+        <v>335</v>
       </c>
       <c r="B141" s="7" t="s">
         <v>75</v>
@@ -11001,7 +11025,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="7" t="s">
-        <v>272</v>
+        <v>336</v>
       </c>
       <c r="B142" s="7" t="s">
         <v>75</v>
@@ -11028,7 +11052,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="7" t="s">
-        <v>273</v>
+        <v>337</v>
       </c>
       <c r="B143" s="7" t="s">
         <v>75</v>
@@ -11055,7 +11079,7 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="7" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="B144" s="7" t="s">
         <v>75</v>
@@ -11082,7 +11106,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="7" t="s">
-        <v>276</v>
+        <v>339</v>
       </c>
       <c r="B145" s="7" t="s">
         <v>75</v>
@@ -12239,7 +12263,7 @@
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="5" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="B188" s="5"/>
       <c r="C188" s="5"/>
@@ -12252,7 +12276,7 @@
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="12" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B189" s="12" t="s">
         <v>75</v>
@@ -12267,7 +12291,7 @@
         <v>75</v>
       </c>
       <c r="F189" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G189" s="12" t="n">
         <v>20001</v>
@@ -12276,12 +12300,12 @@
         <v>1</v>
       </c>
       <c r="I189" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="12" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="B190" s="12" t="s">
         <v>75</v>
@@ -12296,7 +12320,7 @@
         <v>75</v>
       </c>
       <c r="F190" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G190" s="12" t="n">
         <v>20002</v>
@@ -12305,12 +12329,12 @@
         <v>1</v>
       </c>
       <c r="I190" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="12" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="B191" s="12" t="s">
         <v>75</v>
@@ -12325,7 +12349,7 @@
         <v>75</v>
       </c>
       <c r="F191" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G191" s="12" t="n">
         <v>20003</v>
@@ -12334,12 +12358,12 @@
         <v>1</v>
       </c>
       <c r="I191" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="12" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="B192" s="12" t="s">
         <v>75</v>
@@ -12354,7 +12378,7 @@
         <v>75</v>
       </c>
       <c r="F192" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G192" s="12" t="n">
         <v>20004</v>
@@ -12363,12 +12387,12 @@
         <v>1</v>
       </c>
       <c r="I192" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="12" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="B193" s="12" t="s">
         <v>75</v>
@@ -12383,7 +12407,7 @@
         <v>75</v>
       </c>
       <c r="F193" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G193" s="12" t="n">
         <v>20005</v>
@@ -12392,12 +12416,12 @@
         <v>1</v>
       </c>
       <c r="I193" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="12" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="B194" s="12" t="s">
         <v>75</v>
@@ -12412,7 +12436,7 @@
         <v>75</v>
       </c>
       <c r="F194" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G194" s="12" t="n">
         <v>20006</v>
@@ -12421,12 +12445,12 @@
         <v>1</v>
       </c>
       <c r="I194" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="12" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B195" s="12" t="s">
         <v>75</v>
@@ -12441,7 +12465,7 @@
         <v>75</v>
       </c>
       <c r="F195" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G195" s="12" t="n">
         <v>20007</v>
@@ -12450,27 +12474,27 @@
         <v>1</v>
       </c>
       <c r="I195" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="B196" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C196" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D196" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E196" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F196" s="12" t="s">
         <v>342</v>
-      </c>
-      <c r="B196" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C196" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D196" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E196" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F196" s="12" t="s">
-        <v>334</v>
       </c>
       <c r="G196" s="12" t="n">
         <v>20008</v>
@@ -12479,12 +12503,12 @@
         <v>1</v>
       </c>
       <c r="I196" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="12" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="B197" s="12" t="s">
         <v>75</v>
@@ -12499,7 +12523,7 @@
         <v>75</v>
       </c>
       <c r="F197" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G197" s="12" t="n">
         <v>30001</v>
@@ -12508,12 +12532,12 @@
         <v>1</v>
       </c>
       <c r="I197" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="12" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="B198" s="12" t="s">
         <v>75</v>
@@ -12528,7 +12552,7 @@
         <v>75</v>
       </c>
       <c r="F198" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G198" s="12" t="n">
         <v>30002</v>
@@ -12537,12 +12561,12 @@
         <v>1</v>
       </c>
       <c r="I198" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="12" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B199" s="12" t="s">
         <v>75</v>
@@ -12557,7 +12581,7 @@
         <v>75</v>
       </c>
       <c r="F199" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G199" s="12" t="n">
         <v>30003</v>
@@ -12566,12 +12590,12 @@
         <v>1</v>
       </c>
       <c r="I199" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="12" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="B200" s="12" t="s">
         <v>75</v>
@@ -12586,7 +12610,7 @@
         <v>75</v>
       </c>
       <c r="F200" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G200" s="12" t="n">
         <v>30004</v>
@@ -12595,12 +12619,12 @@
         <v>1</v>
       </c>
       <c r="I200" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="12" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="B201" s="12" t="s">
         <v>75</v>
@@ -12615,7 +12639,7 @@
         <v>75</v>
       </c>
       <c r="F201" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G201" s="12" t="n">
         <v>30005</v>
@@ -12624,12 +12648,12 @@
         <v>1</v>
       </c>
       <c r="I201" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="12" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="B202" s="12" t="s">
         <v>75</v>
@@ -12644,7 +12668,7 @@
         <v>75</v>
       </c>
       <c r="F202" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G202" s="12" t="n">
         <v>30006</v>
@@ -12653,12 +12677,12 @@
         <v>1</v>
       </c>
       <c r="I202" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="12" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="B203" s="12" t="s">
         <v>75</v>
@@ -12673,7 +12697,7 @@
         <v>75</v>
       </c>
       <c r="F203" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G203" s="12" t="n">
         <v>40001</v>
@@ -12682,12 +12706,12 @@
         <v>1</v>
       </c>
       <c r="I203" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="12" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B204" s="12" t="s">
         <v>75</v>
@@ -12702,7 +12726,7 @@
         <v>75</v>
       </c>
       <c r="F204" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G204" s="12" t="n">
         <v>60001</v>
@@ -12711,12 +12735,12 @@
         <v>1</v>
       </c>
       <c r="I204" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="12" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="B205" s="12" t="s">
         <v>75</v>
@@ -12731,7 +12755,7 @@
         <v>75</v>
       </c>
       <c r="F205" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G205" s="12" t="n">
         <v>60002</v>
@@ -12740,12 +12764,12 @@
         <v>1</v>
       </c>
       <c r="I205" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="12" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B206" s="12" t="s">
         <v>75</v>
@@ -12760,7 +12784,7 @@
         <v>75</v>
       </c>
       <c r="F206" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G206" s="12" t="n">
         <v>60003</v>
@@ -12769,12 +12793,12 @@
         <v>1</v>
       </c>
       <c r="I206" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="12" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="B207" s="12" t="s">
         <v>75</v>
@@ -12789,7 +12813,7 @@
         <v>75</v>
       </c>
       <c r="F207" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G207" s="12" t="n">
         <v>60004</v>
@@ -12798,12 +12822,12 @@
         <v>1</v>
       </c>
       <c r="I207" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B208" s="12" t="s">
         <v>75</v>
@@ -12818,7 +12842,7 @@
         <v>75</v>
       </c>
       <c r="F208" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G208" s="12" t="n">
         <v>60005</v>
@@ -12827,12 +12851,12 @@
         <v>1</v>
       </c>
       <c r="I208" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="B209" s="12" t="s">
         <v>75</v>
@@ -12847,7 +12871,7 @@
         <v>75</v>
       </c>
       <c r="F209" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G209" s="12" t="n">
         <v>60006</v>
@@ -12856,12 +12880,12 @@
         <v>1</v>
       </c>
       <c r="I209" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="B210" s="12" t="s">
         <v>75</v>
@@ -12876,7 +12900,7 @@
         <v>75</v>
       </c>
       <c r="F210" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G210" s="12" t="n">
         <v>60007</v>
@@ -12885,12 +12909,12 @@
         <v>1</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="B211" s="12" t="s">
         <v>75</v>
@@ -12905,7 +12929,7 @@
         <v>75</v>
       </c>
       <c r="F211" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G211" s="12" t="n">
         <v>60008</v>
@@ -12914,7 +12938,7 @@
         <v>1</v>
       </c>
       <c r="I211" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12969,7 +12993,7 @@
     </row>
     <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="5" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="B214" s="5"/>
       <c r="C214" s="5"/>
@@ -12982,7 +13006,7 @@
     </row>
     <row r="215" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="12" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="B215" s="12" t="s">
         <v>75</v>
@@ -12997,7 +13021,7 @@
         <v>75</v>
       </c>
       <c r="F215" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G215" s="12" t="n">
         <v>30001</v>
@@ -13006,12 +13030,12 @@
         <v>1</v>
       </c>
       <c r="I215" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="12" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="B216" s="12" t="s">
         <v>75</v>
@@ -13026,7 +13050,7 @@
         <v>75</v>
       </c>
       <c r="F216" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G216" s="12" t="n">
         <v>30002</v>
@@ -13035,12 +13059,12 @@
         <v>1</v>
       </c>
       <c r="I216" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="12" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B217" s="12" t="s">
         <v>75</v>
@@ -13055,7 +13079,7 @@
         <v>75</v>
       </c>
       <c r="F217" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G217" s="12" t="n">
         <v>30003</v>
@@ -13064,12 +13088,12 @@
         <v>1</v>
       </c>
       <c r="I217" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="12" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="B218" s="12" t="s">
         <v>75</v>
@@ -13084,7 +13108,7 @@
         <v>75</v>
       </c>
       <c r="F218" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G218" s="12" t="n">
         <v>30004</v>
@@ -13093,12 +13117,12 @@
         <v>1</v>
       </c>
       <c r="I218" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="12" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="B219" s="12" t="s">
         <v>75</v>
@@ -13113,7 +13137,7 @@
         <v>75</v>
       </c>
       <c r="F219" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G219" s="12" t="n">
         <v>30005</v>
@@ -13122,12 +13146,12 @@
         <v>1</v>
       </c>
       <c r="I219" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="12" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="B220" s="12" t="s">
         <v>75</v>
@@ -13142,7 +13166,7 @@
         <v>75</v>
       </c>
       <c r="F220" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G220" s="12" t="n">
         <v>30006</v>
@@ -13151,12 +13175,12 @@
         <v>1</v>
       </c>
       <c r="I220" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="12" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="B221" s="12" t="s">
         <v>75</v>
@@ -13171,7 +13195,7 @@
         <v>75</v>
       </c>
       <c r="F221" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G221" s="12" t="n">
         <v>40001</v>
@@ -13180,12 +13204,12 @@
         <v>1</v>
       </c>
       <c r="I221" s="12" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="12" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="B222" s="12" t="s">
         <v>75</v>
@@ -13200,7 +13224,7 @@
         <v>75</v>
       </c>
       <c r="F222" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G222" s="12" t="n">
         <v>45001</v>
@@ -13209,12 +13233,12 @@
         <v>1</v>
       </c>
       <c r="I222" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="12" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B223" s="12" t="s">
         <v>75</v>
@@ -13229,7 +13253,7 @@
         <v>75</v>
       </c>
       <c r="F223" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G223" s="12" t="n">
         <v>60001</v>
@@ -13238,12 +13262,12 @@
         <v>1</v>
       </c>
       <c r="I223" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="12" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="B224" s="12" t="s">
         <v>75</v>
@@ -13258,7 +13282,7 @@
         <v>75</v>
       </c>
       <c r="F224" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G224" s="12" t="n">
         <v>60002</v>
@@ -13267,12 +13291,12 @@
         <v>1</v>
       </c>
       <c r="I224" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="12" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B225" s="12" t="s">
         <v>75</v>
@@ -13287,7 +13311,7 @@
         <v>75</v>
       </c>
       <c r="F225" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G225" s="12" t="n">
         <v>60003</v>
@@ -13296,12 +13320,12 @@
         <v>1</v>
       </c>
       <c r="I225" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="12" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="B226" s="12" t="s">
         <v>75</v>
@@ -13316,7 +13340,7 @@
         <v>75</v>
       </c>
       <c r="F226" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G226" s="12" t="n">
         <v>60004</v>
@@ -13325,12 +13349,12 @@
         <v>1</v>
       </c>
       <c r="I226" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="12" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B227" s="12" t="s">
         <v>75</v>
@@ -13345,7 +13369,7 @@
         <v>75</v>
       </c>
       <c r="F227" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G227" s="12" t="n">
         <v>60005</v>
@@ -13354,12 +13378,12 @@
         <v>1</v>
       </c>
       <c r="I227" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="12" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="B228" s="12" t="s">
         <v>75</v>
@@ -13374,7 +13398,7 @@
         <v>75</v>
       </c>
       <c r="F228" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G228" s="12" t="n">
         <v>60006</v>
@@ -13383,12 +13407,12 @@
         <v>1</v>
       </c>
       <c r="I228" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="12" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="B229" s="12" t="s">
         <v>75</v>
@@ -13403,7 +13427,7 @@
         <v>75</v>
       </c>
       <c r="F229" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G229" s="12" t="n">
         <v>60007</v>
@@ -13412,12 +13436,12 @@
         <v>1</v>
       </c>
       <c r="I229" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="12" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="B230" s="12" t="s">
         <v>75</v>
@@ -13432,7 +13456,7 @@
         <v>75</v>
       </c>
       <c r="F230" s="12" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="G230" s="12" t="n">
         <v>60008</v>
@@ -13441,7 +13465,7 @@
         <v>1</v>
       </c>
       <c r="I230" s="12" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -14077,7 +14101,7 @@
         <v>2</v>
       </c>
       <c r="I254" s="7" t="s">
-        <v>236</v>
+        <v>320</v>
       </c>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14106,7 +14130,7 @@
         <v>2</v>
       </c>
       <c r="I255" s="7" t="s">
-        <v>236</v>
+        <v>321</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14135,7 +14159,7 @@
         <v>2</v>
       </c>
       <c r="I256" s="12" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
     </row>
     <row r="257" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14164,12 +14188,12 @@
         <v>2</v>
       </c>
       <c r="I257" s="12" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="258" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="11" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B258" s="12" t="s">
         <v>75</v>
@@ -14187,18 +14211,18 @@
         <v>26</v>
       </c>
       <c r="G258" s="13" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="H258" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I258" s="12" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
     </row>
     <row r="259" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="11" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B259" s="12" t="s">
         <v>75</v>
@@ -14216,18 +14240,18 @@
         <v>26</v>
       </c>
       <c r="G259" s="13" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="H259" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I259" s="12" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
     </row>
     <row r="260" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="11" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="B260" s="12" t="s">
         <v>75</v>
@@ -14245,13 +14269,13 @@
         <v>26</v>
       </c>
       <c r="G260" s="13" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="H260" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I260" s="12" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
SOCO: Feature: Add flags for visibility in contactor state
Added flags over modbus that helps figure out why a contactor is
closed/not closed.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2571" uniqueCount="384">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -1059,6 +1059,33 @@
   </si>
   <si>
     <t xml:space="preserve">Fans Output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load On Grid </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Not On Grid  As User Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Not On Grid As Grid R Phase Unhealthy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Not On Grid As Solar Contactors On</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load On Solar </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Not On Solar As User Disabled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Not On Solar As Solar R Phase Unhealthy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Not On Solar As Grid Contactors On</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load Not On Solar As DG Running</t>
   </si>
   <si>
     <t xml:space="preserve">READ COIL STATUS (Function Code: 0x01)</t>
@@ -7286,7 +7313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:I265"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.94"/>
@@ -12105,7 +12132,7 @@
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="7" t="s">
-        <v>313</v>
+        <v>340</v>
       </c>
       <c r="B182" s="7" t="s">
         <v>75</v>
@@ -12132,7 +12159,7 @@
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="7" t="s">
-        <v>314</v>
+        <v>341</v>
       </c>
       <c r="B183" s="7" t="s">
         <v>75</v>
@@ -12159,7 +12186,7 @@
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="7" t="s">
-        <v>315</v>
+        <v>342</v>
       </c>
       <c r="B184" s="7" t="s">
         <v>75</v>
@@ -12186,7 +12213,7 @@
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="7" t="s">
-        <v>316</v>
+        <v>343</v>
       </c>
       <c r="B185" s="7" t="s">
         <v>75</v>
@@ -12211,217 +12238,207 @@
       </c>
       <c r="I185" s="7"/>
     </row>
-    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A186" s="3" t="s">
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="B186" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C186" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D186" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E186" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F186" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="G186" s="7" t="n">
+        <v>805</v>
+      </c>
+      <c r="H186" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I186" s="7"/>
+    </row>
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="B187" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C187" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D187" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E187" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F187" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="G187" s="7" t="n">
+        <v>806</v>
+      </c>
+      <c r="H187" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I187" s="7"/>
+    </row>
+    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="B188" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C188" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D188" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E188" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F188" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="G188" s="7" t="n">
+        <v>807</v>
+      </c>
+      <c r="H188" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I188" s="7"/>
+    </row>
+    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="B189" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C189" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D189" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E189" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F189" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="G189" s="7" t="n">
+        <v>808</v>
+      </c>
+      <c r="H189" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I189" s="7"/>
+    </row>
+    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A190" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="B190" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C190" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="D190" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E190" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F190" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="G190" s="7" t="n">
+        <v>809</v>
+      </c>
+      <c r="H190" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I190" s="7"/>
+    </row>
+    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A191" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B186" s="4" t="s">
+      <c r="B191" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C186" s="4" t="s">
+      <c r="C191" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D186" s="3" t="s">
+      <c r="D191" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E186" s="4" t="s">
+      <c r="E191" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F186" s="3" t="s">
+      <c r="F191" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G186" s="4" t="s">
+      <c r="G191" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H186" s="4" t="s">
+      <c r="H191" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I186" s="3" t="s">
+      <c r="I191" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A187" s="3"/>
-      <c r="B187" s="4" t="s">
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="3"/>
+      <c r="B192" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C187" s="4" t="s">
+      <c r="C192" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D187" s="3"/>
-      <c r="E187" s="4" t="s">
+      <c r="D192" s="3"/>
+      <c r="E192" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F187" s="3"/>
-      <c r="G187" s="4" t="s">
+      <c r="F192" s="3"/>
+      <c r="G192" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H187" s="4" t="s">
+      <c r="H192" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I187" s="3"/>
-    </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A188" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="B188" s="5"/>
-      <c r="C188" s="5"/>
-      <c r="D188" s="5"/>
-      <c r="E188" s="5"/>
-      <c r="F188" s="5"/>
-      <c r="G188" s="5"/>
-      <c r="H188" s="5"/>
-      <c r="I188" s="5"/>
-    </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A189" s="12" t="s">
-        <v>341</v>
-      </c>
-      <c r="B189" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C189" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D189" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E189" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F189" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G189" s="12" t="n">
-        <v>20001</v>
-      </c>
-      <c r="H189" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I189" s="12" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A190" s="12" t="s">
-        <v>344</v>
-      </c>
-      <c r="B190" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C190" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D190" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E190" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F190" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G190" s="12" t="n">
-        <v>20002</v>
-      </c>
-      <c r="H190" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I190" s="12" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A191" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="B191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C191" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E191" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F191" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G191" s="12" t="n">
-        <v>20003</v>
-      </c>
-      <c r="H191" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I191" s="12" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A192" s="12" t="s">
-        <v>346</v>
-      </c>
-      <c r="B192" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C192" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D192" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E192" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F192" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G192" s="12" t="n">
-        <v>20004</v>
-      </c>
-      <c r="H192" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I192" s="12" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A193" s="12" t="s">
-        <v>347</v>
-      </c>
-      <c r="B193" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C193" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D193" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E193" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F193" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G193" s="12" t="n">
-        <v>20005</v>
-      </c>
-      <c r="H193" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I193" s="12" t="s">
-        <v>343</v>
-      </c>
+      <c r="I192" s="3"/>
+    </row>
+    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A193" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="B193" s="5"/>
+      <c r="C193" s="5"/>
+      <c r="D193" s="5"/>
+      <c r="E193" s="5"/>
+      <c r="F193" s="5"/>
+      <c r="G193" s="5"/>
+      <c r="H193" s="5"/>
+      <c r="I193" s="5"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="12" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B194" s="12" t="s">
         <v>75</v>
@@ -12436,21 +12453,21 @@
         <v>75</v>
       </c>
       <c r="F194" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G194" s="12" t="n">
-        <v>20006</v>
+        <v>20001</v>
       </c>
       <c r="H194" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I194" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="12" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B195" s="12" t="s">
         <v>75</v>
@@ -12465,21 +12482,21 @@
         <v>75</v>
       </c>
       <c r="F195" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G195" s="12" t="n">
-        <v>20007</v>
+        <v>20002</v>
       </c>
       <c r="H195" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I195" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="12" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="B196" s="12" t="s">
         <v>75</v>
@@ -12494,79 +12511,79 @@
         <v>75</v>
       </c>
       <c r="F196" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G196" s="12" t="n">
-        <v>20008</v>
+        <v>20003</v>
       </c>
       <c r="H196" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I196" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="12" t="s">
+        <v>355</v>
+      </c>
+      <c r="B197" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C197" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D197" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E197" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F197" s="12" t="s">
         <v>351</v>
       </c>
-      <c r="B197" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C197" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D197" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E197" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F197" s="12" t="s">
-        <v>342</v>
-      </c>
       <c r="G197" s="12" t="n">
-        <v>30001</v>
+        <v>20004</v>
       </c>
       <c r="H197" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I197" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="12" t="s">
+        <v>356</v>
+      </c>
+      <c r="B198" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C198" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D198" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E198" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F198" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G198" s="12" t="n">
+        <v>20005</v>
+      </c>
+      <c r="H198" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I198" s="12" t="s">
         <v>352</v>
-      </c>
-      <c r="B198" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C198" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D198" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E198" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F198" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G198" s="12" t="n">
-        <v>30002</v>
-      </c>
-      <c r="H198" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I198" s="12" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="12" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B199" s="12" t="s">
         <v>75</v>
@@ -12581,21 +12598,21 @@
         <v>75</v>
       </c>
       <c r="F199" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G199" s="12" t="n">
-        <v>30003</v>
+        <v>20006</v>
       </c>
       <c r="H199" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I199" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="12" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="B200" s="12" t="s">
         <v>75</v>
@@ -12610,21 +12627,21 @@
         <v>75</v>
       </c>
       <c r="F200" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G200" s="12" t="n">
-        <v>30004</v>
+        <v>20007</v>
       </c>
       <c r="H200" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I200" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="12" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="B201" s="12" t="s">
         <v>75</v>
@@ -12639,21 +12656,21 @@
         <v>75</v>
       </c>
       <c r="F201" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G201" s="12" t="n">
-        <v>30005</v>
+        <v>20008</v>
       </c>
       <c r="H201" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I201" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="12" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B202" s="12" t="s">
         <v>75</v>
@@ -12668,21 +12685,21 @@
         <v>75</v>
       </c>
       <c r="F202" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G202" s="12" t="n">
-        <v>30006</v>
+        <v>30001</v>
       </c>
       <c r="H202" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I202" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="12" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B203" s="12" t="s">
         <v>75</v>
@@ -12697,21 +12714,21 @@
         <v>75</v>
       </c>
       <c r="F203" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G203" s="12" t="n">
-        <v>40001</v>
+        <v>30002</v>
       </c>
       <c r="H203" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I203" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="12" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B204" s="12" t="s">
         <v>75</v>
@@ -12726,21 +12743,21 @@
         <v>75</v>
       </c>
       <c r="F204" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G204" s="12" t="n">
-        <v>60001</v>
+        <v>30003</v>
       </c>
       <c r="H204" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I204" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="12" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="B205" s="12" t="s">
         <v>75</v>
@@ -12755,21 +12772,21 @@
         <v>75</v>
       </c>
       <c r="F205" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G205" s="12" t="n">
-        <v>60002</v>
+        <v>30004</v>
       </c>
       <c r="H205" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I205" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="12" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="B206" s="12" t="s">
         <v>75</v>
@@ -12784,21 +12801,21 @@
         <v>75</v>
       </c>
       <c r="F206" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G206" s="12" t="n">
-        <v>60003</v>
+        <v>30005</v>
       </c>
       <c r="H206" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I206" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="12" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B207" s="12" t="s">
         <v>75</v>
@@ -12813,21 +12830,21 @@
         <v>75</v>
       </c>
       <c r="F207" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G207" s="12" t="n">
-        <v>60004</v>
+        <v>30006</v>
       </c>
       <c r="H207" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I207" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="B208" s="12" t="s">
         <v>75</v>
@@ -12842,21 +12859,21 @@
         <v>75</v>
       </c>
       <c r="F208" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G208" s="12" t="n">
-        <v>60005</v>
+        <v>40001</v>
       </c>
       <c r="H208" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I208" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="B209" s="12" t="s">
         <v>75</v>
@@ -12871,21 +12888,21 @@
         <v>75</v>
       </c>
       <c r="F209" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G209" s="12" t="n">
-        <v>60006</v>
+        <v>60001</v>
       </c>
       <c r="H209" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I209" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B210" s="12" t="s">
         <v>75</v>
@@ -12900,21 +12917,21 @@
         <v>75</v>
       </c>
       <c r="F210" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G210" s="12" t="n">
-        <v>60007</v>
+        <v>60002</v>
       </c>
       <c r="H210" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B211" s="12" t="s">
         <v>75</v>
@@ -12929,229 +12946,229 @@
         <v>75</v>
       </c>
       <c r="F211" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G211" s="12" t="n">
+        <v>60003</v>
+      </c>
+      <c r="H211" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I211" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A212" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="B212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C212" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E212" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F212" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G212" s="12" t="n">
+        <v>60004</v>
+      </c>
+      <c r="H212" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I212" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A213" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="B213" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C213" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D213" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E213" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F213" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G213" s="12" t="n">
+        <v>60005</v>
+      </c>
+      <c r="H213" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I213" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="B214" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C214" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D214" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E214" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F214" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G214" s="12" t="n">
+        <v>60006</v>
+      </c>
+      <c r="H214" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I214" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="B215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C215" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E215" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F215" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G215" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H215" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I215" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C216" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F216" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G216" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H211" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I211" s="12" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A212" s="3" t="s">
+      <c r="H216" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I216" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A217" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B212" s="4" t="s">
+      <c r="B217" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C212" s="4" t="s">
+      <c r="C217" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D212" s="3" t="s">
+      <c r="D217" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E212" s="4" t="s">
+      <c r="E217" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F212" s="3" t="s">
+      <c r="F217" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G212" s="4" t="s">
+      <c r="G217" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H212" s="4" t="s">
+      <c r="H217" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I212" s="3" t="s">
+      <c r="I217" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A213" s="3"/>
-      <c r="B213" s="4" t="s">
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="3"/>
+      <c r="B218" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C213" s="4" t="s">
+      <c r="C218" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D213" s="3"/>
-      <c r="E213" s="4" t="s">
+      <c r="D218" s="3"/>
+      <c r="E218" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F213" s="3"/>
-      <c r="G213" s="4" t="s">
+      <c r="F218" s="3"/>
+      <c r="G218" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H213" s="4" t="s">
+      <c r="H218" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I213" s="3"/>
-    </row>
-    <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A214" s="5" t="s">
-        <v>366</v>
-      </c>
-      <c r="B214" s="5"/>
-      <c r="C214" s="5"/>
-      <c r="D214" s="5"/>
-      <c r="E214" s="5"/>
-      <c r="F214" s="5"/>
-      <c r="G214" s="5"/>
-      <c r="H214" s="5"/>
-      <c r="I214" s="5"/>
-    </row>
-    <row r="215" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A215" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="B215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C215" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F215" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G215" s="12" t="n">
-        <v>30001</v>
-      </c>
-      <c r="H215" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I215" s="12" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="216" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A216" s="12" t="s">
-        <v>352</v>
-      </c>
-      <c r="B216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C216" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F216" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G216" s="12" t="n">
-        <v>30002</v>
-      </c>
-      <c r="H216" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I216" s="12" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="217" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A217" s="12" t="s">
-        <v>353</v>
-      </c>
-      <c r="B217" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C217" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D217" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E217" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F217" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G217" s="12" t="n">
-        <v>30003</v>
-      </c>
-      <c r="H217" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I217" s="12" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="218" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A218" s="12" t="s">
-        <v>354</v>
-      </c>
-      <c r="B218" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C218" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D218" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E218" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F218" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G218" s="12" t="n">
-        <v>30004</v>
-      </c>
-      <c r="H218" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I218" s="12" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="219" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A219" s="12" t="s">
-        <v>355</v>
-      </c>
-      <c r="B219" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C219" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D219" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E219" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F219" s="12" t="s">
-        <v>342</v>
-      </c>
-      <c r="G219" s="12" t="n">
-        <v>30005</v>
-      </c>
-      <c r="H219" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I219" s="12" t="s">
-        <v>367</v>
-      </c>
+      <c r="I218" s="3"/>
+    </row>
+    <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A219" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="B219" s="5"/>
+      <c r="C219" s="5"/>
+      <c r="D219" s="5"/>
+      <c r="E219" s="5"/>
+      <c r="F219" s="5"/>
+      <c r="G219" s="5"/>
+      <c r="H219" s="5"/>
+      <c r="I219" s="5"/>
     </row>
     <row r="220" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="12" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="B220" s="12" t="s">
         <v>75</v>
@@ -13166,21 +13183,21 @@
         <v>75</v>
       </c>
       <c r="F220" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G220" s="12" t="n">
-        <v>30006</v>
+        <v>30001</v>
       </c>
       <c r="H220" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I220" s="12" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="12" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B221" s="12" t="s">
         <v>75</v>
@@ -13195,21 +13212,21 @@
         <v>75</v>
       </c>
       <c r="F221" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G221" s="12" t="n">
-        <v>40001</v>
+        <v>30002</v>
       </c>
       <c r="H221" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I221" s="12" t="s">
-        <v>343</v>
+        <v>376</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="12" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="B222" s="12" t="s">
         <v>75</v>
@@ -13224,21 +13241,21 @@
         <v>75</v>
       </c>
       <c r="F222" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G222" s="12" t="n">
-        <v>45001</v>
+        <v>30003</v>
       </c>
       <c r="H222" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I222" s="12" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="12" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B223" s="12" t="s">
         <v>75</v>
@@ -13253,21 +13270,21 @@
         <v>75</v>
       </c>
       <c r="F223" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G223" s="12" t="n">
-        <v>60001</v>
+        <v>30004</v>
       </c>
       <c r="H223" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I223" s="12" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="12" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B224" s="12" t="s">
         <v>75</v>
@@ -13282,21 +13299,21 @@
         <v>75</v>
       </c>
       <c r="F224" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G224" s="12" t="n">
-        <v>60002</v>
+        <v>30005</v>
       </c>
       <c r="H224" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I224" s="12" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="12" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="B225" s="12" t="s">
         <v>75</v>
@@ -13311,21 +13328,21 @@
         <v>75</v>
       </c>
       <c r="F225" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G225" s="12" t="n">
-        <v>60003</v>
+        <v>30006</v>
       </c>
       <c r="H225" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I225" s="12" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="226" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="12" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B226" s="12" t="s">
         <v>75</v>
@@ -13340,21 +13357,21 @@
         <v>75</v>
       </c>
       <c r="F226" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G226" s="12" t="n">
-        <v>60004</v>
+        <v>40001</v>
       </c>
       <c r="H226" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I226" s="12" t="s">
-        <v>367</v>
+        <v>352</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="12" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="B227" s="12" t="s">
         <v>75</v>
@@ -13369,21 +13386,21 @@
         <v>75</v>
       </c>
       <c r="F227" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G227" s="12" t="n">
-        <v>60005</v>
+        <v>45001</v>
       </c>
       <c r="H227" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I227" s="12" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="12" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="B228" s="12" t="s">
         <v>75</v>
@@ -13398,21 +13415,21 @@
         <v>75</v>
       </c>
       <c r="F228" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G228" s="12" t="n">
-        <v>60006</v>
+        <v>60001</v>
       </c>
       <c r="H228" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I228" s="12" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="12" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B229" s="12" t="s">
         <v>75</v>
@@ -13427,21 +13444,21 @@
         <v>75</v>
       </c>
       <c r="F229" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G229" s="12" t="n">
-        <v>60007</v>
+        <v>60002</v>
       </c>
       <c r="H229" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I229" s="12" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="12" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="B230" s="12" t="s">
         <v>75</v>
@@ -13456,226 +13473,232 @@
         <v>75</v>
       </c>
       <c r="F230" s="12" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="G230" s="12" t="n">
+        <v>60003</v>
+      </c>
+      <c r="H230" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I230" s="12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="B231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C231" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E231" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F231" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G231" s="12" t="n">
+        <v>60004</v>
+      </c>
+      <c r="H231" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I231" s="12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="B232" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C232" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D232" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E232" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F232" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G232" s="12" t="n">
+        <v>60005</v>
+      </c>
+      <c r="H232" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I232" s="12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="B233" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C233" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D233" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E233" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F233" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G233" s="12" t="n">
+        <v>60006</v>
+      </c>
+      <c r="H233" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I233" s="12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="234" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="B234" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C234" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D234" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E234" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F234" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G234" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H234" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I234" s="12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B235" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C235" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D235" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E235" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F235" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G235" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H230" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I230" s="12" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A231" s="3" t="s">
+      <c r="H235" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I235" s="12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A236" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B231" s="4" t="s">
+      <c r="B236" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C231" s="4" t="s">
+      <c r="C236" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D231" s="3" t="s">
+      <c r="D236" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E231" s="4" t="s">
+      <c r="E236" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F231" s="3" t="s">
+      <c r="F236" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G231" s="4" t="s">
+      <c r="G236" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H231" s="4" t="s">
+      <c r="H236" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I231" s="3" t="s">
+      <c r="I236" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A232" s="3"/>
-      <c r="B232" s="4" t="s">
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="3"/>
+      <c r="B237" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C232" s="4" t="s">
+      <c r="C237" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D232" s="3"/>
-      <c r="E232" s="4" t="s">
+      <c r="D237" s="3"/>
+      <c r="E237" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F232" s="3"/>
-      <c r="G232" s="4" t="s">
+      <c r="F237" s="3"/>
+      <c r="G237" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H232" s="4" t="s">
+      <c r="H237" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I232" s="3"/>
-    </row>
-    <row r="233" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A233" s="5" t="s">
+      <c r="I237" s="3"/>
+    </row>
+    <row r="238" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A238" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="B233" s="5"/>
-      <c r="C233" s="5"/>
-      <c r="D233" s="5"/>
-      <c r="E233" s="5"/>
-      <c r="F233" s="5"/>
-      <c r="G233" s="5"/>
-      <c r="H233" s="5"/>
-      <c r="I233" s="5"/>
-    </row>
-    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A234" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B234" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C234" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D234" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E234" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F234" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G234" s="10" t="s">
-        <v>318</v>
-      </c>
-      <c r="H234" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I234" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A235" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="B235" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C235" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D235" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E235" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F235" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G235" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="H235" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I235" s="7" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A236" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="B236" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C236" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D236" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E236" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F236" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G236" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="H236" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I236" s="7"/>
-    </row>
-    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A237" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="B237" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C237" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D237" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E237" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F237" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G237" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="H237" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I237" s="7"/>
-    </row>
-    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A238" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="B238" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C238" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D238" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E238" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F238" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G238" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="H238" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I238" s="7"/>
+      <c r="B238" s="5"/>
+      <c r="C238" s="5"/>
+      <c r="D238" s="5"/>
+      <c r="E238" s="5"/>
+      <c r="F238" s="5"/>
+      <c r="G238" s="5"/>
+      <c r="H238" s="5"/>
+      <c r="I238" s="5"/>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="9" t="s">
-        <v>203</v>
+        <v>108</v>
       </c>
       <c r="B239" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C239" s="7" t="s">
         <v>110</v>
@@ -13690,16 +13713,18 @@
         <v>26</v>
       </c>
       <c r="G239" s="10" t="s">
-        <v>204</v>
+        <v>318</v>
       </c>
       <c r="H239" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I239" s="7"/>
+      <c r="I239" s="7" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="9" t="s">
-        <v>205</v>
+        <v>187</v>
       </c>
       <c r="B240" s="7" t="s">
         <v>109</v>
@@ -13717,19 +13742,21 @@
         <v>26</v>
       </c>
       <c r="G240" s="10" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="H240" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I240" s="7"/>
+      <c r="I240" s="7" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="9" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="B241" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C241" s="7" t="s">
         <v>110</v>
@@ -13744,7 +13771,7 @@
         <v>26</v>
       </c>
       <c r="G241" s="10" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="H241" s="7" t="n">
         <v>2</v>
@@ -13753,7 +13780,7 @@
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="9" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="B242" s="7" t="s">
         <v>24</v>
@@ -13771,7 +13798,7 @@
         <v>26</v>
       </c>
       <c r="G242" s="10" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="H242" s="7" t="n">
         <v>2</v>
@@ -13780,7 +13807,7 @@
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="9" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="B243" s="7" t="s">
         <v>24</v>
@@ -13798,7 +13825,7 @@
         <v>26</v>
       </c>
       <c r="G243" s="10" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="H243" s="7" t="n">
         <v>2</v>
@@ -13807,7 +13834,7 @@
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="9" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="B244" s="7" t="s">
         <v>24</v>
@@ -13825,7 +13852,7 @@
         <v>26</v>
       </c>
       <c r="G244" s="10" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="H244" s="7" t="n">
         <v>2</v>
@@ -13834,10 +13861,10 @@
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="9" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="B245" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C245" s="7" t="s">
         <v>110</v>
@@ -13852,7 +13879,7 @@
         <v>26</v>
       </c>
       <c r="G245" s="10" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="H245" s="7" t="n">
         <v>2</v>
@@ -13861,7 +13888,7 @@
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="9" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="B246" s="7" t="s">
         <v>109</v>
@@ -13879,7 +13906,7 @@
         <v>26</v>
       </c>
       <c r="G246" s="10" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="H246" s="7" t="n">
         <v>2</v>
@@ -13888,10 +13915,10 @@
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="9" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="B247" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C247" s="7" t="s">
         <v>110</v>
@@ -13906,7 +13933,7 @@
         <v>26</v>
       </c>
       <c r="G247" s="10" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="H247" s="7" t="n">
         <v>2</v>
@@ -13915,10 +13942,10 @@
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="9" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="B248" s="7" t="s">
-        <v>222</v>
+        <v>24</v>
       </c>
       <c r="C248" s="7" t="s">
         <v>110</v>
@@ -13933,7 +13960,7 @@
         <v>26</v>
       </c>
       <c r="G248" s="10" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="H248" s="7" t="n">
         <v>2</v>
@@ -13942,10 +13969,10 @@
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="9" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="B249" s="7" t="s">
-        <v>222</v>
+        <v>24</v>
       </c>
       <c r="C249" s="7" t="s">
         <v>110</v>
@@ -13960,7 +13987,7 @@
         <v>26</v>
       </c>
       <c r="G249" s="10" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="H249" s="7" t="n">
         <v>2</v>
@@ -13969,10 +13996,10 @@
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="9" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="B250" s="7" t="s">
-        <v>195</v>
+        <v>24</v>
       </c>
       <c r="C250" s="7" t="s">
         <v>110</v>
@@ -13987,7 +14014,7 @@
         <v>26</v>
       </c>
       <c r="G250" s="10" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="H250" s="7" t="n">
         <v>2</v>
@@ -13996,10 +14023,10 @@
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="9" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="B251" s="7" t="s">
-        <v>195</v>
+        <v>109</v>
       </c>
       <c r="C251" s="7" t="s">
         <v>110</v>
@@ -14014,7 +14041,7 @@
         <v>26</v>
       </c>
       <c r="G251" s="10" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="H251" s="7" t="n">
         <v>2</v>
@@ -14023,7 +14050,7 @@
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="9" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="B252" s="7" t="s">
         <v>109</v>
@@ -14041,7 +14068,7 @@
         <v>26</v>
       </c>
       <c r="G252" s="10" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="H252" s="7" t="n">
         <v>2</v>
@@ -14050,10 +14077,10 @@
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="9" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="B253" s="7" t="s">
-        <v>109</v>
+        <v>222</v>
       </c>
       <c r="C253" s="7" t="s">
         <v>110</v>
@@ -14068,7 +14095,7 @@
         <v>26</v>
       </c>
       <c r="G253" s="10" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="H253" s="7" t="n">
         <v>2</v>
@@ -14076,11 +14103,11 @@
       <c r="I253" s="7"/>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A254" s="7" t="s">
-        <v>234</v>
+      <c r="A254" s="9" t="s">
+        <v>224</v>
       </c>
       <c r="B254" s="7" t="s">
-        <v>75</v>
+        <v>222</v>
       </c>
       <c r="C254" s="7" t="s">
         <v>110</v>
@@ -14095,21 +14122,19 @@
         <v>26</v>
       </c>
       <c r="G254" s="10" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="H254" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I254" s="7" t="s">
-        <v>320</v>
-      </c>
+      <c r="I254" s="7"/>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A255" s="7" t="s">
-        <v>237</v>
+      <c r="A255" s="9" t="s">
+        <v>226</v>
       </c>
       <c r="B255" s="7" t="s">
-        <v>75</v>
+        <v>195</v>
       </c>
       <c r="C255" s="7" t="s">
         <v>110</v>
@@ -14124,161 +14149,297 @@
         <v>26</v>
       </c>
       <c r="G255" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="H255" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I255" s="7"/>
+    </row>
+    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A256" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="B256" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C256" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D256" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E256" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F256" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G256" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="H256" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I256" s="7"/>
+    </row>
+    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A257" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B257" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C257" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D257" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E257" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F257" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G257" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H257" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I257" s="7"/>
+    </row>
+    <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A258" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B258" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C258" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D258" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E258" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F258" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G258" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="H258" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I258" s="7"/>
+    </row>
+    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A259" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="B259" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C259" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D259" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E259" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F259" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G259" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="H259" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I259" s="7" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A260" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B260" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C260" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D260" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E260" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F260" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G260" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="H255" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I255" s="7" t="s">
+      <c r="H260" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I260" s="7" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="256" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A256" s="12" t="s">
+    <row r="261" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A261" s="12" t="s">
         <v>239</v>
       </c>
-      <c r="B256" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C256" s="12" t="s">
+      <c r="B261" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C261" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D256" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E256" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F256" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G256" s="12" t="s">
+      <c r="D261" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E261" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F261" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G261" s="12" t="s">
         <v>240</v>
       </c>
-      <c r="H256" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I256" s="12" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="257" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A257" s="12" t="s">
+      <c r="H261" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I261" s="12" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="262" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A262" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="B257" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C257" s="12" t="s">
+      <c r="B262" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C262" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D257" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E257" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F257" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G257" s="12" t="s">
+      <c r="D262" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E262" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F262" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G262" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="H257" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I257" s="12" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="258" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A258" s="11" t="s">
+      <c r="H262" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I262" s="12" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="263" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A263" s="11" t="s">
         <v>325</v>
       </c>
-      <c r="B258" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C258" s="12" t="s">
+      <c r="B263" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C263" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D258" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E258" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F258" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G258" s="13" t="s">
+      <c r="D263" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E263" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F263" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G263" s="13" t="s">
         <v>326</v>
       </c>
-      <c r="H258" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I258" s="12" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="259" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A259" s="11" t="s">
+      <c r="H263" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I263" s="12" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="264" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A264" s="11" t="s">
         <v>328</v>
       </c>
-      <c r="B259" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C259" s="12" t="s">
+      <c r="B264" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C264" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D259" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E259" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F259" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G259" s="13" t="s">
+      <c r="D264" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E264" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F264" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G264" s="13" t="s">
         <v>329</v>
       </c>
-      <c r="H259" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I259" s="12" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="260" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A260" s="11" t="s">
-        <v>373</v>
-      </c>
-      <c r="B260" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C260" s="12" t="s">
+      <c r="H264" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I264" s="12" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="265" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A265" s="11" t="s">
+        <v>382</v>
+      </c>
+      <c r="B265" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C265" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D260" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E260" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F260" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G260" s="13" t="s">
+      <c r="D265" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E265" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F265" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G265" s="13" t="s">
         <v>332</v>
       </c>
-      <c r="H260" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I260" s="12" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="H265" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I265" s="12" t="s">
+        <v>383</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="25">
     <mergeCell ref="A6:A7"/>
@@ -14291,21 +14452,21 @@
     <mergeCell ref="F115:F116"/>
     <mergeCell ref="I115:I116"/>
     <mergeCell ref="A117:I117"/>
-    <mergeCell ref="A186:A187"/>
-    <mergeCell ref="D186:D187"/>
-    <mergeCell ref="F186:F187"/>
-    <mergeCell ref="I186:I187"/>
-    <mergeCell ref="A188:I188"/>
-    <mergeCell ref="A212:A213"/>
-    <mergeCell ref="D212:D213"/>
-    <mergeCell ref="F212:F213"/>
-    <mergeCell ref="I212:I213"/>
-    <mergeCell ref="A214:I214"/>
-    <mergeCell ref="A231:A232"/>
-    <mergeCell ref="D231:D232"/>
-    <mergeCell ref="F231:F232"/>
-    <mergeCell ref="I231:I232"/>
-    <mergeCell ref="A233:I233"/>
+    <mergeCell ref="A191:A192"/>
+    <mergeCell ref="D191:D192"/>
+    <mergeCell ref="F191:F192"/>
+    <mergeCell ref="I191:I192"/>
+    <mergeCell ref="A193:I193"/>
+    <mergeCell ref="A217:A218"/>
+    <mergeCell ref="D217:D218"/>
+    <mergeCell ref="F217:F218"/>
+    <mergeCell ref="I217:I218"/>
+    <mergeCell ref="A219:I219"/>
+    <mergeCell ref="A236:A237"/>
+    <mergeCell ref="D236:D237"/>
+    <mergeCell ref="F236:F237"/>
+    <mergeCell ref="I236:I237"/>
+    <mergeCell ref="A238:I238"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
SOCO: Bugfix: Fix address of contactors alarms as per modbus table
Alarams addresses didn't match the document we had sent to the customer.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2571" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2427" uniqueCount="384">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -7313,7 +7313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I265"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.94"/>
@@ -11160,7 +11160,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="7" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
       <c r="B146" s="7" t="s">
         <v>75</v>
@@ -11178,7 +11178,7 @@
         <v>248</v>
       </c>
       <c r="G146" s="7" t="n">
-        <v>501</v>
+        <v>601</v>
       </c>
       <c r="H146" s="7" t="n">
         <v>1</v>
@@ -11187,7 +11187,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="7" t="s">
-        <v>278</v>
+        <v>295</v>
       </c>
       <c r="B147" s="7" t="s">
         <v>75</v>
@@ -11205,7 +11205,7 @@
         <v>248</v>
       </c>
       <c r="G147" s="7" t="n">
-        <v>502</v>
+        <v>602</v>
       </c>
       <c r="H147" s="7" t="n">
         <v>1</v>
@@ -11214,7 +11214,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="7" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="B148" s="7" t="s">
         <v>75</v>
@@ -11232,7 +11232,7 @@
         <v>248</v>
       </c>
       <c r="G148" s="7" t="n">
-        <v>503</v>
+        <v>603</v>
       </c>
       <c r="H148" s="7" t="n">
         <v>1</v>
@@ -11241,7 +11241,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="7" t="s">
-        <v>280</v>
+        <v>296</v>
       </c>
       <c r="B149" s="7" t="s">
         <v>75</v>
@@ -11259,7 +11259,7 @@
         <v>248</v>
       </c>
       <c r="G149" s="7" t="n">
-        <v>504</v>
+        <v>604</v>
       </c>
       <c r="H149" s="7" t="n">
         <v>1</v>
@@ -11268,7 +11268,7 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="7" t="s">
-        <v>281</v>
+        <v>291</v>
       </c>
       <c r="B150" s="7" t="s">
         <v>75</v>
@@ -11286,7 +11286,7 @@
         <v>248</v>
       </c>
       <c r="G150" s="7" t="n">
-        <v>505</v>
+        <v>605</v>
       </c>
       <c r="H150" s="7" t="n">
         <v>1</v>
@@ -11295,7 +11295,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="7" t="s">
-        <v>282</v>
+        <v>297</v>
       </c>
       <c r="B151" s="7" t="s">
         <v>75</v>
@@ -11313,7 +11313,7 @@
         <v>248</v>
       </c>
       <c r="G151" s="7" t="n">
-        <v>506</v>
+        <v>606</v>
       </c>
       <c r="H151" s="7" t="n">
         <v>1</v>
@@ -11322,7 +11322,7 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="7" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="B152" s="7" t="s">
         <v>75</v>
@@ -11340,7 +11340,7 @@
         <v>248</v>
       </c>
       <c r="G152" s="7" t="n">
-        <v>507</v>
+        <v>607</v>
       </c>
       <c r="H152" s="7" t="n">
         <v>1</v>
@@ -11349,7 +11349,7 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="7" t="s">
-        <v>284</v>
+        <v>298</v>
       </c>
       <c r="B153" s="7" t="s">
         <v>75</v>
@@ -11367,7 +11367,7 @@
         <v>248</v>
       </c>
       <c r="G153" s="7" t="n">
-        <v>508</v>
+        <v>608</v>
       </c>
       <c r="H153" s="7" t="n">
         <v>1</v>
@@ -11376,7 +11376,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="7" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="B154" s="7" t="s">
         <v>75</v>
@@ -11394,7 +11394,7 @@
         <v>248</v>
       </c>
       <c r="G154" s="7" t="n">
-        <v>509</v>
+        <v>609</v>
       </c>
       <c r="H154" s="7" t="n">
         <v>1</v>
@@ -11403,7 +11403,7 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="7" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="B155" s="7" t="s">
         <v>75</v>
@@ -11421,7 +11421,7 @@
         <v>248</v>
       </c>
       <c r="G155" s="7" t="n">
-        <v>510</v>
+        <v>610</v>
       </c>
       <c r="H155" s="7" t="n">
         <v>1</v>
@@ -11430,7 +11430,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="7" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="B156" s="7" t="s">
         <v>75</v>
@@ -11448,7 +11448,7 @@
         <v>248</v>
       </c>
       <c r="G156" s="7" t="n">
-        <v>511</v>
+        <v>611</v>
       </c>
       <c r="H156" s="7" t="n">
         <v>1</v>
@@ -11457,7 +11457,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="7" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="B157" s="7" t="s">
         <v>75</v>
@@ -11475,7 +11475,7 @@
         <v>248</v>
       </c>
       <c r="G157" s="7" t="n">
-        <v>512</v>
+        <v>612</v>
       </c>
       <c r="H157" s="7" t="n">
         <v>1</v>
@@ -11484,7 +11484,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
-        <v>289</v>
+        <v>340</v>
       </c>
       <c r="B158" s="7" t="s">
         <v>75</v>
@@ -11502,7 +11502,7 @@
         <v>248</v>
       </c>
       <c r="G158" s="7" t="n">
-        <v>601</v>
+        <v>801</v>
       </c>
       <c r="H158" s="7" t="n">
         <v>1</v>
@@ -11511,7 +11511,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="7" t="s">
-        <v>290</v>
+        <v>341</v>
       </c>
       <c r="B159" s="7" t="s">
         <v>75</v>
@@ -11529,7 +11529,7 @@
         <v>248</v>
       </c>
       <c r="G159" s="7" t="n">
-        <v>602</v>
+        <v>802</v>
       </c>
       <c r="H159" s="7" t="n">
         <v>1</v>
@@ -11538,7 +11538,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="7" t="s">
-        <v>291</v>
+        <v>342</v>
       </c>
       <c r="B160" s="7" t="s">
         <v>75</v>
@@ -11556,7 +11556,7 @@
         <v>248</v>
       </c>
       <c r="G160" s="7" t="n">
-        <v>603</v>
+        <v>803</v>
       </c>
       <c r="H160" s="7" t="n">
         <v>1</v>
@@ -11565,7 +11565,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="7" t="s">
-        <v>292</v>
+        <v>343</v>
       </c>
       <c r="B161" s="7" t="s">
         <v>75</v>
@@ -11583,7 +11583,7 @@
         <v>248</v>
       </c>
       <c r="G161" s="7" t="n">
-        <v>604</v>
+        <v>804</v>
       </c>
       <c r="H161" s="7" t="n">
         <v>1</v>
@@ -11592,7 +11592,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="7" t="s">
-        <v>293</v>
+        <v>344</v>
       </c>
       <c r="B162" s="7" t="s">
         <v>75</v>
@@ -11610,7 +11610,7 @@
         <v>248</v>
       </c>
       <c r="G162" s="7" t="n">
-        <v>605</v>
+        <v>805</v>
       </c>
       <c r="H162" s="7" t="n">
         <v>1</v>
@@ -11619,7 +11619,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="7" t="s">
-        <v>294</v>
+        <v>345</v>
       </c>
       <c r="B163" s="7" t="s">
         <v>75</v>
@@ -11637,7 +11637,7 @@
         <v>248</v>
       </c>
       <c r="G163" s="7" t="n">
-        <v>606</v>
+        <v>806</v>
       </c>
       <c r="H163" s="7" t="n">
         <v>1</v>
@@ -11646,7 +11646,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="7" t="s">
-        <v>295</v>
+        <v>346</v>
       </c>
       <c r="B164" s="7" t="s">
         <v>75</v>
@@ -11664,7 +11664,7 @@
         <v>248</v>
       </c>
       <c r="G164" s="7" t="n">
-        <v>607</v>
+        <v>807</v>
       </c>
       <c r="H164" s="7" t="n">
         <v>1</v>
@@ -11673,7 +11673,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="7" t="s">
-        <v>296</v>
+        <v>347</v>
       </c>
       <c r="B165" s="7" t="s">
         <v>75</v>
@@ -11691,7 +11691,7 @@
         <v>248</v>
       </c>
       <c r="G165" s="7" t="n">
-        <v>608</v>
+        <v>808</v>
       </c>
       <c r="H165" s="7" t="n">
         <v>1</v>
@@ -11700,7 +11700,7 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="7" t="s">
-        <v>297</v>
+        <v>348</v>
       </c>
       <c r="B166" s="7" t="s">
         <v>75</v>
@@ -11718,785 +11718,809 @@
         <v>248</v>
       </c>
       <c r="G166" s="7" t="n">
-        <v>609</v>
+        <v>809</v>
       </c>
       <c r="H166" s="7" t="n">
         <v>1</v>
       </c>
       <c r="I166" s="7"/>
     </row>
-    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="7" t="s">
-        <v>298</v>
-      </c>
-      <c r="B167" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C167" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D167" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E167" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F167" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G167" s="7" t="n">
-        <v>610</v>
-      </c>
-      <c r="H167" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I167" s="7"/>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A167" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D167" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E167" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F167" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G167" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H167" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I167" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="7" t="s">
-        <v>299</v>
-      </c>
-      <c r="B168" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C168" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D168" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E168" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F168" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G168" s="7" t="n">
-        <v>611</v>
-      </c>
-      <c r="H168" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I168" s="7"/>
-    </row>
-    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A169" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="B169" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C169" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D169" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E169" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F169" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G169" s="7" t="n">
-        <v>612</v>
-      </c>
-      <c r="H169" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I169" s="7"/>
+      <c r="A168" s="3"/>
+      <c r="B168" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D168" s="3"/>
+      <c r="E168" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F168" s="3"/>
+      <c r="G168" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H168" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I168" s="3"/>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A169" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="B169" s="5"/>
+      <c r="C169" s="5"/>
+      <c r="D169" s="5"/>
+      <c r="E169" s="5"/>
+      <c r="F169" s="5"/>
+      <c r="G169" s="5"/>
+      <c r="H169" s="5"/>
+      <c r="I169" s="5"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A170" s="7" t="s">
-        <v>301</v>
-      </c>
-      <c r="B170" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C170" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D170" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E170" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F170" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G170" s="7" t="n">
-        <v>701</v>
-      </c>
-      <c r="H170" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I170" s="7"/>
+      <c r="A170" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="B170" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C170" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D170" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E170" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F170" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G170" s="12" t="n">
+        <v>20001</v>
+      </c>
+      <c r="H170" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I170" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A171" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="B171" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C171" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D171" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E171" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F171" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G171" s="7" t="n">
-        <v>702</v>
-      </c>
-      <c r="H171" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I171" s="7"/>
+      <c r="A171" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="B171" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C171" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D171" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E171" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F171" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G171" s="12" t="n">
+        <v>20002</v>
+      </c>
+      <c r="H171" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I171" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A172" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="B172" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C172" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D172" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E172" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F172" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G172" s="7" t="n">
-        <v>703</v>
-      </c>
-      <c r="H172" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I172" s="7"/>
+      <c r="A172" s="12" t="s">
+        <v>354</v>
+      </c>
+      <c r="B172" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C172" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D172" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E172" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F172" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G172" s="12" t="n">
+        <v>20003</v>
+      </c>
+      <c r="H172" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I172" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A173" s="7" t="s">
-        <v>304</v>
-      </c>
-      <c r="B173" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C173" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D173" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E173" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F173" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G173" s="7" t="n">
-        <v>704</v>
-      </c>
-      <c r="H173" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I173" s="7"/>
+      <c r="A173" s="12" t="s">
+        <v>355</v>
+      </c>
+      <c r="B173" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C173" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D173" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E173" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F173" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G173" s="12" t="n">
+        <v>20004</v>
+      </c>
+      <c r="H173" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I173" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A174" s="7" t="s">
-        <v>305</v>
-      </c>
-      <c r="B174" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C174" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D174" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E174" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F174" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G174" s="7" t="n">
-        <v>705</v>
-      </c>
-      <c r="H174" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I174" s="7"/>
+      <c r="A174" s="12" t="s">
+        <v>356</v>
+      </c>
+      <c r="B174" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C174" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D174" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E174" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F174" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G174" s="12" t="n">
+        <v>20005</v>
+      </c>
+      <c r="H174" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I174" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A175" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="B175" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C175" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D175" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E175" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F175" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G175" s="7" t="n">
-        <v>706</v>
-      </c>
-      <c r="H175" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I175" s="7"/>
+      <c r="A175" s="12" t="s">
+        <v>357</v>
+      </c>
+      <c r="B175" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C175" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D175" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E175" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F175" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G175" s="12" t="n">
+        <v>20006</v>
+      </c>
+      <c r="H175" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I175" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="B176" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C176" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D176" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E176" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F176" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G176" s="7" t="n">
-        <v>707</v>
-      </c>
-      <c r="H176" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I176" s="7"/>
+      <c r="A176" s="12" t="s">
+        <v>358</v>
+      </c>
+      <c r="B176" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C176" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D176" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E176" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F176" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G176" s="12" t="n">
+        <v>20007</v>
+      </c>
+      <c r="H176" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I176" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="7" t="s">
-        <v>308</v>
-      </c>
-      <c r="B177" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C177" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D177" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E177" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F177" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G177" s="7" t="n">
-        <v>708</v>
-      </c>
-      <c r="H177" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I177" s="7"/>
+      <c r="A177" s="12" t="s">
+        <v>359</v>
+      </c>
+      <c r="B177" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C177" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D177" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E177" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F177" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G177" s="12" t="n">
+        <v>20008</v>
+      </c>
+      <c r="H177" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I177" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="B178" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C178" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D178" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E178" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F178" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G178" s="7" t="n">
-        <v>709</v>
-      </c>
-      <c r="H178" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I178" s="7"/>
+      <c r="A178" s="12" t="s">
+        <v>360</v>
+      </c>
+      <c r="B178" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C178" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D178" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E178" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F178" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G178" s="12" t="n">
+        <v>30001</v>
+      </c>
+      <c r="H178" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I178" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="B179" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C179" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D179" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E179" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F179" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G179" s="7" t="n">
-        <v>710</v>
-      </c>
-      <c r="H179" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I179" s="7"/>
+      <c r="A179" s="12" t="s">
+        <v>361</v>
+      </c>
+      <c r="B179" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C179" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D179" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E179" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F179" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G179" s="12" t="n">
+        <v>30002</v>
+      </c>
+      <c r="H179" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I179" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A180" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="B180" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C180" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D180" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E180" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F180" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G180" s="7" t="n">
-        <v>711</v>
-      </c>
-      <c r="H180" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I180" s="7"/>
+      <c r="A180" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="B180" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C180" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D180" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E180" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F180" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G180" s="12" t="n">
+        <v>30003</v>
+      </c>
+      <c r="H180" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I180" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A181" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="B181" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C181" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D181" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E181" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F181" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G181" s="7" t="n">
-        <v>712</v>
-      </c>
-      <c r="H181" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I181" s="7"/>
+      <c r="A181" s="12" t="s">
+        <v>363</v>
+      </c>
+      <c r="B181" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C181" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D181" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E181" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F181" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G181" s="12" t="n">
+        <v>30004</v>
+      </c>
+      <c r="H181" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I181" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A182" s="7" t="s">
-        <v>340</v>
-      </c>
-      <c r="B182" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C182" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D182" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E182" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F182" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G182" s="7" t="n">
-        <v>801</v>
-      </c>
-      <c r="H182" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I182" s="7"/>
+      <c r="A182" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="B182" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C182" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D182" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E182" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F182" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G182" s="12" t="n">
+        <v>30005</v>
+      </c>
+      <c r="H182" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I182" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A183" s="7" t="s">
-        <v>341</v>
-      </c>
-      <c r="B183" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C183" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D183" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E183" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F183" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G183" s="7" t="n">
-        <v>802</v>
-      </c>
-      <c r="H183" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I183" s="7"/>
+      <c r="A183" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="B183" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C183" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D183" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E183" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F183" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G183" s="12" t="n">
+        <v>30006</v>
+      </c>
+      <c r="H183" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I183" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A184" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="B184" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C184" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D184" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E184" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F184" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G184" s="7" t="n">
-        <v>803</v>
-      </c>
-      <c r="H184" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I184" s="7"/>
+      <c r="A184" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="B184" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C184" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D184" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E184" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F184" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G184" s="12" t="n">
+        <v>40001</v>
+      </c>
+      <c r="H184" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I184" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A185" s="7" t="s">
-        <v>343</v>
-      </c>
-      <c r="B185" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C185" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D185" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E185" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F185" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G185" s="7" t="n">
-        <v>804</v>
-      </c>
-      <c r="H185" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I185" s="7"/>
+      <c r="A185" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="B185" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C185" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D185" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E185" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F185" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G185" s="12" t="n">
+        <v>60001</v>
+      </c>
+      <c r="H185" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I185" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A186" s="7" t="s">
-        <v>344</v>
-      </c>
-      <c r="B186" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C186" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D186" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E186" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F186" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G186" s="7" t="n">
-        <v>805</v>
-      </c>
-      <c r="H186" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I186" s="7"/>
+      <c r="A186" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="B186" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C186" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D186" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E186" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F186" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G186" s="12" t="n">
+        <v>60002</v>
+      </c>
+      <c r="H186" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I186" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A187" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="B187" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C187" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D187" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E187" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F187" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G187" s="7" t="n">
-        <v>806</v>
-      </c>
-      <c r="H187" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I187" s="7"/>
+      <c r="A187" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="B187" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C187" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D187" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E187" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F187" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G187" s="12" t="n">
+        <v>60003</v>
+      </c>
+      <c r="H187" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I187" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A188" s="7" t="s">
-        <v>346</v>
-      </c>
-      <c r="B188" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C188" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D188" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E188" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F188" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G188" s="7" t="n">
-        <v>807</v>
-      </c>
-      <c r="H188" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I188" s="7"/>
+      <c r="A188" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="B188" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C188" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D188" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E188" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F188" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G188" s="12" t="n">
+        <v>60004</v>
+      </c>
+      <c r="H188" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I188" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A189" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="B189" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C189" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D189" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E189" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F189" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G189" s="7" t="n">
-        <v>808</v>
-      </c>
-      <c r="H189" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I189" s="7"/>
+      <c r="A189" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="B189" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C189" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D189" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E189" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F189" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G189" s="12" t="n">
+        <v>60005</v>
+      </c>
+      <c r="H189" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I189" s="12" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A190" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="B190" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C190" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="D190" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E190" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F190" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="G190" s="7" t="n">
-        <v>809</v>
-      </c>
-      <c r="H190" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I190" s="7"/>
-    </row>
-    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A191" s="3" t="s">
+      <c r="A190" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="B190" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C190" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D190" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E190" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F190" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G190" s="12" t="n">
+        <v>60006</v>
+      </c>
+      <c r="H190" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I190" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A191" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="B191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C191" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E191" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F191" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G191" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H191" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I191" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A192" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B192" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C192" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D192" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E192" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F192" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="G192" s="12" t="n">
+        <v>60008</v>
+      </c>
+      <c r="H192" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I192" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A193" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B191" s="4" t="s">
+      <c r="B193" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C191" s="4" t="s">
+      <c r="C193" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D191" s="3" t="s">
+      <c r="D193" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E191" s="4" t="s">
+      <c r="E193" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F191" s="3" t="s">
+      <c r="F193" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G191" s="4" t="s">
+      <c r="G193" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H191" s="4" t="s">
+      <c r="H193" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I191" s="3" t="s">
+      <c r="I193" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A192" s="3"/>
-      <c r="B192" s="4" t="s">
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A194" s="3"/>
+      <c r="B194" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C192" s="4" t="s">
+      <c r="C194" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D192" s="3"/>
-      <c r="E192" s="4" t="s">
+      <c r="D194" s="3"/>
+      <c r="E194" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F192" s="3"/>
-      <c r="G192" s="4" t="s">
+      <c r="F194" s="3"/>
+      <c r="G194" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H192" s="4" t="s">
+      <c r="H194" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I192" s="3"/>
-    </row>
-    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A193" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="B193" s="5"/>
-      <c r="C193" s="5"/>
-      <c r="D193" s="5"/>
-      <c r="E193" s="5"/>
-      <c r="F193" s="5"/>
-      <c r="G193" s="5"/>
-      <c r="H193" s="5"/>
-      <c r="I193" s="5"/>
-    </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A194" s="12" t="s">
-        <v>350</v>
-      </c>
-      <c r="B194" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C194" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D194" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E194" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F194" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G194" s="12" t="n">
-        <v>20001</v>
-      </c>
-      <c r="H194" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I194" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A195" s="12" t="s">
-        <v>353</v>
-      </c>
-      <c r="B195" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C195" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D195" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E195" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F195" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G195" s="12" t="n">
-        <v>20002</v>
-      </c>
-      <c r="H195" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I195" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I194" s="3"/>
+    </row>
+    <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A195" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="B195" s="5"/>
+      <c r="C195" s="5"/>
+      <c r="D195" s="5"/>
+      <c r="E195" s="5"/>
+      <c r="F195" s="5"/>
+      <c r="G195" s="5"/>
+      <c r="H195" s="5"/>
+      <c r="I195" s="5"/>
+    </row>
+    <row r="196" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="12" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="B196" s="12" t="s">
         <v>75</v>
@@ -12514,18 +12538,18 @@
         <v>351</v>
       </c>
       <c r="G196" s="12" t="n">
-        <v>20003</v>
+        <v>30001</v>
       </c>
       <c r="H196" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I196" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="12" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="B197" s="12" t="s">
         <v>75</v>
@@ -12543,18 +12567,18 @@
         <v>351</v>
       </c>
       <c r="G197" s="12" t="n">
-        <v>20004</v>
+        <v>30002</v>
       </c>
       <c r="H197" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I197" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="12" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="B198" s="12" t="s">
         <v>75</v>
@@ -12572,18 +12596,18 @@
         <v>351</v>
       </c>
       <c r="G198" s="12" t="n">
-        <v>20005</v>
+        <v>30003</v>
       </c>
       <c r="H198" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I198" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="12" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="B199" s="12" t="s">
         <v>75</v>
@@ -12601,18 +12625,18 @@
         <v>351</v>
       </c>
       <c r="G199" s="12" t="n">
-        <v>20006</v>
+        <v>30004</v>
       </c>
       <c r="H199" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I199" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="12" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="B200" s="12" t="s">
         <v>75</v>
@@ -12630,18 +12654,18 @@
         <v>351</v>
       </c>
       <c r="G200" s="12" t="n">
-        <v>20007</v>
+        <v>30005</v>
       </c>
       <c r="H200" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I200" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="12" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B201" s="12" t="s">
         <v>75</v>
@@ -12659,18 +12683,18 @@
         <v>351</v>
       </c>
       <c r="G201" s="12" t="n">
-        <v>20008</v>
+        <v>30006</v>
       </c>
       <c r="H201" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I201" s="12" t="s">
-        <v>352</v>
+        <v>376</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="12" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="B202" s="12" t="s">
         <v>75</v>
@@ -12688,7 +12712,7 @@
         <v>351</v>
       </c>
       <c r="G202" s="12" t="n">
-        <v>30001</v>
+        <v>40001</v>
       </c>
       <c r="H202" s="12" t="n">
         <v>1</v>
@@ -12697,9 +12721,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="12" t="s">
-        <v>361</v>
+        <v>377</v>
       </c>
       <c r="B203" s="12" t="s">
         <v>75</v>
@@ -12717,18 +12741,18 @@
         <v>351</v>
       </c>
       <c r="G203" s="12" t="n">
-        <v>30002</v>
+        <v>45001</v>
       </c>
       <c r="H203" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I203" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="12" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="B204" s="12" t="s">
         <v>75</v>
@@ -12746,18 +12770,18 @@
         <v>351</v>
       </c>
       <c r="G204" s="12" t="n">
-        <v>30003</v>
+        <v>60001</v>
       </c>
       <c r="H204" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I204" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="12" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="B205" s="12" t="s">
         <v>75</v>
@@ -12775,18 +12799,18 @@
         <v>351</v>
       </c>
       <c r="G205" s="12" t="n">
-        <v>30004</v>
+        <v>60002</v>
       </c>
       <c r="H205" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I205" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="206" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="12" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="B206" s="12" t="s">
         <v>75</v>
@@ -12804,18 +12828,18 @@
         <v>351</v>
       </c>
       <c r="G206" s="12" t="n">
-        <v>30005</v>
+        <v>60003</v>
       </c>
       <c r="H206" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I206" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="12" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="B207" s="12" t="s">
         <v>75</v>
@@ -12833,18 +12857,18 @@
         <v>351</v>
       </c>
       <c r="G207" s="12" t="n">
-        <v>30006</v>
+        <v>60004</v>
       </c>
       <c r="H207" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I207" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="B208" s="12" t="s">
         <v>75</v>
@@ -12862,18 +12886,18 @@
         <v>351</v>
       </c>
       <c r="G208" s="12" t="n">
-        <v>40001</v>
+        <v>60005</v>
       </c>
       <c r="H208" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I208" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="B209" s="12" t="s">
         <v>75</v>
@@ -12891,18 +12915,18 @@
         <v>351</v>
       </c>
       <c r="G209" s="12" t="n">
-        <v>60001</v>
+        <v>60006</v>
       </c>
       <c r="H209" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I209" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="210" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="B210" s="12" t="s">
         <v>75</v>
@@ -12920,18 +12944,18 @@
         <v>351</v>
       </c>
       <c r="G210" s="12" t="n">
-        <v>60002</v>
+        <v>60007</v>
       </c>
       <c r="H210" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="211" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="B211" s="12" t="s">
         <v>75</v>
@@ -12949,1497 +12973,849 @@
         <v>351</v>
       </c>
       <c r="G211" s="12" t="n">
-        <v>60003</v>
+        <v>60008</v>
       </c>
       <c r="H211" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I211" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A212" s="12" t="s">
-        <v>370</v>
-      </c>
-      <c r="B212" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C212" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D212" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E212" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F212" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G212" s="12" t="n">
-        <v>60004</v>
-      </c>
-      <c r="H212" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I212" s="12" t="s">
-        <v>352</v>
+        <v>376</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A212" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B212" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C212" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D212" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E212" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F212" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G212" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H212" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I212" s="3" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A213" s="12" t="s">
-        <v>371</v>
-      </c>
-      <c r="B213" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C213" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D213" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E213" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F213" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G213" s="12" t="n">
-        <v>60005</v>
-      </c>
-      <c r="H213" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I213" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A214" s="12" t="s">
-        <v>372</v>
-      </c>
-      <c r="B214" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C214" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D214" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E214" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F214" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G214" s="12" t="n">
-        <v>60006</v>
-      </c>
-      <c r="H214" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I214" s="12" t="s">
-        <v>352</v>
-      </c>
+      <c r="A213" s="3"/>
+      <c r="B213" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C213" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D213" s="3"/>
+      <c r="E213" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F213" s="3"/>
+      <c r="G213" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H213" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I213" s="3"/>
+    </row>
+    <row r="214" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A214" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="B214" s="5"/>
+      <c r="C214" s="5"/>
+      <c r="D214" s="5"/>
+      <c r="E214" s="5"/>
+      <c r="F214" s="5"/>
+      <c r="G214" s="5"/>
+      <c r="H214" s="5"/>
+      <c r="I214" s="5"/>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A215" s="12" t="s">
-        <v>373</v>
-      </c>
-      <c r="B215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C215" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E215" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F215" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G215" s="12" t="n">
-        <v>60007</v>
-      </c>
-      <c r="H215" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I215" s="12" t="s">
-        <v>352</v>
+      <c r="A215" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B215" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C215" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D215" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E215" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F215" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G215" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="H215" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I215" s="7" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A216" s="12" t="s">
-        <v>374</v>
-      </c>
-      <c r="B216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C216" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E216" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F216" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G216" s="12" t="n">
-        <v>60008</v>
-      </c>
-      <c r="H216" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I216" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A217" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B217" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C217" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D217" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E217" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F217" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G217" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H217" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I217" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="A216" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="B216" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C216" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D216" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E216" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F216" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G216" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="H216" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I216" s="7" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="B217" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C217" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D217" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E217" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F217" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G217" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="H217" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I217" s="7"/>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A218" s="3"/>
-      <c r="B218" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C218" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D218" s="3"/>
-      <c r="E218" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F218" s="3"/>
-      <c r="G218" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H218" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I218" s="3"/>
-    </row>
-    <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A219" s="5" t="s">
-        <v>375</v>
-      </c>
-      <c r="B219" s="5"/>
-      <c r="C219" s="5"/>
-      <c r="D219" s="5"/>
-      <c r="E219" s="5"/>
-      <c r="F219" s="5"/>
-      <c r="G219" s="5"/>
-      <c r="H219" s="5"/>
-      <c r="I219" s="5"/>
-    </row>
-    <row r="220" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A220" s="12" t="s">
-        <v>360</v>
-      </c>
-      <c r="B220" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C220" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D220" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E220" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F220" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G220" s="12" t="n">
-        <v>30001</v>
-      </c>
-      <c r="H220" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I220" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="221" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A221" s="12" t="s">
-        <v>361</v>
-      </c>
-      <c r="B221" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C221" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D221" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E221" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F221" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G221" s="12" t="n">
-        <v>30002</v>
-      </c>
-      <c r="H221" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I221" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="222" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A222" s="12" t="s">
-        <v>362</v>
-      </c>
-      <c r="B222" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C222" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D222" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E222" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F222" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G222" s="12" t="n">
-        <v>30003</v>
-      </c>
-      <c r="H222" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I222" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="223" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A223" s="12" t="s">
-        <v>363</v>
-      </c>
-      <c r="B223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C223" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E223" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F223" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G223" s="12" t="n">
-        <v>30004</v>
-      </c>
-      <c r="H223" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I223" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="224" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A224" s="12" t="s">
-        <v>364</v>
-      </c>
-      <c r="B224" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C224" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D224" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E224" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F224" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G224" s="12" t="n">
-        <v>30005</v>
-      </c>
-      <c r="H224" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I224" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="225" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A225" s="12" t="s">
-        <v>365</v>
-      </c>
-      <c r="B225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C225" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E225" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F225" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G225" s="12" t="n">
-        <v>30006</v>
-      </c>
-      <c r="H225" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I225" s="12" t="s">
-        <v>376</v>
-      </c>
+      <c r="A218" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="B218" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C218" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D218" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E218" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F218" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G218" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="H218" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I218" s="7"/>
+    </row>
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="B219" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C219" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D219" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E219" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F219" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G219" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="H219" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I219" s="7"/>
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="B220" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C220" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D220" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E220" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F220" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G220" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="H220" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I220" s="7"/>
+    </row>
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B221" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C221" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D221" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E221" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F221" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G221" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="H221" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I221" s="7"/>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B222" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C222" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D222" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E222" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F222" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G222" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="H222" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I222" s="7"/>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B223" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C223" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D223" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E223" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F223" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G223" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="H223" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I223" s="7"/>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="B224" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C224" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D224" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E224" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F224" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G224" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="H224" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I224" s="7"/>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="B225" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C225" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D225" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E225" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F225" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G225" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="H225" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I225" s="7"/>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A226" s="12" t="s">
-        <v>366</v>
-      </c>
-      <c r="B226" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C226" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D226" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E226" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F226" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G226" s="12" t="n">
-        <v>40001</v>
-      </c>
-      <c r="H226" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I226" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="227" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A227" s="12" t="s">
-        <v>377</v>
-      </c>
-      <c r="B227" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C227" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D227" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E227" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F227" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G227" s="12" t="n">
-        <v>45001</v>
-      </c>
-      <c r="H227" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I227" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="228" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A228" s="12" t="s">
-        <v>367</v>
-      </c>
-      <c r="B228" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C228" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D228" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E228" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F228" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G228" s="12" t="n">
-        <v>60001</v>
-      </c>
-      <c r="H228" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I228" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="229" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A229" s="12" t="s">
-        <v>368</v>
-      </c>
-      <c r="B229" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C229" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D229" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E229" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F229" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G229" s="12" t="n">
-        <v>60002</v>
-      </c>
-      <c r="H229" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I229" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="230" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A230" s="12" t="s">
-        <v>369</v>
-      </c>
-      <c r="B230" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C230" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D230" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E230" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F230" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G230" s="12" t="n">
-        <v>60003</v>
-      </c>
-      <c r="H230" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I230" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="231" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A231" s="12" t="s">
-        <v>370</v>
-      </c>
-      <c r="B231" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C231" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D231" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E231" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F231" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G231" s="12" t="n">
-        <v>60004</v>
-      </c>
-      <c r="H231" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I231" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="232" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A232" s="12" t="s">
-        <v>371</v>
-      </c>
-      <c r="B232" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C232" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D232" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E232" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F232" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G232" s="12" t="n">
-        <v>60005</v>
-      </c>
-      <c r="H232" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I232" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="233" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A233" s="12" t="s">
-        <v>372</v>
-      </c>
-      <c r="B233" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C233" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D233" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E233" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F233" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G233" s="12" t="n">
-        <v>60006</v>
-      </c>
-      <c r="H233" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I233" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="234" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A234" s="12" t="s">
-        <v>373</v>
-      </c>
-      <c r="B234" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C234" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D234" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E234" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F234" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G234" s="12" t="n">
-        <v>60007</v>
-      </c>
-      <c r="H234" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I234" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="235" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A235" s="12" t="s">
-        <v>374</v>
-      </c>
-      <c r="B235" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C235" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="D235" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E235" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F235" s="12" t="s">
-        <v>351</v>
-      </c>
-      <c r="G235" s="12" t="n">
-        <v>60008</v>
-      </c>
-      <c r="H235" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I235" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A236" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B236" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C236" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D236" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E236" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F236" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G236" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H236" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I236" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A237" s="3"/>
-      <c r="B237" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C237" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D237" s="3"/>
-      <c r="E237" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F237" s="3"/>
-      <c r="G237" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H237" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I237" s="3"/>
-    </row>
-    <row r="238" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A238" s="5" t="s">
-        <v>317</v>
-      </c>
-      <c r="B238" s="5"/>
-      <c r="C238" s="5"/>
-      <c r="D238" s="5"/>
-      <c r="E238" s="5"/>
-      <c r="F238" s="5"/>
-      <c r="G238" s="5"/>
-      <c r="H238" s="5"/>
-      <c r="I238" s="5"/>
-    </row>
-    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A239" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B239" s="7" t="s">
+      <c r="A226" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="B226" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C226" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D226" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E226" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F226" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G226" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="H226" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I226" s="7"/>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="B227" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C239" s="7" t="s">
+      <c r="C227" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D239" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E239" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F239" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G239" s="10" t="s">
-        <v>318</v>
-      </c>
-      <c r="H239" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I239" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A240" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="B240" s="7" t="s">
+      <c r="D227" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E227" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F227" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G227" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="H227" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I227" s="7"/>
+    </row>
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="B228" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C240" s="7" t="s">
+      <c r="C228" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D240" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E240" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F240" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G240" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="H240" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I240" s="7" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A241" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="B241" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C241" s="7" t="s">
+      <c r="D228" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E228" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F228" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G228" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H228" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I228" s="7"/>
+    </row>
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="B229" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="C229" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D241" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E241" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F241" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G241" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="H241" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I241" s="7"/>
-    </row>
-    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A242" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="B242" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C242" s="7" t="s">
+      <c r="D229" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E229" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F229" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G229" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="H229" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I229" s="7"/>
+    </row>
+    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="B230" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="C230" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D242" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E242" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F242" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G242" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="H242" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I242" s="7"/>
-    </row>
-    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A243" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="B243" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C243" s="7" t="s">
+      <c r="D230" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E230" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F230" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G230" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="H230" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I230" s="7"/>
+    </row>
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="B231" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C231" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D243" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E243" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F243" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G243" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="H243" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I243" s="7"/>
-    </row>
-    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A244" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="B244" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C244" s="7" t="s">
+      <c r="D231" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E231" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F231" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G231" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="H231" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I231" s="7"/>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="B232" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C232" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D244" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E244" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F244" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G244" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="H244" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I244" s="7"/>
-    </row>
-    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A245" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="B245" s="7" t="s">
+      <c r="D232" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E232" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F232" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G232" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="H232" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I232" s="7"/>
+    </row>
+    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B233" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C245" s="7" t="s">
+      <c r="C233" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D245" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E245" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F245" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G245" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="H245" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I245" s="7"/>
-    </row>
-    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A246" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="B246" s="7" t="s">
+      <c r="D233" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E233" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F233" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G233" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H233" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I233" s="7"/>
+    </row>
+    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B234" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C246" s="7" t="s">
+      <c r="C234" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D246" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E246" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F246" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G246" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="H246" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I246" s="7"/>
-    </row>
-    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A247" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="B247" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C247" s="7" t="s">
+      <c r="D234" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E234" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F234" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G234" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="H234" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I234" s="7"/>
+    </row>
+    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="B235" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C235" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D247" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E247" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F247" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G247" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="H247" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I247" s="7"/>
-    </row>
-    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A248" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="B248" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C248" s="7" t="s">
+      <c r="D235" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E235" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F235" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G235" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="H235" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I235" s="7" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B236" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C236" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D248" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E248" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F248" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G248" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="H248" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I248" s="7"/>
-    </row>
-    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A249" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="B249" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C249" s="7" t="s">
+      <c r="D236" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E236" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F236" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G236" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="H236" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I236" s="7" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="B237" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C237" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D249" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E249" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F249" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G249" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="H249" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I249" s="7"/>
-    </row>
-    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A250" s="9" t="s">
-        <v>215</v>
-      </c>
-      <c r="B250" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C250" s="7" t="s">
+      <c r="D237" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E237" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F237" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G237" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="H237" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I237" s="12" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="238" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="B238" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C238" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D250" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E250" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F250" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G250" s="10" t="s">
-        <v>216</v>
-      </c>
-      <c r="H250" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I250" s="7"/>
-    </row>
-    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A251" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="B251" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C251" s="7" t="s">
+      <c r="D238" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E238" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F238" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G238" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="H238" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I238" s="12" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="239" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A239" s="11" t="s">
+        <v>325</v>
+      </c>
+      <c r="B239" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C239" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D251" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E251" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F251" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G251" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="H251" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I251" s="7"/>
-    </row>
-    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A252" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="B252" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C252" s="7" t="s">
+      <c r="D239" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E239" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F239" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G239" s="13" t="s">
+        <v>326</v>
+      </c>
+      <c r="H239" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I239" s="12" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="240" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A240" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="B240" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C240" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D252" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E252" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F252" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G252" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="H252" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I252" s="7"/>
-    </row>
-    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A253" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="B253" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="C253" s="7" t="s">
+      <c r="D240" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E240" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F240" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G240" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="H240" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I240" s="12" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="241" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="11" t="s">
+        <v>382</v>
+      </c>
+      <c r="B241" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C241" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D253" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E253" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F253" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G253" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="H253" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I253" s="7"/>
-    </row>
-    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A254" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="B254" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="C254" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D254" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E254" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F254" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G254" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="H254" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I254" s="7"/>
-    </row>
-    <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A255" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="B255" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="C255" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D255" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E255" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F255" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G255" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="H255" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I255" s="7"/>
-    </row>
-    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A256" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="B256" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="C256" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D256" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E256" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F256" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G256" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="H256" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I256" s="7"/>
-    </row>
-    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A257" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="B257" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C257" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D257" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E257" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F257" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G257" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="H257" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I257" s="7"/>
-    </row>
-    <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A258" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="B258" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C258" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D258" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E258" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F258" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G258" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="H258" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I258" s="7"/>
-    </row>
-    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A259" s="7" t="s">
-        <v>234</v>
-      </c>
-      <c r="B259" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C259" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D259" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E259" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F259" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G259" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="H259" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I259" s="7" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A260" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="B260" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C260" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D260" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E260" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F260" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G260" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="H260" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I260" s="7" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="261" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A261" s="12" t="s">
-        <v>239</v>
-      </c>
-      <c r="B261" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C261" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D261" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E261" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F261" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G261" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="H261" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I261" s="12" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="262" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A262" s="12" t="s">
-        <v>241</v>
-      </c>
-      <c r="B262" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C262" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D262" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E262" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F262" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G262" s="12" t="s">
-        <v>242</v>
-      </c>
-      <c r="H262" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I262" s="12" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="263" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A263" s="11" t="s">
-        <v>325</v>
-      </c>
-      <c r="B263" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C263" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D263" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E263" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F263" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G263" s="13" t="s">
-        <v>326</v>
-      </c>
-      <c r="H263" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I263" s="12" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="264" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A264" s="11" t="s">
-        <v>328</v>
-      </c>
-      <c r="B264" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C264" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D264" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E264" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F264" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G264" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="H264" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I264" s="12" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="265" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A265" s="11" t="s">
-        <v>382</v>
-      </c>
-      <c r="B265" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C265" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D265" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E265" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F265" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G265" s="13" t="s">
+      <c r="D241" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E241" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F241" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G241" s="13" t="s">
         <v>332</v>
       </c>
-      <c r="H265" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I265" s="12" t="s">
+      <c r="H241" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I241" s="12" t="s">
         <v>383</v>
       </c>
     </row>
+    <row r="1048553" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048555" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048556" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="25">
     <mergeCell ref="A6:A7"/>
@@ -14452,21 +13828,21 @@
     <mergeCell ref="F115:F116"/>
     <mergeCell ref="I115:I116"/>
     <mergeCell ref="A117:I117"/>
-    <mergeCell ref="A191:A192"/>
-    <mergeCell ref="D191:D192"/>
-    <mergeCell ref="F191:F192"/>
-    <mergeCell ref="I191:I192"/>
-    <mergeCell ref="A193:I193"/>
-    <mergeCell ref="A217:A218"/>
-    <mergeCell ref="D217:D218"/>
-    <mergeCell ref="F217:F218"/>
-    <mergeCell ref="I217:I218"/>
-    <mergeCell ref="A219:I219"/>
-    <mergeCell ref="A236:A237"/>
-    <mergeCell ref="D236:D237"/>
-    <mergeCell ref="F236:F237"/>
-    <mergeCell ref="I236:I237"/>
-    <mergeCell ref="A238:I238"/>
+    <mergeCell ref="A167:A168"/>
+    <mergeCell ref="D167:D168"/>
+    <mergeCell ref="F167:F168"/>
+    <mergeCell ref="I167:I168"/>
+    <mergeCell ref="A169:I169"/>
+    <mergeCell ref="A193:A194"/>
+    <mergeCell ref="D193:D194"/>
+    <mergeCell ref="F193:F194"/>
+    <mergeCell ref="I193:I194"/>
+    <mergeCell ref="A195:I195"/>
+    <mergeCell ref="A212:A213"/>
+    <mergeCell ref="D212:D213"/>
+    <mergeCell ref="F212:F213"/>
+    <mergeCell ref="I212:I213"/>
+    <mergeCell ref="A214:I214"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
SOCO: Improv: Add rated current in datasheet
Also committed any changes in modbus table.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Modbus Table" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Internal Modbus Table" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="EMS Testing Firmware" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2355" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="384">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -1104,6 +1105,102 @@
     <t xml:space="preserve">Internal Only. Not visible to customer. 
 If set to non-zero, it advances the calibration state machine when it is waiting for external input. Only writtable when test mode enabled.</t>
   </si>
+  <si>
+    <t xml:space="preserve">EMS (Energy Management System)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel Test Firmware V1.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RS485 Port of EMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">READ MULTIPLE HOLDING REGISTERS (Function Code: 0x03)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temperature Sensor 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temperature sensor #1 reading</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temperature Sensor 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temperature sensor #2 reading</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery Voltage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">48VDC Battery voltage (Analog Input 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAN Connectivity Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0: Disconnected, 1: Connected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0: Inactive, 1: Active</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">65015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTES (Panel Test Firmware Behaviour)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. EMS Serial parameters are (baud rate: 9600, parity: No parity, stop bits: 1, slave ID: 1). These are same as the default modbus parameters for SOCO.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. The customer Modbus master connects to the  RS-485 port 1 of the EMS. The EMS in turn talks to SOCO over its RS-485 port 2. Only the port 1 is exposed externally for panel testing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. EMS routes incoming requests on a per-address basis: holding registers in the 65001-65016 range listed above are answered locally by the EMS (panel test firmware). Every other request - regardless of function code (0x01 Read Coils, 0x02 Read Discrete Inputs, 0x03 Read Holding Registers outside 65001-65016, 0x05 Write Single Coil, 0x06 Write Single Holding Register, 0x10 Write Multiple Holding Registers, etc.) - is forwarded transparently to SOCO and the SOCO response is relayed back to the master.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. The EMS-local register block (65001-65016) was chosen to sit above the highest SOCO Modbus address currently in use while still fitting inside the Modbus 16-bit address space (maximum 1-based address = 65536, since the on-the-wire address field is 2 bytes). This leaves clear separation from SOCO and still keeps every byte of every frame within the standard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. All EMS-local entries are exposed only via Function Code 0x03 (Read Multiple Holding Registers). Writes to 65001-65016 will be rejected with Modbus exception 0x02 (Illegal Data Address).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Float values use IEEE-754 32-bit, transmitted high-word first (big-endian word order), matching the SOCO convention. The two Modbus registers must be read together in a single request.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Boolean values (Digital Input 1-4, LAN Connectivity Status) are encoded as 32-bit unsigned integers in the same 2-register format. Only the LSB carries information: 0 = inactive/disconnected, 1 = active/connected. All other bits are reserved and read as 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. The Digital Inputs reflect the raw electrical state of the EMS DI pins after debouncing; their mapping to panel signals is defined by the panel wiring drawing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. The 'LAN Connectivity Status' bit is set when the Ethernet PHY reports link-up AND a valid IPv4 address has been acquired (static or DHCP). It is cleared on link-down or IP loss.</t>
+  </si>
 </sst>
 </file>
 
@@ -1112,7 +1209,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1161,6 +1258,28 @@
     <font>
       <b val="true"/>
       <sz val="8"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1285,7 +1404,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1340,6 +1459,30 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1592,7 +1735,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I1048576"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.94"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.15"/>
@@ -12056,7 +12199,7 @@
       <c r="H199" s="5"/>
       <c r="I199" s="5"/>
     </row>
-    <row r="200" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="12" t="s">
         <v>328</v>
       </c>
@@ -12085,7 +12228,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="12" t="s">
         <v>329</v>
       </c>
@@ -12114,7 +12257,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="12" t="s">
         <v>330</v>
       </c>
@@ -12143,7 +12286,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="12" t="s">
         <v>331</v>
       </c>
@@ -12172,7 +12315,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="12" t="s">
         <v>332</v>
       </c>
@@ -12201,7 +12344,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="12" t="s">
         <v>333</v>
       </c>
@@ -12259,7 +12402,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="12" t="s">
         <v>345</v>
       </c>
@@ -12288,7 +12431,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
         <v>335</v>
       </c>
@@ -12317,7 +12460,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
         <v>336</v>
       </c>
@@ -12346,7 +12489,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
         <v>337</v>
       </c>
@@ -12375,7 +12518,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
         <v>338</v>
       </c>
@@ -12404,7 +12547,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="212" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="12" t="s">
         <v>339</v>
       </c>
@@ -12433,7 +12576,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="12" t="s">
         <v>340</v>
       </c>
@@ -12462,7 +12605,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="12" t="s">
         <v>341</v>
       </c>
@@ -12491,7 +12634,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="12" t="s">
         <v>342</v>
       </c>
@@ -13185,7 +13328,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="12" t="s">
         <v>240</v>
       </c>
@@ -13214,7 +13357,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="12" t="s">
         <v>242</v>
       </c>
@@ -13243,7 +13386,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="243" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="45.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="11" t="s">
         <v>308</v>
       </c>
@@ -13272,7 +13415,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="244" customFormat="false" ht="47.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="244" customFormat="false" ht="36.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="11" t="s">
         <v>311</v>
       </c>
@@ -13301,7 +13444,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="11" t="s">
         <v>350</v>
       </c>
@@ -13386,4 +13529,516 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40.86"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
+        <v>354</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="16"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="H10" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="18" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="H11" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="18" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="H12" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="18" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>366</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="H13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="H14" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="18" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="H15" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" s="18" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="18" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="18" t="s">
+        <v>373</v>
+      </c>
+      <c r="H17" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" s="18" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+    </row>
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
+        <v>375</v>
+      </c>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19"/>
+    </row>
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19" t="s">
+        <v>376</v>
+      </c>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="19"/>
+      <c r="I22" s="19"/>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19" t="s">
+        <v>377</v>
+      </c>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="19" t="s">
+        <v>378</v>
+      </c>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="19"/>
+      <c r="I24" s="19"/>
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="19" t="s">
+        <v>379</v>
+      </c>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="19" t="s">
+        <v>380</v>
+      </c>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="19" t="s">
+        <v>381</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="19" t="s">
+        <v>382</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="19" t="s">
+        <v>383</v>
+      </c>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="19"/>
+      <c r="I29" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A29:I29"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
SOCO: Feature: Add a scratchpad over Modbus
Allows testing team to detect any unintential/accidental POR of SOCO during
testing.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Customer Modbus Table" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2450" uniqueCount="387">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -991,6 +991,16 @@
 26,27,28: Low Point Calibration In Progress
 127: Calibration Completed Successfully
 126: Error occured during calibration. Please restart controller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scratch Pad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal Only. Not visible to customer. 
+Used to store a temporarily value. Resets when SOCO restarts on POR.</t>
   </si>
   <si>
     <t xml:space="preserve">READ COIL STATUS (Function Code: 0x01)</t>
@@ -1404,7 +1414,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1461,27 +1471,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9912,99 +9914,101 @@
         <v>316</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A115" s="3" t="s">
+    <row r="115" customFormat="false" ht="36.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A115" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="B115" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C115" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D115" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E115" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G115" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="H115" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I115" s="12" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B115" s="4" t="s">
+      <c r="B116" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C115" s="4" t="s">
+      <c r="C116" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D115" s="3" t="s">
+      <c r="D116" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E115" s="4" t="s">
+      <c r="E116" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F115" s="3" t="s">
+      <c r="F116" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G115" s="4" t="s">
+      <c r="G116" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H115" s="4" t="s">
+      <c r="H116" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I115" s="3" t="s">
+      <c r="I116" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="3"/>
-      <c r="B116" s="4" t="s">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="3"/>
+      <c r="B117" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C116" s="4" t="s">
+      <c r="C117" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D116" s="3"/>
-      <c r="E116" s="4" t="s">
+      <c r="D117" s="3"/>
+      <c r="E117" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F116" s="3"/>
-      <c r="G116" s="4" t="s">
+      <c r="F117" s="3"/>
+      <c r="G117" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H116" s="4" t="s">
+      <c r="H117" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I116" s="3"/>
-    </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A117" s="5" t="s">
+      <c r="I117" s="3"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A118" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="B117" s="5"/>
-      <c r="C117" s="5"/>
-      <c r="D117" s="5"/>
-      <c r="E117" s="5"/>
-      <c r="F117" s="5"/>
-      <c r="G117" s="5"/>
-      <c r="H117" s="5"/>
-      <c r="I117" s="5"/>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="B118" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C118" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="D118" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E118" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F118" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="G118" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H118" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I118" s="7"/>
+      <c r="B118" s="5"/>
+      <c r="C118" s="5"/>
+      <c r="D118" s="5"/>
+      <c r="E118" s="5"/>
+      <c r="F118" s="5"/>
+      <c r="G118" s="5"/>
+      <c r="H118" s="5"/>
+      <c r="I118" s="5"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="7" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B119" s="7" t="s">
         <v>75</v>
@@ -10022,7 +10026,7 @@
         <v>249</v>
       </c>
       <c r="G119" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H119" s="7" t="n">
         <v>1</v>
@@ -10031,7 +10035,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B120" s="7" t="s">
         <v>75</v>
@@ -10049,7 +10053,7 @@
         <v>249</v>
       </c>
       <c r="G120" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H120" s="7" t="n">
         <v>1</v>
@@ -10058,7 +10062,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B121" s="7" t="s">
         <v>75</v>
@@ -10076,7 +10080,7 @@
         <v>249</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H121" s="7" t="n">
         <v>1</v>
@@ -10085,7 +10089,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B122" s="7" t="s">
         <v>75</v>
@@ -10103,7 +10107,7 @@
         <v>249</v>
       </c>
       <c r="G122" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H122" s="7" t="n">
         <v>1</v>
@@ -10112,7 +10116,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B123" s="7" t="s">
         <v>75</v>
@@ -10130,7 +10134,7 @@
         <v>249</v>
       </c>
       <c r="G123" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H123" s="7" t="n">
         <v>1</v>
@@ -10139,7 +10143,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B124" s="7" t="s">
         <v>75</v>
@@ -10157,7 +10161,7 @@
         <v>249</v>
       </c>
       <c r="G124" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H124" s="7" t="n">
         <v>1</v>
@@ -10166,7 +10170,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B125" s="7" t="s">
         <v>75</v>
@@ -10184,7 +10188,7 @@
         <v>249</v>
       </c>
       <c r="G125" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H125" s="7" t="n">
         <v>1</v>
@@ -10193,7 +10197,7 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B126" s="7" t="s">
         <v>75</v>
@@ -10211,7 +10215,7 @@
         <v>249</v>
       </c>
       <c r="G126" s="7" t="n">
-        <v>201</v>
+        <v>8</v>
       </c>
       <c r="H126" s="7" t="n">
         <v>1</v>
@@ -10220,7 +10224,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B127" s="7" t="s">
         <v>75</v>
@@ -10238,7 +10242,7 @@
         <v>249</v>
       </c>
       <c r="G127" s="7" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H127" s="7" t="n">
         <v>1</v>
@@ -10247,7 +10251,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B128" s="7" t="s">
         <v>75</v>
@@ -10265,7 +10269,7 @@
         <v>249</v>
       </c>
       <c r="G128" s="7" t="n">
-        <v>301</v>
+        <v>202</v>
       </c>
       <c r="H128" s="7" t="n">
         <v>1</v>
@@ -10274,7 +10278,7 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B129" s="7" t="s">
         <v>75</v>
@@ -10292,7 +10296,7 @@
         <v>249</v>
       </c>
       <c r="G129" s="7" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H129" s="7" t="n">
         <v>1</v>
@@ -10301,7 +10305,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B130" s="7" t="s">
         <v>75</v>
@@ -10319,7 +10323,7 @@
         <v>249</v>
       </c>
       <c r="G130" s="7" t="n">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H130" s="7" t="n">
         <v>1</v>
@@ -10328,7 +10332,7 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B131" s="7" t="s">
         <v>75</v>
@@ -10346,7 +10350,7 @@
         <v>249</v>
       </c>
       <c r="G131" s="7" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H131" s="7" t="n">
         <v>1</v>
@@ -10355,7 +10359,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B132" s="7" t="s">
         <v>75</v>
@@ -10373,7 +10377,7 @@
         <v>249</v>
       </c>
       <c r="G132" s="7" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H132" s="7" t="n">
         <v>1</v>
@@ -10382,7 +10386,7 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B133" s="7" t="s">
         <v>75</v>
@@ -10400,7 +10404,7 @@
         <v>249</v>
       </c>
       <c r="G133" s="7" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H133" s="7" t="n">
         <v>1</v>
@@ -10409,7 +10413,7 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B134" s="7" t="s">
         <v>75</v>
@@ -10427,7 +10431,7 @@
         <v>249</v>
       </c>
       <c r="G134" s="7" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H134" s="7" t="n">
         <v>1</v>
@@ -10436,7 +10440,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="7" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B135" s="7" t="s">
         <v>75</v>
@@ -10454,7 +10458,7 @@
         <v>249</v>
       </c>
       <c r="G135" s="7" t="n">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H135" s="7" t="n">
         <v>1</v>
@@ -10463,7 +10467,7 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B136" s="7" t="s">
         <v>75</v>
@@ -10481,7 +10485,7 @@
         <v>249</v>
       </c>
       <c r="G136" s="7" t="n">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H136" s="7" t="n">
         <v>1</v>
@@ -10490,7 +10494,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B137" s="7" t="s">
         <v>75</v>
@@ -10508,7 +10512,7 @@
         <v>249</v>
       </c>
       <c r="G137" s="7" t="n">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H137" s="7" t="n">
         <v>1</v>
@@ -10517,7 +10521,7 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B138" s="7" t="s">
         <v>75</v>
@@ -10535,7 +10539,7 @@
         <v>249</v>
       </c>
       <c r="G138" s="7" t="n">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H138" s="7" t="n">
         <v>1</v>
@@ -10544,7 +10548,7 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B139" s="7" t="s">
         <v>75</v>
@@ -10562,7 +10566,7 @@
         <v>249</v>
       </c>
       <c r="G139" s="7" t="n">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H139" s="7" t="n">
         <v>1</v>
@@ -10571,7 +10575,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B140" s="7" t="s">
         <v>75</v>
@@ -10589,7 +10593,7 @@
         <v>249</v>
       </c>
       <c r="G140" s="7" t="n">
-        <v>401</v>
+        <v>312</v>
       </c>
       <c r="H140" s="7" t="n">
         <v>1</v>
@@ -10598,7 +10602,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B141" s="7" t="s">
         <v>75</v>
@@ -10616,7 +10620,7 @@
         <v>249</v>
       </c>
       <c r="G141" s="7" t="n">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H141" s="7" t="n">
         <v>1</v>
@@ -10625,7 +10629,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="7" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B142" s="7" t="s">
         <v>75</v>
@@ -10643,7 +10647,7 @@
         <v>249</v>
       </c>
       <c r="G142" s="7" t="n">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="H142" s="7" t="n">
         <v>1</v>
@@ -10652,7 +10656,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B143" s="7" t="s">
         <v>75</v>
@@ -10670,7 +10674,7 @@
         <v>249</v>
       </c>
       <c r="G143" s="7" t="n">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="H143" s="7" t="n">
         <v>1</v>
@@ -10679,7 +10683,7 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B144" s="7" t="s">
         <v>75</v>
@@ -10697,7 +10701,7 @@
         <v>249</v>
       </c>
       <c r="G144" s="7" t="n">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="H144" s="7" t="n">
         <v>1</v>
@@ -10706,7 +10710,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B145" s="7" t="s">
         <v>75</v>
@@ -10724,7 +10728,7 @@
         <v>249</v>
       </c>
       <c r="G145" s="7" t="n">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="H145" s="7" t="n">
         <v>1</v>
@@ -10733,7 +10737,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B146" s="7" t="s">
         <v>75</v>
@@ -10751,7 +10755,7 @@
         <v>249</v>
       </c>
       <c r="G146" s="7" t="n">
-        <v>601</v>
+        <v>406</v>
       </c>
       <c r="H146" s="7" t="n">
         <v>1</v>
@@ -10760,7 +10764,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B147" s="7" t="s">
         <v>75</v>
@@ -10778,7 +10782,7 @@
         <v>249</v>
       </c>
       <c r="G147" s="7" t="n">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="H147" s="7" t="n">
         <v>1</v>
@@ -10787,7 +10791,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B148" s="7" t="s">
         <v>75</v>
@@ -10805,7 +10809,7 @@
         <v>249</v>
       </c>
       <c r="G148" s="7" t="n">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="H148" s="7" t="n">
         <v>1</v>
@@ -10814,7 +10818,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="7" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B149" s="7" t="s">
         <v>75</v>
@@ -10832,7 +10836,7 @@
         <v>249</v>
       </c>
       <c r="G149" s="7" t="n">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="H149" s="7" t="n">
         <v>1</v>
@@ -10841,7 +10845,7 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="7" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B150" s="7" t="s">
         <v>75</v>
@@ -10859,7 +10863,7 @@
         <v>249</v>
       </c>
       <c r="G150" s="7" t="n">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="H150" s="7" t="n">
         <v>1</v>
@@ -10868,7 +10872,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="7" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B151" s="7" t="s">
         <v>75</v>
@@ -10886,7 +10890,7 @@
         <v>249</v>
       </c>
       <c r="G151" s="7" t="n">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="H151" s="7" t="n">
         <v>1</v>
@@ -10895,7 +10899,7 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B152" s="7" t="s">
         <v>75</v>
@@ -10913,7 +10917,7 @@
         <v>249</v>
       </c>
       <c r="G152" s="7" t="n">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="H152" s="7" t="n">
         <v>1</v>
@@ -10922,7 +10926,7 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B153" s="7" t="s">
         <v>75</v>
@@ -10940,7 +10944,7 @@
         <v>249</v>
       </c>
       <c r="G153" s="7" t="n">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="H153" s="7" t="n">
         <v>1</v>
@@ -10949,7 +10953,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="7" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B154" s="7" t="s">
         <v>75</v>
@@ -10967,7 +10971,7 @@
         <v>249</v>
       </c>
       <c r="G154" s="7" t="n">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="H154" s="7" t="n">
         <v>1</v>
@@ -10976,7 +10980,7 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B155" s="7" t="s">
         <v>75</v>
@@ -10994,7 +10998,7 @@
         <v>249</v>
       </c>
       <c r="G155" s="7" t="n">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="H155" s="7" t="n">
         <v>1</v>
@@ -11003,7 +11007,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B156" s="7" t="s">
         <v>75</v>
@@ -11021,7 +11025,7 @@
         <v>249</v>
       </c>
       <c r="G156" s="7" t="n">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="H156" s="7" t="n">
         <v>1</v>
@@ -11030,7 +11034,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="7" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B157" s="7" t="s">
         <v>75</v>
@@ -11048,7 +11052,7 @@
         <v>249</v>
       </c>
       <c r="G157" s="7" t="n">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="H157" s="7" t="n">
         <v>1</v>
@@ -11057,7 +11061,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B158" s="7" t="s">
         <v>75</v>
@@ -11075,7 +11079,7 @@
         <v>249</v>
       </c>
       <c r="G158" s="7" t="n">
-        <v>801</v>
+        <v>612</v>
       </c>
       <c r="H158" s="7" t="n">
         <v>1</v>
@@ -11084,7 +11088,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B159" s="7" t="s">
         <v>75</v>
@@ -11102,7 +11106,7 @@
         <v>249</v>
       </c>
       <c r="G159" s="7" t="n">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="H159" s="7" t="n">
         <v>1</v>
@@ -11111,7 +11115,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B160" s="7" t="s">
         <v>75</v>
@@ -11129,7 +11133,7 @@
         <v>249</v>
       </c>
       <c r="G160" s="7" t="n">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="H160" s="7" t="n">
         <v>1</v>
@@ -11138,7 +11142,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="7" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B161" s="7" t="s">
         <v>75</v>
@@ -11156,7 +11160,7 @@
         <v>249</v>
       </c>
       <c r="G161" s="7" t="n">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="H161" s="7" t="n">
         <v>1</v>
@@ -11165,7 +11169,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="7" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B162" s="7" t="s">
         <v>75</v>
@@ -11183,7 +11187,7 @@
         <v>249</v>
       </c>
       <c r="G162" s="7" t="n">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="H162" s="7" t="n">
         <v>1</v>
@@ -11192,7 +11196,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B163" s="7" t="s">
         <v>75</v>
@@ -11210,7 +11214,7 @@
         <v>249</v>
       </c>
       <c r="G163" s="7" t="n">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="H163" s="7" t="n">
         <v>1</v>
@@ -11219,7 +11223,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B164" s="7" t="s">
         <v>75</v>
@@ -11237,7 +11241,7 @@
         <v>249</v>
       </c>
       <c r="G164" s="7" t="n">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="H164" s="7" t="n">
         <v>1</v>
@@ -11246,7 +11250,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B165" s="7" t="s">
         <v>75</v>
@@ -11264,7 +11268,7 @@
         <v>249</v>
       </c>
       <c r="G165" s="7" t="n">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="H165" s="7" t="n">
         <v>1</v>
@@ -11273,7 +11277,7 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B166" s="7" t="s">
         <v>75</v>
@@ -11291,7 +11295,7 @@
         <v>249</v>
       </c>
       <c r="G166" s="7" t="n">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="H166" s="7" t="n">
         <v>1</v>
@@ -11300,7 +11304,7 @@
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B167" s="7" t="s">
         <v>75</v>
@@ -11318,7 +11322,7 @@
         <v>249</v>
       </c>
       <c r="G167" s="7" t="n">
-        <v>901</v>
+        <v>809</v>
       </c>
       <c r="H167" s="7" t="n">
         <v>1</v>
@@ -11327,7 +11331,7 @@
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="7" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B168" s="7" t="s">
         <v>75</v>
@@ -11345,7 +11349,7 @@
         <v>249</v>
       </c>
       <c r="G168" s="7" t="n">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="H168" s="7" t="n">
         <v>1</v>
@@ -11354,7 +11358,7 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="7" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B169" s="7" t="s">
         <v>75</v>
@@ -11372,7 +11376,7 @@
         <v>249</v>
       </c>
       <c r="G169" s="7" t="n">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="H169" s="7" t="n">
         <v>1</v>
@@ -11381,7 +11385,7 @@
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="7" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B170" s="7" t="s">
         <v>75</v>
@@ -11399,104 +11403,102 @@
         <v>249</v>
       </c>
       <c r="G170" s="7" t="n">
+        <v>903</v>
+      </c>
+      <c r="H170" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I170" s="7"/>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="B171" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C171" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D171" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E171" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F171" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G171" s="7" t="n">
         <v>904</v>
       </c>
-      <c r="H170" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I170" s="7"/>
-    </row>
-    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A171" s="3" t="s">
+      <c r="H171" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I171" s="7"/>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A172" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B171" s="4" t="s">
+      <c r="B172" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C171" s="4" t="s">
+      <c r="C172" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D171" s="3" t="s">
+      <c r="D172" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E171" s="4" t="s">
+      <c r="E172" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F171" s="3" t="s">
+      <c r="F172" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G171" s="4" t="s">
+      <c r="G172" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H171" s="4" t="s">
+      <c r="H172" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I171" s="3" t="s">
+      <c r="I172" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A172" s="3"/>
-      <c r="B172" s="4" t="s">
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="3"/>
+      <c r="B173" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C172" s="4" t="s">
+      <c r="C173" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D172" s="3"/>
-      <c r="E172" s="4" t="s">
+      <c r="D173" s="3"/>
+      <c r="E173" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F172" s="3"/>
-      <c r="G172" s="4" t="s">
+      <c r="F173" s="3"/>
+      <c r="G173" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H172" s="4" t="s">
+      <c r="H173" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I172" s="3"/>
-    </row>
-    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A173" s="5" t="s">
-        <v>317</v>
-      </c>
-      <c r="B173" s="5"/>
-      <c r="C173" s="5"/>
-      <c r="D173" s="5"/>
-      <c r="E173" s="5"/>
-      <c r="F173" s="5"/>
-      <c r="G173" s="5"/>
-      <c r="H173" s="5"/>
-      <c r="I173" s="5"/>
-    </row>
-    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A174" s="12" t="s">
-        <v>318</v>
-      </c>
-      <c r="B174" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C174" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D174" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E174" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F174" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="G174" s="12" t="n">
-        <v>20001</v>
-      </c>
-      <c r="H174" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I174" s="12" t="s">
+      <c r="I173" s="3"/>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A174" s="5" t="s">
         <v>320</v>
       </c>
+      <c r="B174" s="5"/>
+      <c r="C174" s="5"/>
+      <c r="D174" s="5"/>
+      <c r="E174" s="5"/>
+      <c r="F174" s="5"/>
+      <c r="G174" s="5"/>
+      <c r="H174" s="5"/>
+      <c r="I174" s="5"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="12" t="s">
@@ -11515,79 +11517,79 @@
         <v>75</v>
       </c>
       <c r="F175" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G175" s="12" t="n">
-        <v>20002</v>
+        <v>20001</v>
       </c>
       <c r="H175" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I175" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="12" t="s">
+        <v>324</v>
+      </c>
+      <c r="B176" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C176" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D176" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E176" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F176" s="12" t="s">
         <v>322</v>
       </c>
-      <c r="B176" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C176" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D176" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E176" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F176" s="12" t="s">
-        <v>319</v>
-      </c>
       <c r="G176" s="12" t="n">
-        <v>20003</v>
+        <v>20002</v>
       </c>
       <c r="H176" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I176" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="12" t="s">
+        <v>325</v>
+      </c>
+      <c r="B177" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C177" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D177" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E177" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F177" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="G177" s="12" t="n">
+        <v>20003</v>
+      </c>
+      <c r="H177" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I177" s="12" t="s">
         <v>323</v>
-      </c>
-      <c r="B177" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C177" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D177" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E177" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F177" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="G177" s="12" t="n">
-        <v>20004</v>
-      </c>
-      <c r="H177" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I177" s="12" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="12" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B178" s="12" t="s">
         <v>75</v>
@@ -11602,21 +11604,21 @@
         <v>75</v>
       </c>
       <c r="F178" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G178" s="12" t="n">
-        <v>20005</v>
+        <v>20004</v>
       </c>
       <c r="H178" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I178" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="12" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B179" s="12" t="s">
         <v>75</v>
@@ -11631,21 +11633,21 @@
         <v>75</v>
       </c>
       <c r="F179" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G179" s="12" t="n">
-        <v>20006</v>
+        <v>20005</v>
       </c>
       <c r="H179" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I179" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="12" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B180" s="12" t="s">
         <v>75</v>
@@ -11660,21 +11662,21 @@
         <v>75</v>
       </c>
       <c r="F180" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G180" s="12" t="n">
-        <v>20007</v>
+        <v>20006</v>
       </c>
       <c r="H180" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I180" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="12" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B181" s="12" t="s">
         <v>75</v>
@@ -11689,21 +11691,21 @@
         <v>75</v>
       </c>
       <c r="F181" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G181" s="12" t="n">
-        <v>20008</v>
+        <v>20007</v>
       </c>
       <c r="H181" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I181" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="12" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B182" s="12" t="s">
         <v>75</v>
@@ -11718,21 +11720,21 @@
         <v>75</v>
       </c>
       <c r="F182" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G182" s="12" t="n">
-        <v>30001</v>
+        <v>20008</v>
       </c>
       <c r="H182" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I182" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="12" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B183" s="12" t="s">
         <v>75</v>
@@ -11747,21 +11749,21 @@
         <v>75</v>
       </c>
       <c r="F183" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G183" s="12" t="n">
-        <v>30002</v>
+        <v>30001</v>
       </c>
       <c r="H183" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I183" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="12" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B184" s="12" t="s">
         <v>75</v>
@@ -11776,21 +11778,21 @@
         <v>75</v>
       </c>
       <c r="F184" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G184" s="12" t="n">
-        <v>30003</v>
+        <v>30002</v>
       </c>
       <c r="H184" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I184" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="12" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B185" s="12" t="s">
         <v>75</v>
@@ -11805,21 +11807,21 @@
         <v>75</v>
       </c>
       <c r="F185" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G185" s="12" t="n">
-        <v>30004</v>
+        <v>30003</v>
       </c>
       <c r="H185" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I185" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="12" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B186" s="12" t="s">
         <v>75</v>
@@ -11834,21 +11836,21 @@
         <v>75</v>
       </c>
       <c r="F186" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G186" s="12" t="n">
-        <v>30005</v>
+        <v>30004</v>
       </c>
       <c r="H186" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I186" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="12" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B187" s="12" t="s">
         <v>75</v>
@@ -11863,21 +11865,21 @@
         <v>75</v>
       </c>
       <c r="F187" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G187" s="12" t="n">
-        <v>30006</v>
+        <v>30005</v>
       </c>
       <c r="H187" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I187" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="12" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B188" s="12" t="s">
         <v>75</v>
@@ -11892,21 +11894,21 @@
         <v>75</v>
       </c>
       <c r="F188" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G188" s="12" t="n">
-        <v>40001</v>
+        <v>30006</v>
       </c>
       <c r="H188" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I188" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="12" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B189" s="12" t="s">
         <v>75</v>
@@ -11921,21 +11923,21 @@
         <v>75</v>
       </c>
       <c r="F189" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G189" s="12" t="n">
-        <v>60001</v>
+        <v>40001</v>
       </c>
       <c r="H189" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I189" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="12" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B190" s="12" t="s">
         <v>75</v>
@@ -11950,21 +11952,21 @@
         <v>75</v>
       </c>
       <c r="F190" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G190" s="12" t="n">
-        <v>60002</v>
+        <v>60001</v>
       </c>
       <c r="H190" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I190" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="12" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B191" s="12" t="s">
         <v>75</v>
@@ -11979,21 +11981,21 @@
         <v>75</v>
       </c>
       <c r="F191" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G191" s="12" t="n">
-        <v>60003</v>
+        <v>60002</v>
       </c>
       <c r="H191" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I191" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="12" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B192" s="12" t="s">
         <v>75</v>
@@ -12008,21 +12010,21 @@
         <v>75</v>
       </c>
       <c r="F192" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G192" s="12" t="n">
-        <v>60004</v>
+        <v>60003</v>
       </c>
       <c r="H192" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I192" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="12" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B193" s="12" t="s">
         <v>75</v>
@@ -12037,21 +12039,21 @@
         <v>75</v>
       </c>
       <c r="F193" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G193" s="12" t="n">
-        <v>60005</v>
+        <v>60004</v>
       </c>
       <c r="H193" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I193" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B194" s="12" t="s">
         <v>75</v>
@@ -12066,21 +12068,21 @@
         <v>75</v>
       </c>
       <c r="F194" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G194" s="12" t="n">
-        <v>60006</v>
+        <v>60005</v>
       </c>
       <c r="H194" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I194" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B195" s="12" t="s">
         <v>75</v>
@@ -12095,21 +12097,21 @@
         <v>75</v>
       </c>
       <c r="F195" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G195" s="12" t="n">
-        <v>60007</v>
+        <v>60006</v>
       </c>
       <c r="H195" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I195" s="12" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B196" s="12" t="s">
         <v>75</v>
@@ -12124,113 +12126,113 @@
         <v>75</v>
       </c>
       <c r="F196" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G196" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H196" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I196" s="12" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A197" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="B197" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C197" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D197" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E197" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F197" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="G197" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H196" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I196" s="12" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A197" s="3" t="s">
+      <c r="H197" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I197" s="12" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A198" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B197" s="4" t="s">
+      <c r="B198" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C197" s="4" t="s">
+      <c r="C198" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D197" s="3" t="s">
+      <c r="D198" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E197" s="4" t="s">
+      <c r="E198" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F197" s="3" t="s">
+      <c r="F198" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G197" s="4" t="s">
+      <c r="G198" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H197" s="4" t="s">
+      <c r="H198" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I197" s="3" t="s">
+      <c r="I198" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A198" s="3"/>
-      <c r="B198" s="4" t="s">
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="3"/>
+      <c r="B199" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C198" s="4" t="s">
+      <c r="C199" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D198" s="3"/>
-      <c r="E198" s="4" t="s">
+      <c r="D199" s="3"/>
+      <c r="E199" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F198" s="3"/>
-      <c r="G198" s="4" t="s">
+      <c r="F199" s="3"/>
+      <c r="G199" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H198" s="4" t="s">
+      <c r="H199" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I198" s="3"/>
-    </row>
-    <row r="199" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A199" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="B199" s="5"/>
-      <c r="C199" s="5"/>
-      <c r="D199" s="5"/>
-      <c r="E199" s="5"/>
-      <c r="F199" s="5"/>
-      <c r="G199" s="5"/>
-      <c r="H199" s="5"/>
-      <c r="I199" s="5"/>
-    </row>
-    <row r="200" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A200" s="12" t="s">
-        <v>328</v>
-      </c>
-      <c r="B200" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C200" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D200" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E200" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F200" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="G200" s="12" t="n">
-        <v>30001</v>
-      </c>
-      <c r="H200" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I200" s="12" t="s">
-        <v>344</v>
-      </c>
+      <c r="I199" s="3"/>
+    </row>
+    <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A200" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="B200" s="5"/>
+      <c r="C200" s="5"/>
+      <c r="D200" s="5"/>
+      <c r="E200" s="5"/>
+      <c r="F200" s="5"/>
+      <c r="G200" s="5"/>
+      <c r="H200" s="5"/>
+      <c r="I200" s="5"/>
     </row>
     <row r="201" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="12" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B201" s="12" t="s">
         <v>75</v>
@@ -12245,21 +12247,21 @@
         <v>75</v>
       </c>
       <c r="F201" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G201" s="12" t="n">
-        <v>30002</v>
+        <v>30001</v>
       </c>
       <c r="H201" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I201" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="12" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B202" s="12" t="s">
         <v>75</v>
@@ -12274,21 +12276,21 @@
         <v>75</v>
       </c>
       <c r="F202" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G202" s="12" t="n">
-        <v>30003</v>
+        <v>30002</v>
       </c>
       <c r="H202" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I202" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="12" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B203" s="12" t="s">
         <v>75</v>
@@ -12303,21 +12305,21 @@
         <v>75</v>
       </c>
       <c r="F203" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G203" s="12" t="n">
-        <v>30004</v>
+        <v>30003</v>
       </c>
       <c r="H203" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I203" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="12" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B204" s="12" t="s">
         <v>75</v>
@@ -12332,21 +12334,21 @@
         <v>75</v>
       </c>
       <c r="F204" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G204" s="12" t="n">
-        <v>30005</v>
+        <v>30004</v>
       </c>
       <c r="H204" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I204" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="12" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B205" s="12" t="s">
         <v>75</v>
@@ -12361,79 +12363,79 @@
         <v>75</v>
       </c>
       <c r="F205" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G205" s="12" t="n">
+        <v>30005</v>
+      </c>
+      <c r="H205" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I205" s="12" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="206" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="B206" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C206" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D206" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E206" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F206" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="G206" s="12" t="n">
         <v>30006</v>
       </c>
-      <c r="H205" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I205" s="12" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A206" s="12" t="s">
-        <v>334</v>
-      </c>
-      <c r="B206" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C206" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D206" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E206" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F206" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="G206" s="12" t="n">
+      <c r="H206" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I206" s="12" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A207" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="B207" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C207" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D207" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E207" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F207" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="G207" s="12" t="n">
         <v>40001</v>
       </c>
-      <c r="H206" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I206" s="12" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="207" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A207" s="12" t="s">
-        <v>345</v>
-      </c>
-      <c r="B207" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C207" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D207" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E207" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F207" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="G207" s="12" t="n">
-        <v>45001</v>
-      </c>
       <c r="H207" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I207" s="12" t="s">
-        <v>344</v>
+        <v>323</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="B208" s="12" t="s">
         <v>75</v>
@@ -12448,21 +12450,21 @@
         <v>75</v>
       </c>
       <c r="F208" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G208" s="12" t="n">
-        <v>60001</v>
+        <v>45001</v>
       </c>
       <c r="H208" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I208" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B209" s="12" t="s">
         <v>75</v>
@@ -12477,21 +12479,21 @@
         <v>75</v>
       </c>
       <c r="F209" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G209" s="12" t="n">
-        <v>60002</v>
+        <v>60001</v>
       </c>
       <c r="H209" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I209" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B210" s="12" t="s">
         <v>75</v>
@@ -12506,21 +12508,21 @@
         <v>75</v>
       </c>
       <c r="F210" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G210" s="12" t="n">
-        <v>60003</v>
+        <v>60002</v>
       </c>
       <c r="H210" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B211" s="12" t="s">
         <v>75</v>
@@ -12535,21 +12537,21 @@
         <v>75</v>
       </c>
       <c r="F211" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G211" s="12" t="n">
-        <v>60004</v>
+        <v>60003</v>
       </c>
       <c r="H211" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I211" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="12" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B212" s="12" t="s">
         <v>75</v>
@@ -12564,21 +12566,21 @@
         <v>75</v>
       </c>
       <c r="F212" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G212" s="12" t="n">
-        <v>60005</v>
+        <v>60004</v>
       </c>
       <c r="H212" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I212" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B213" s="12" t="s">
         <v>75</v>
@@ -12593,21 +12595,21 @@
         <v>75</v>
       </c>
       <c r="F213" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G213" s="12" t="n">
-        <v>60006</v>
+        <v>60005</v>
       </c>
       <c r="H213" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I213" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B214" s="12" t="s">
         <v>75</v>
@@ -12622,21 +12624,21 @@
         <v>75</v>
       </c>
       <c r="F214" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G214" s="12" t="n">
-        <v>60007</v>
+        <v>60006</v>
       </c>
       <c r="H214" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I214" s="12" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B215" s="12" t="s">
         <v>75</v>
@@ -12651,113 +12653,113 @@
         <v>75</v>
       </c>
       <c r="F215" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="G215" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H215" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I215" s="12" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="B216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C216" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E216" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F216" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="G216" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H215" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I215" s="12" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A216" s="3" t="s">
+      <c r="H216" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I216" s="12" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A217" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B216" s="4" t="s">
+      <c r="B217" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C216" s="4" t="s">
+      <c r="C217" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D216" s="3" t="s">
+      <c r="D217" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E216" s="4" t="s">
+      <c r="E217" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F216" s="3" t="s">
+      <c r="F217" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G216" s="4" t="s">
+      <c r="G217" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H216" s="4" t="s">
+      <c r="H217" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I216" s="3" t="s">
+      <c r="I217" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A217" s="3"/>
-      <c r="B217" s="4" t="s">
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="3"/>
+      <c r="B218" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C217" s="4" t="s">
+      <c r="C218" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D217" s="3"/>
-      <c r="E217" s="4" t="s">
+      <c r="D218" s="3"/>
+      <c r="E218" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F217" s="3"/>
-      <c r="G217" s="4" t="s">
+      <c r="F218" s="3"/>
+      <c r="G218" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H217" s="4" t="s">
+      <c r="H218" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I217" s="3"/>
-    </row>
-    <row r="218" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A218" s="5" t="s">
+      <c r="I218" s="3"/>
+    </row>
+    <row r="219" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A219" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="B218" s="5"/>
-      <c r="C218" s="5"/>
-      <c r="D218" s="5"/>
-      <c r="E218" s="5"/>
-      <c r="F218" s="5"/>
-      <c r="G218" s="5"/>
-      <c r="H218" s="5"/>
-      <c r="I218" s="5"/>
-    </row>
-    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A219" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B219" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C219" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D219" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E219" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F219" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G219" s="10" t="s">
-        <v>303</v>
-      </c>
-      <c r="H219" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I219" s="7" t="s">
-        <v>112</v>
-      </c>
+      <c r="B219" s="5"/>
+      <c r="C219" s="5"/>
+      <c r="D219" s="5"/>
+      <c r="E219" s="5"/>
+      <c r="F219" s="5"/>
+      <c r="G219" s="5"/>
+      <c r="H219" s="5"/>
+      <c r="I219" s="5"/>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="9" t="s">
-        <v>187</v>
+        <v>108</v>
       </c>
       <c r="B220" s="7" t="s">
         <v>109</v>
@@ -12775,21 +12777,21 @@
         <v>26</v>
       </c>
       <c r="G220" s="10" t="s">
-        <v>188</v>
+        <v>303</v>
       </c>
       <c r="H220" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I220" s="7" t="s">
-        <v>189</v>
+        <v>112</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="9" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="B221" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C221" s="7" t="s">
         <v>110</v>
@@ -12804,16 +12806,18 @@
         <v>26</v>
       </c>
       <c r="G221" s="10" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="H221" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I221" s="7"/>
+      <c r="I221" s="7" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B222" s="7" t="s">
         <v>24</v>
@@ -12831,7 +12835,7 @@
         <v>26</v>
       </c>
       <c r="G222" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H222" s="7" t="n">
         <v>2</v>
@@ -12840,7 +12844,7 @@
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="9" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B223" s="7" t="s">
         <v>24</v>
@@ -12858,7 +12862,7 @@
         <v>26</v>
       </c>
       <c r="G223" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H223" s="7" t="n">
         <v>2</v>
@@ -12867,7 +12871,7 @@
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B224" s="7" t="s">
         <v>24</v>
@@ -12885,7 +12889,7 @@
         <v>26</v>
       </c>
       <c r="G224" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="H224" s="7" t="n">
         <v>2</v>
@@ -12894,10 +12898,10 @@
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="9" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B225" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C225" s="7" t="s">
         <v>110</v>
@@ -12912,7 +12916,7 @@
         <v>26</v>
       </c>
       <c r="G225" s="10" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H225" s="7" t="n">
         <v>2</v>
@@ -12921,7 +12925,7 @@
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="9" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B226" s="7" t="s">
         <v>109</v>
@@ -12939,7 +12943,7 @@
         <v>26</v>
       </c>
       <c r="G226" s="10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H226" s="7" t="n">
         <v>2</v>
@@ -12948,10 +12952,10 @@
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="9" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B227" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C227" s="7" t="s">
         <v>110</v>
@@ -12966,7 +12970,7 @@
         <v>26</v>
       </c>
       <c r="G227" s="10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="H227" s="7" t="n">
         <v>2</v>
@@ -12975,7 +12979,7 @@
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B228" s="7" t="s">
         <v>24</v>
@@ -12993,7 +12997,7 @@
         <v>26</v>
       </c>
       <c r="G228" s="10" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H228" s="7" t="n">
         <v>2</v>
@@ -13002,7 +13006,7 @@
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B229" s="7" t="s">
         <v>24</v>
@@ -13020,7 +13024,7 @@
         <v>26</v>
       </c>
       <c r="G229" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="H229" s="7" t="n">
         <v>2</v>
@@ -13029,7 +13033,7 @@
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B230" s="7" t="s">
         <v>24</v>
@@ -13047,7 +13051,7 @@
         <v>26</v>
       </c>
       <c r="G230" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H230" s="7" t="n">
         <v>2</v>
@@ -13056,10 +13060,10 @@
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="9" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B231" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C231" s="7" t="s">
         <v>110</v>
@@ -13074,7 +13078,7 @@
         <v>26</v>
       </c>
       <c r="G231" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="H231" s="7" t="n">
         <v>2</v>
@@ -13083,7 +13087,7 @@
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B232" s="7" t="s">
         <v>109</v>
@@ -13101,7 +13105,7 @@
         <v>26</v>
       </c>
       <c r="G232" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="H232" s="7" t="n">
         <v>2</v>
@@ -13110,10 +13114,10 @@
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B233" s="7" t="s">
-        <v>222</v>
+        <v>109</v>
       </c>
       <c r="C233" s="7" t="s">
         <v>110</v>
@@ -13128,7 +13132,7 @@
         <v>26</v>
       </c>
       <c r="G233" s="10" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="H233" s="7" t="n">
         <v>2</v>
@@ -13137,7 +13141,7 @@
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B234" s="7" t="s">
         <v>222</v>
@@ -13155,7 +13159,7 @@
         <v>26</v>
       </c>
       <c r="G234" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H234" s="7" t="n">
         <v>2</v>
@@ -13164,10 +13168,10 @@
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="9" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B235" s="7" t="s">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="C235" s="7" t="s">
         <v>110</v>
@@ -13182,7 +13186,7 @@
         <v>26</v>
       </c>
       <c r="G235" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H235" s="7" t="n">
         <v>2</v>
@@ -13191,7 +13195,7 @@
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="9" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B236" s="7" t="s">
         <v>195</v>
@@ -13209,7 +13213,7 @@
         <v>26</v>
       </c>
       <c r="G236" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H236" s="7" t="n">
         <v>2</v>
@@ -13218,10 +13222,10 @@
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="9" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B237" s="7" t="s">
-        <v>109</v>
+        <v>195</v>
       </c>
       <c r="C237" s="7" t="s">
         <v>110</v>
@@ -13236,7 +13240,7 @@
         <v>26</v>
       </c>
       <c r="G237" s="10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H237" s="7" t="n">
         <v>2</v>
@@ -13245,7 +13249,7 @@
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="9" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B238" s="7" t="s">
         <v>109</v>
@@ -13263,7 +13267,7 @@
         <v>26</v>
       </c>
       <c r="G238" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H238" s="7" t="n">
         <v>2</v>
@@ -13271,11 +13275,11 @@
       <c r="I238" s="7"/>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A239" s="7" t="s">
-        <v>304</v>
+      <c r="A239" s="9" t="s">
+        <v>232</v>
       </c>
       <c r="B239" s="7" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C239" s="7" t="s">
         <v>110</v>
@@ -13290,18 +13294,16 @@
         <v>26</v>
       </c>
       <c r="G239" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H239" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I239" s="7" t="s">
-        <v>236</v>
-      </c>
+      <c r="I239" s="7"/>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="7" t="s">
-        <v>237</v>
+        <v>304</v>
       </c>
       <c r="B240" s="7" t="s">
         <v>75</v>
@@ -13319,47 +13321,47 @@
         <v>26</v>
       </c>
       <c r="G240" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="H240" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I240" s="7" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A241" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B241" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C241" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D241" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E241" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F241" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G241" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="H240" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I240" s="7" t="s">
+      <c r="H241" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I241" s="7" t="s">
         <v>239</v>
-      </c>
-    </row>
-    <row r="241" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A241" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="B241" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C241" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D241" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E241" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F241" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G241" s="12" t="s">
-        <v>241</v>
-      </c>
-      <c r="H241" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I241" s="12" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="242" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="12" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B242" s="12" t="s">
         <v>75</v>
@@ -13377,18 +13379,18 @@
         <v>26</v>
       </c>
       <c r="G242" s="12" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H242" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I242" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="243" customFormat="false" ht="45.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A243" s="11" t="s">
-        <v>308</v>
+        <v>349</v>
+      </c>
+    </row>
+    <row r="243" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="12" t="s">
+        <v>242</v>
       </c>
       <c r="B243" s="12" t="s">
         <v>75</v>
@@ -13405,19 +13407,19 @@
       <c r="F243" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="G243" s="13" t="s">
-        <v>309</v>
+      <c r="G243" s="12" t="s">
+        <v>243</v>
       </c>
       <c r="H243" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I243" s="12" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="244" customFormat="false" ht="36.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="244" customFormat="false" ht="45.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="11" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B244" s="12" t="s">
         <v>75</v>
@@ -13435,18 +13437,18 @@
         <v>26</v>
       </c>
       <c r="G244" s="13" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="H244" s="12" t="n">
         <v>2</v>
       </c>
       <c r="I244" s="12" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="245" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="245" customFormat="false" ht="36.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="11" t="s">
-        <v>350</v>
+        <v>311</v>
       </c>
       <c r="B245" s="12" t="s">
         <v>75</v>
@@ -13464,16 +13466,73 @@
         <v>26</v>
       </c>
       <c r="G245" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="H245" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I245" s="12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="246" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="11" t="s">
+        <v>353</v>
+      </c>
+      <c r="B246" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C246" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D246" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E246" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F246" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G246" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="H245" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I245" s="12" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="1048557" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="H246" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I246" s="12" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="247" customFormat="false" ht="28.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="B247" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C247" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D247" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E247" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F247" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G247" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="H247" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I247" s="12" t="s">
+        <v>319</v>
+      </c>
+    </row>
     <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -13500,26 +13559,26 @@
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A115:A116"/>
-    <mergeCell ref="D115:D116"/>
-    <mergeCell ref="F115:F116"/>
-    <mergeCell ref="I115:I116"/>
-    <mergeCell ref="A117:I117"/>
-    <mergeCell ref="A171:A172"/>
-    <mergeCell ref="D171:D172"/>
-    <mergeCell ref="F171:F172"/>
-    <mergeCell ref="I171:I172"/>
-    <mergeCell ref="A173:I173"/>
-    <mergeCell ref="A197:A198"/>
-    <mergeCell ref="D197:D198"/>
-    <mergeCell ref="F197:F198"/>
-    <mergeCell ref="I197:I198"/>
-    <mergeCell ref="A199:I199"/>
-    <mergeCell ref="A216:A217"/>
-    <mergeCell ref="D216:D217"/>
-    <mergeCell ref="F216:F217"/>
-    <mergeCell ref="I216:I217"/>
-    <mergeCell ref="A218:I218"/>
+    <mergeCell ref="A116:A117"/>
+    <mergeCell ref="D116:D117"/>
+    <mergeCell ref="F116:F117"/>
+    <mergeCell ref="I116:I117"/>
+    <mergeCell ref="A118:I118"/>
+    <mergeCell ref="A172:A173"/>
+    <mergeCell ref="D172:D173"/>
+    <mergeCell ref="F172:F173"/>
+    <mergeCell ref="I172:I173"/>
+    <mergeCell ref="A174:I174"/>
+    <mergeCell ref="A198:A199"/>
+    <mergeCell ref="D198:D199"/>
+    <mergeCell ref="F198:F199"/>
+    <mergeCell ref="I198:I199"/>
+    <mergeCell ref="A200:I200"/>
+    <mergeCell ref="A217:A218"/>
+    <mergeCell ref="D217:D218"/>
+    <mergeCell ref="F217:F218"/>
+    <mergeCell ref="I217:I218"/>
+    <mergeCell ref="A219:I219"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13539,15 +13598,15 @@
   <dimension ref="A1:I29"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="18.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="40.86"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13555,7 +13614,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13563,7 +13622,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13584,436 +13643,436 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="16" t="s">
+      <c r="D7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="F7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="16" t="s">
+      <c r="H7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="I7" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16" t="s">
+      <c r="D8" s="4"/>
+      <c r="E8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16" t="s">
+      <c r="F8" s="4"/>
+      <c r="G8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="16" t="s">
+      <c r="H8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="16"/>
+      <c r="I8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>356</v>
-      </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
+      <c r="A9" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>357</v>
-      </c>
-      <c r="B10" s="18" t="s">
+      <c r="A10" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="G10" s="18" t="s">
-        <v>358</v>
-      </c>
-      <c r="H10" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I10" s="18" t="s">
-        <v>359</v>
+      <c r="C10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>360</v>
-      </c>
-      <c r="B11" s="18" t="s">
+      <c r="A11" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E11" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="18" t="s">
-        <v>361</v>
-      </c>
-      <c r="H11" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I11" s="18" t="s">
-        <v>362</v>
+      <c r="C11" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="B12" s="18" t="s">
+      <c r="A12" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E12" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12" s="18" t="s">
-        <v>364</v>
-      </c>
-      <c r="H12" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I12" s="18" t="s">
-        <v>365</v>
+      <c r="C12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="s">
-        <v>366</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C13" s="18" t="s">
+      <c r="A13" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D13" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="18" t="s">
-        <v>367</v>
-      </c>
-      <c r="H13" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I13" s="18" t="s">
-        <v>368</v>
+      <c r="D13" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>371</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C14" s="18" t="s">
+      <c r="A14" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D14" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="G14" s="18" t="s">
-        <v>369</v>
-      </c>
-      <c r="H14" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I14" s="18" t="s">
-        <v>370</v>
+      <c r="D14" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" s="18" t="s">
+      <c r="A15" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D15" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E15" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="G15" s="18" t="s">
-        <v>371</v>
-      </c>
-      <c r="H15" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I15" s="18" t="s">
-        <v>370</v>
+      <c r="D15" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C16" s="18" t="s">
+      <c r="A16" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D16" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16" s="18" t="s">
-        <v>372</v>
-      </c>
-      <c r="H16" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I16" s="18" t="s">
-        <v>370</v>
+      <c r="D16" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
-        <v>323</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" s="18" t="s">
+      <c r="A17" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D17" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E17" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="G17" s="18" t="s">
+      <c r="D17" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" s="7" t="s">
         <v>373</v>
       </c>
-      <c r="H17" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="I17" s="18" t="s">
-        <v>370</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
-        <v>374</v>
-      </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
+      <c r="A20" s="16" t="s">
+        <v>377</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
-        <v>375</v>
-      </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
+      <c r="A21" s="17" t="s">
+        <v>378</v>
+      </c>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>376</v>
-      </c>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
+      <c r="A22" s="17" t="s">
+        <v>379</v>
+      </c>
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
-        <v>377</v>
-      </c>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
+      <c r="A23" s="17" t="s">
+        <v>380</v>
+      </c>
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="s">
-        <v>378</v>
-      </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
+      <c r="A24" s="17" t="s">
+        <v>381</v>
+      </c>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
-        <v>379</v>
-      </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
+      <c r="A25" s="17" t="s">
+        <v>382</v>
+      </c>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="s">
-        <v>380</v>
-      </c>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
+      <c r="A26" s="17" t="s">
+        <v>383</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="s">
-        <v>381</v>
-      </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
+      <c r="A27" s="17" t="s">
+        <v>384</v>
+      </c>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="s">
-        <v>382</v>
-      </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
+      <c r="A28" s="17" t="s">
+        <v>385</v>
+      </c>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
-        <v>383</v>
-      </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="19"/>
+      <c r="A29" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="15">

</xml_diff>

<commit_message>
SOCO: Feature: Don't report under-voltage on phase loss
When there is a phase loss, the customer doesn't want the "under-voltage" flag
to be set.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2450" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2498" uniqueCount="397">
   <si>
     <t xml:space="preserve">Controller:</t>
   </si>
@@ -937,6 +937,15 @@
   </si>
   <si>
     <t xml:space="preserve">DG Detection Enable/Disable Setting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firmware Upgrade Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0: No Firmware Upgrade Ongoing/Firmware Upgrade completed, 1:Firmware Uploading Ongoing, 2: Firmware Updating Ongoing, 127: Error Occured</t>
   </si>
   <si>
     <t xml:space="preserve">Switch Pressed</t>
@@ -1003,6 +1012,24 @@
 Used to store a temporarily value. Resets when SOCO restarts on POR.</t>
   </si>
   <si>
+    <t xml:space="preserve">Grid R Phase Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grid Y Phase Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grid B Phase Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solar R Phase Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solar Y Phase Loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solar B Phase Loss</t>
+  </si>
+  <si>
     <t xml:space="preserve">READ COIL STATUS (Function Code: 0x01)</t>
   </si>
   <si>
@@ -1089,6 +1116,9 @@
   </si>
   <si>
     <t xml:space="preserve">Restart Controller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0: No Action, 1:Signals start of Firmware Uploading, 2: Signals end of Firmware Uploading</t>
   </si>
   <si>
     <t xml:space="preserve">Internal Only. Not visible to customer. 
@@ -9717,65 +9747,67 @@
         <v>239</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="86.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A108" s="11" t="s">
+    <row r="108" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="B108" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C108" s="12" t="s">
+      <c r="B108" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C108" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D108" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E108" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F108" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G108" s="13" t="s">
+      <c r="D108" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E108" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G108" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="H108" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I108" s="12" t="s">
+      <c r="H108" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I108" s="7" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="B109" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C109" s="7" t="s">
+    <row r="109" customFormat="false" ht="86.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="B109" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C109" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D109" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E109" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F109" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G109" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="H109" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I109" s="7"/>
+      <c r="D109" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E109" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G109" s="13" t="s">
+        <v>309</v>
+      </c>
+      <c r="H109" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I109" s="12" t="s">
+        <v>310</v>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="7" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B110" s="7" t="s">
         <v>75</v>
@@ -9793,7 +9825,7 @@
         <v>26</v>
       </c>
       <c r="G110" s="7" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H110" s="7" t="n">
         <v>2</v>
@@ -9802,7 +9834,7 @@
     </row>
     <row r="111" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B111" s="7" t="s">
         <v>75</v>
@@ -9814,47 +9846,45 @@
         <v>4</v>
       </c>
       <c r="E111" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G111" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="H111" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I111" s="7"/>
+    </row>
+    <row r="112" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A112" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="B112" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C112" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D112" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E112" s="7" t="n">
         <v>0.01</v>
       </c>
-      <c r="F111" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G111" s="7" t="s">
+      <c r="F112" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G112" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="H111" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I111" s="7"/>
-    </row>
-    <row r="112" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A112" s="11" t="s">
-        <v>308</v>
-      </c>
-      <c r="B112" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C112" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D112" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E112" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F112" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G112" s="13" t="s">
-        <v>309</v>
-      </c>
-      <c r="H112" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I112" s="12" t="s">
-        <v>310</v>
-      </c>
+      <c r="H112" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I112" s="7"/>
     </row>
     <row r="113" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
@@ -9885,7 +9915,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="236.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="47.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="11" t="s">
         <v>314</v>
       </c>
@@ -9914,7 +9944,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="36.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="236.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
         <v>317</v>
       </c>
@@ -9943,99 +9973,101 @@
         <v>319</v>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A116" s="3" t="s">
+    <row r="116" customFormat="false" ht="36.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A116" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="B116" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C116" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="D116" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E116" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G116" s="13" t="s">
+        <v>321</v>
+      </c>
+      <c r="H116" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I116" s="12" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A117" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B116" s="4" t="s">
+      <c r="B117" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C116" s="4" t="s">
+      <c r="C117" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D116" s="3" t="s">
+      <c r="D117" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E116" s="4" t="s">
+      <c r="E117" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F116" s="3" t="s">
+      <c r="F117" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G116" s="4" t="s">
+      <c r="G117" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H116" s="4" t="s">
+      <c r="H117" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I116" s="3" t="s">
+      <c r="I117" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="3"/>
-      <c r="B117" s="4" t="s">
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="3"/>
+      <c r="B118" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C117" s="4" t="s">
+      <c r="C118" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D117" s="3"/>
-      <c r="E117" s="4" t="s">
+      <c r="D118" s="3"/>
+      <c r="E118" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F117" s="3"/>
-      <c r="G117" s="4" t="s">
+      <c r="F118" s="3"/>
+      <c r="G118" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H117" s="4" t="s">
+      <c r="H118" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I117" s="3"/>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A118" s="5" t="s">
+      <c r="I118" s="3"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A119" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="B118" s="5"/>
-      <c r="C118" s="5"/>
-      <c r="D118" s="5"/>
-      <c r="E118" s="5"/>
-      <c r="F118" s="5"/>
-      <c r="G118" s="5"/>
-      <c r="H118" s="5"/>
-      <c r="I118" s="5"/>
-    </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="B119" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="C119" s="7" t="s">
-        <v>248</v>
-      </c>
-      <c r="D119" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E119" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F119" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="G119" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H119" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I119" s="7"/>
+      <c r="B119" s="5"/>
+      <c r="C119" s="5"/>
+      <c r="D119" s="5"/>
+      <c r="E119" s="5"/>
+      <c r="F119" s="5"/>
+      <c r="G119" s="5"/>
+      <c r="H119" s="5"/>
+      <c r="I119" s="5"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="7" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B120" s="7" t="s">
         <v>75</v>
@@ -10053,7 +10085,7 @@
         <v>249</v>
       </c>
       <c r="G120" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H120" s="7" t="n">
         <v>1</v>
@@ -10062,7 +10094,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B121" s="7" t="s">
         <v>75</v>
@@ -10080,7 +10112,7 @@
         <v>249</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H121" s="7" t="n">
         <v>1</v>
@@ -10089,7 +10121,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B122" s="7" t="s">
         <v>75</v>
@@ -10107,7 +10139,7 @@
         <v>249</v>
       </c>
       <c r="G122" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H122" s="7" t="n">
         <v>1</v>
@@ -10116,7 +10148,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B123" s="7" t="s">
         <v>75</v>
@@ -10134,7 +10166,7 @@
         <v>249</v>
       </c>
       <c r="G123" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H123" s="7" t="n">
         <v>1</v>
@@ -10143,7 +10175,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B124" s="7" t="s">
         <v>75</v>
@@ -10161,7 +10193,7 @@
         <v>249</v>
       </c>
       <c r="G124" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H124" s="7" t="n">
         <v>1</v>
@@ -10170,7 +10202,7 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B125" s="7" t="s">
         <v>75</v>
@@ -10188,7 +10220,7 @@
         <v>249</v>
       </c>
       <c r="G125" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H125" s="7" t="n">
         <v>1</v>
@@ -10197,7 +10229,7 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B126" s="7" t="s">
         <v>75</v>
@@ -10215,7 +10247,7 @@
         <v>249</v>
       </c>
       <c r="G126" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H126" s="7" t="n">
         <v>1</v>
@@ -10224,7 +10256,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B127" s="7" t="s">
         <v>75</v>
@@ -10242,7 +10274,7 @@
         <v>249</v>
       </c>
       <c r="G127" s="7" t="n">
-        <v>201</v>
+        <v>8</v>
       </c>
       <c r="H127" s="7" t="n">
         <v>1</v>
@@ -10251,7 +10283,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B128" s="7" t="s">
         <v>75</v>
@@ -10269,7 +10301,7 @@
         <v>249</v>
       </c>
       <c r="G128" s="7" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H128" s="7" t="n">
         <v>1</v>
@@ -10278,7 +10310,7 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B129" s="7" t="s">
         <v>75</v>
@@ -10296,7 +10328,7 @@
         <v>249</v>
       </c>
       <c r="G129" s="7" t="n">
-        <v>301</v>
+        <v>202</v>
       </c>
       <c r="H129" s="7" t="n">
         <v>1</v>
@@ -10305,7 +10337,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="7" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B130" s="7" t="s">
         <v>75</v>
@@ -10323,7 +10355,7 @@
         <v>249</v>
       </c>
       <c r="G130" s="7" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H130" s="7" t="n">
         <v>1</v>
@@ -10332,7 +10364,7 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="7" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B131" s="7" t="s">
         <v>75</v>
@@ -10350,7 +10382,7 @@
         <v>249</v>
       </c>
       <c r="G131" s="7" t="n">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H131" s="7" t="n">
         <v>1</v>
@@ -10359,7 +10391,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="7" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B132" s="7" t="s">
         <v>75</v>
@@ -10377,7 +10409,7 @@
         <v>249</v>
       </c>
       <c r="G132" s="7" t="n">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H132" s="7" t="n">
         <v>1</v>
@@ -10386,7 +10418,7 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="7" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B133" s="7" t="s">
         <v>75</v>
@@ -10404,7 +10436,7 @@
         <v>249</v>
       </c>
       <c r="G133" s="7" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H133" s="7" t="n">
         <v>1</v>
@@ -10413,7 +10445,7 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B134" s="7" t="s">
         <v>75</v>
@@ -10431,7 +10463,7 @@
         <v>249</v>
       </c>
       <c r="G134" s="7" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H134" s="7" t="n">
         <v>1</v>
@@ -10440,7 +10472,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B135" s="7" t="s">
         <v>75</v>
@@ -10458,7 +10490,7 @@
         <v>249</v>
       </c>
       <c r="G135" s="7" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H135" s="7" t="n">
         <v>1</v>
@@ -10467,7 +10499,7 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="7" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B136" s="7" t="s">
         <v>75</v>
@@ -10485,7 +10517,7 @@
         <v>249</v>
       </c>
       <c r="G136" s="7" t="n">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="H136" s="7" t="n">
         <v>1</v>
@@ -10494,7 +10526,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B137" s="7" t="s">
         <v>75</v>
@@ -10512,7 +10544,7 @@
         <v>249</v>
       </c>
       <c r="G137" s="7" t="n">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H137" s="7" t="n">
         <v>1</v>
@@ -10521,7 +10553,7 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B138" s="7" t="s">
         <v>75</v>
@@ -10539,7 +10571,7 @@
         <v>249</v>
       </c>
       <c r="G138" s="7" t="n">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="H138" s="7" t="n">
         <v>1</v>
@@ -10548,7 +10580,7 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B139" s="7" t="s">
         <v>75</v>
@@ -10566,7 +10598,7 @@
         <v>249</v>
       </c>
       <c r="G139" s="7" t="n">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H139" s="7" t="n">
         <v>1</v>
@@ -10575,7 +10607,7 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B140" s="7" t="s">
         <v>75</v>
@@ -10593,7 +10625,7 @@
         <v>249</v>
       </c>
       <c r="G140" s="7" t="n">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H140" s="7" t="n">
         <v>1</v>
@@ -10602,7 +10634,7 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B141" s="7" t="s">
         <v>75</v>
@@ -10620,7 +10652,7 @@
         <v>249</v>
       </c>
       <c r="G141" s="7" t="n">
-        <v>401</v>
+        <v>312</v>
       </c>
       <c r="H141" s="7" t="n">
         <v>1</v>
@@ -10629,7 +10661,7 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="7" t="s">
-        <v>272</v>
+        <v>323</v>
       </c>
       <c r="B142" s="7" t="s">
         <v>75</v>
@@ -10647,7 +10679,7 @@
         <v>249</v>
       </c>
       <c r="G142" s="7" t="n">
-        <v>402</v>
+        <v>313</v>
       </c>
       <c r="H142" s="7" t="n">
         <v>1</v>
@@ -10656,7 +10688,7 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="7" t="s">
-        <v>273</v>
+        <v>324</v>
       </c>
       <c r="B143" s="7" t="s">
         <v>75</v>
@@ -10674,7 +10706,7 @@
         <v>249</v>
       </c>
       <c r="G143" s="7" t="n">
-        <v>403</v>
+        <v>314</v>
       </c>
       <c r="H143" s="7" t="n">
         <v>1</v>
@@ -10683,7 +10715,7 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="7" t="s">
-        <v>274</v>
+        <v>325</v>
       </c>
       <c r="B144" s="7" t="s">
         <v>75</v>
@@ -10701,7 +10733,7 @@
         <v>249</v>
       </c>
       <c r="G144" s="7" t="n">
-        <v>404</v>
+        <v>315</v>
       </c>
       <c r="H144" s="7" t="n">
         <v>1</v>
@@ -10710,7 +10742,7 @@
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="7" t="s">
-        <v>275</v>
+        <v>326</v>
       </c>
       <c r="B145" s="7" t="s">
         <v>75</v>
@@ -10728,7 +10760,7 @@
         <v>249</v>
       </c>
       <c r="G145" s="7" t="n">
-        <v>405</v>
+        <v>316</v>
       </c>
       <c r="H145" s="7" t="n">
         <v>1</v>
@@ -10737,7 +10769,7 @@
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="7" t="s">
-        <v>276</v>
+        <v>327</v>
       </c>
       <c r="B146" s="7" t="s">
         <v>75</v>
@@ -10755,7 +10787,7 @@
         <v>249</v>
       </c>
       <c r="G146" s="7" t="n">
-        <v>406</v>
+        <v>317</v>
       </c>
       <c r="H146" s="7" t="n">
         <v>1</v>
@@ -10764,7 +10796,7 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="7" t="s">
-        <v>277</v>
+        <v>328</v>
       </c>
       <c r="B147" s="7" t="s">
         <v>75</v>
@@ -10782,7 +10814,7 @@
         <v>249</v>
       </c>
       <c r="G147" s="7" t="n">
-        <v>601</v>
+        <v>318</v>
       </c>
       <c r="H147" s="7" t="n">
         <v>1</v>
@@ -10791,7 +10823,7 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="7" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="B148" s="7" t="s">
         <v>75</v>
@@ -10809,7 +10841,7 @@
         <v>249</v>
       </c>
       <c r="G148" s="7" t="n">
-        <v>602</v>
+        <v>401</v>
       </c>
       <c r="H148" s="7" t="n">
         <v>1</v>
@@ -10818,7 +10850,7 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="7" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="B149" s="7" t="s">
         <v>75</v>
@@ -10836,7 +10868,7 @@
         <v>249</v>
       </c>
       <c r="G149" s="7" t="n">
-        <v>603</v>
+        <v>402</v>
       </c>
       <c r="H149" s="7" t="n">
         <v>1</v>
@@ -10845,7 +10877,7 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="7" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="B150" s="7" t="s">
         <v>75</v>
@@ -10863,7 +10895,7 @@
         <v>249</v>
       </c>
       <c r="G150" s="7" t="n">
-        <v>604</v>
+        <v>403</v>
       </c>
       <c r="H150" s="7" t="n">
         <v>1</v>
@@ -10872,7 +10904,7 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="7" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="B151" s="7" t="s">
         <v>75</v>
@@ -10890,7 +10922,7 @@
         <v>249</v>
       </c>
       <c r="G151" s="7" t="n">
-        <v>605</v>
+        <v>404</v>
       </c>
       <c r="H151" s="7" t="n">
         <v>1</v>
@@ -10899,7 +10931,7 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="7" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="B152" s="7" t="s">
         <v>75</v>
@@ -10917,7 +10949,7 @@
         <v>249</v>
       </c>
       <c r="G152" s="7" t="n">
-        <v>606</v>
+        <v>405</v>
       </c>
       <c r="H152" s="7" t="n">
         <v>1</v>
@@ -10926,7 +10958,7 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="7" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="B153" s="7" t="s">
         <v>75</v>
@@ -10944,7 +10976,7 @@
         <v>249</v>
       </c>
       <c r="G153" s="7" t="n">
-        <v>607</v>
+        <v>406</v>
       </c>
       <c r="H153" s="7" t="n">
         <v>1</v>
@@ -10953,7 +10985,7 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="7" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="B154" s="7" t="s">
         <v>75</v>
@@ -10971,7 +11003,7 @@
         <v>249</v>
       </c>
       <c r="G154" s="7" t="n">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="H154" s="7" t="n">
         <v>1</v>
@@ -10980,7 +11012,7 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="7" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="B155" s="7" t="s">
         <v>75</v>
@@ -10998,7 +11030,7 @@
         <v>249</v>
       </c>
       <c r="G155" s="7" t="n">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="H155" s="7" t="n">
         <v>1</v>
@@ -11007,7 +11039,7 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="7" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="B156" s="7" t="s">
         <v>75</v>
@@ -11025,7 +11057,7 @@
         <v>249</v>
       </c>
       <c r="G156" s="7" t="n">
-        <v>610</v>
+        <v>603</v>
       </c>
       <c r="H156" s="7" t="n">
         <v>1</v>
@@ -11034,7 +11066,7 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="7" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="B157" s="7" t="s">
         <v>75</v>
@@ -11052,7 +11084,7 @@
         <v>249</v>
       </c>
       <c r="G157" s="7" t="n">
-        <v>611</v>
+        <v>604</v>
       </c>
       <c r="H157" s="7" t="n">
         <v>1</v>
@@ -11061,7 +11093,7 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="B158" s="7" t="s">
         <v>75</v>
@@ -11079,7 +11111,7 @@
         <v>249</v>
       </c>
       <c r="G158" s="7" t="n">
-        <v>612</v>
+        <v>605</v>
       </c>
       <c r="H158" s="7" t="n">
         <v>1</v>
@@ -11088,7 +11120,7 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="7" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="B159" s="7" t="s">
         <v>75</v>
@@ -11106,7 +11138,7 @@
         <v>249</v>
       </c>
       <c r="G159" s="7" t="n">
-        <v>801</v>
+        <v>606</v>
       </c>
       <c r="H159" s="7" t="n">
         <v>1</v>
@@ -11115,7 +11147,7 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="7" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="B160" s="7" t="s">
         <v>75</v>
@@ -11133,7 +11165,7 @@
         <v>249</v>
       </c>
       <c r="G160" s="7" t="n">
-        <v>802</v>
+        <v>607</v>
       </c>
       <c r="H160" s="7" t="n">
         <v>1</v>
@@ -11142,7 +11174,7 @@
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="7" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="B161" s="7" t="s">
         <v>75</v>
@@ -11160,7 +11192,7 @@
         <v>249</v>
       </c>
       <c r="G161" s="7" t="n">
-        <v>803</v>
+        <v>608</v>
       </c>
       <c r="H161" s="7" t="n">
         <v>1</v>
@@ -11169,7 +11201,7 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="7" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="B162" s="7" t="s">
         <v>75</v>
@@ -11187,7 +11219,7 @@
         <v>249</v>
       </c>
       <c r="G162" s="7" t="n">
-        <v>804</v>
+        <v>609</v>
       </c>
       <c r="H162" s="7" t="n">
         <v>1</v>
@@ -11196,7 +11228,7 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="7" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="B163" s="7" t="s">
         <v>75</v>
@@ -11214,7 +11246,7 @@
         <v>249</v>
       </c>
       <c r="G163" s="7" t="n">
-        <v>805</v>
+        <v>610</v>
       </c>
       <c r="H163" s="7" t="n">
         <v>1</v>
@@ -11223,7 +11255,7 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="7" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="B164" s="7" t="s">
         <v>75</v>
@@ -11241,7 +11273,7 @@
         <v>249</v>
       </c>
       <c r="G164" s="7" t="n">
-        <v>806</v>
+        <v>611</v>
       </c>
       <c r="H164" s="7" t="n">
         <v>1</v>
@@ -11250,7 +11282,7 @@
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="7" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="B165" s="7" t="s">
         <v>75</v>
@@ -11268,7 +11300,7 @@
         <v>249</v>
       </c>
       <c r="G165" s="7" t="n">
-        <v>807</v>
+        <v>612</v>
       </c>
       <c r="H165" s="7" t="n">
         <v>1</v>
@@ -11277,7 +11309,7 @@
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="7" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="B166" s="7" t="s">
         <v>75</v>
@@ -11295,7 +11327,7 @@
         <v>249</v>
       </c>
       <c r="G166" s="7" t="n">
-        <v>808</v>
+        <v>801</v>
       </c>
       <c r="H166" s="7" t="n">
         <v>1</v>
@@ -11304,7 +11336,7 @@
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="7" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="B167" s="7" t="s">
         <v>75</v>
@@ -11322,7 +11354,7 @@
         <v>249</v>
       </c>
       <c r="G167" s="7" t="n">
-        <v>809</v>
+        <v>802</v>
       </c>
       <c r="H167" s="7" t="n">
         <v>1</v>
@@ -11331,7 +11363,7 @@
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="7" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="B168" s="7" t="s">
         <v>75</v>
@@ -11349,7 +11381,7 @@
         <v>249</v>
       </c>
       <c r="G168" s="7" t="n">
-        <v>901</v>
+        <v>803</v>
       </c>
       <c r="H168" s="7" t="n">
         <v>1</v>
@@ -11358,7 +11390,7 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="7" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="B169" s="7" t="s">
         <v>75</v>
@@ -11376,7 +11408,7 @@
         <v>249</v>
       </c>
       <c r="G169" s="7" t="n">
-        <v>902</v>
+        <v>804</v>
       </c>
       <c r="H169" s="7" t="n">
         <v>1</v>
@@ -11385,7 +11417,7 @@
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="7" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="B170" s="7" t="s">
         <v>75</v>
@@ -11403,7 +11435,7 @@
         <v>249</v>
       </c>
       <c r="G170" s="7" t="n">
-        <v>903</v>
+        <v>805</v>
       </c>
       <c r="H170" s="7" t="n">
         <v>1</v>
@@ -11412,7 +11444,7 @@
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="7" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="B171" s="7" t="s">
         <v>75</v>
@@ -11430,278 +11462,264 @@
         <v>249</v>
       </c>
       <c r="G171" s="7" t="n">
+        <v>806</v>
+      </c>
+      <c r="H171" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I171" s="7"/>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="B172" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C172" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D172" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E172" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F172" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G172" s="7" t="n">
+        <v>807</v>
+      </c>
+      <c r="H172" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I172" s="7"/>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="B173" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C173" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D173" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E173" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F173" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G173" s="7" t="n">
+        <v>808</v>
+      </c>
+      <c r="H173" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I173" s="7"/>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="B174" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C174" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D174" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E174" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F174" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G174" s="7" t="n">
+        <v>809</v>
+      </c>
+      <c r="H174" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I174" s="7"/>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="B175" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C175" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D175" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E175" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F175" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G175" s="7" t="n">
+        <v>901</v>
+      </c>
+      <c r="H175" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I175" s="7"/>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="B176" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C176" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D176" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E176" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F176" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G176" s="7" t="n">
+        <v>902</v>
+      </c>
+      <c r="H176" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I176" s="7"/>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C177" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D177" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E177" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F177" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G177" s="7" t="n">
+        <v>903</v>
+      </c>
+      <c r="H177" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I177" s="7"/>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="B178" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C178" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="D178" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E178" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="F178" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G178" s="7" t="n">
         <v>904</v>
       </c>
-      <c r="H171" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I171" s="7"/>
-    </row>
-    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A172" s="3" t="s">
+      <c r="H178" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I178" s="7"/>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A179" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B172" s="4" t="s">
+      <c r="B179" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C172" s="4" t="s">
+      <c r="C179" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D172" s="3" t="s">
+      <c r="D179" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E172" s="4" t="s">
+      <c r="E179" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F172" s="3" t="s">
+      <c r="F179" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G172" s="4" t="s">
+      <c r="G179" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H172" s="4" t="s">
+      <c r="H179" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I172" s="3" t="s">
+      <c r="I179" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A173" s="3"/>
-      <c r="B173" s="4" t="s">
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="3"/>
+      <c r="B180" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C173" s="4" t="s">
+      <c r="C180" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D173" s="3"/>
-      <c r="E173" s="4" t="s">
+      <c r="D180" s="3"/>
+      <c r="E180" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F173" s="3"/>
-      <c r="G173" s="4" t="s">
+      <c r="F180" s="3"/>
+      <c r="G180" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H173" s="4" t="s">
+      <c r="H180" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I173" s="3"/>
-    </row>
-    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A174" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="B174" s="5"/>
-      <c r="C174" s="5"/>
-      <c r="D174" s="5"/>
-      <c r="E174" s="5"/>
-      <c r="F174" s="5"/>
-      <c r="G174" s="5"/>
-      <c r="H174" s="5"/>
-      <c r="I174" s="5"/>
-    </row>
-    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A175" s="12" t="s">
-        <v>321</v>
-      </c>
-      <c r="B175" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C175" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D175" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E175" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F175" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G175" s="12" t="n">
-        <v>20001</v>
-      </c>
-      <c r="H175" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I175" s="12" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="12" t="s">
-        <v>324</v>
-      </c>
-      <c r="B176" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C176" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D176" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E176" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F176" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G176" s="12" t="n">
-        <v>20002</v>
-      </c>
-      <c r="H176" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I176" s="12" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="12" t="s">
-        <v>325</v>
-      </c>
-      <c r="B177" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C177" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D177" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E177" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F177" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G177" s="12" t="n">
-        <v>20003</v>
-      </c>
-      <c r="H177" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I177" s="12" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="12" t="s">
-        <v>326</v>
-      </c>
-      <c r="B178" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C178" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D178" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E178" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F178" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G178" s="12" t="n">
-        <v>20004</v>
-      </c>
-      <c r="H178" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I178" s="12" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="12" t="s">
-        <v>327</v>
-      </c>
-      <c r="B179" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C179" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D179" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E179" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F179" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G179" s="12" t="n">
-        <v>20005</v>
-      </c>
-      <c r="H179" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I179" s="12" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A180" s="12" t="s">
-        <v>328</v>
-      </c>
-      <c r="B180" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C180" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D180" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E180" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F180" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G180" s="12" t="n">
-        <v>20006</v>
-      </c>
-      <c r="H180" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I180" s="12" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A181" s="12" t="s">
+      <c r="I180" s="3"/>
+    </row>
+    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A181" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="B181" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C181" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D181" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E181" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F181" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G181" s="12" t="n">
-        <v>20007</v>
-      </c>
-      <c r="H181" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I181" s="12" t="s">
-        <v>323</v>
-      </c>
+      <c r="B181" s="5"/>
+      <c r="C181" s="5"/>
+      <c r="D181" s="5"/>
+      <c r="E181" s="5"/>
+      <c r="F181" s="5"/>
+      <c r="G181" s="5"/>
+      <c r="H181" s="5"/>
+      <c r="I181" s="5"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="12" t="s">
@@ -11720,79 +11738,79 @@
         <v>75</v>
       </c>
       <c r="F182" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G182" s="12" t="n">
-        <v>20008</v>
+        <v>20001</v>
       </c>
       <c r="H182" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I182" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="B183" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C183" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D183" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E183" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F183" s="12" t="s">
         <v>331</v>
       </c>
-      <c r="B183" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C183" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D183" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E183" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F183" s="12" t="s">
-        <v>322</v>
-      </c>
       <c r="G183" s="12" t="n">
-        <v>30001</v>
+        <v>20002</v>
       </c>
       <c r="H183" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I183" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="12" t="s">
+        <v>334</v>
+      </c>
+      <c r="B184" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C184" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D184" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E184" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F184" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G184" s="12" t="n">
+        <v>20003</v>
+      </c>
+      <c r="H184" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I184" s="12" t="s">
         <v>332</v>
-      </c>
-      <c r="B184" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C184" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D184" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E184" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F184" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G184" s="12" t="n">
-        <v>30002</v>
-      </c>
-      <c r="H184" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I184" s="12" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="12" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B185" s="12" t="s">
         <v>75</v>
@@ -11807,21 +11825,21 @@
         <v>75</v>
       </c>
       <c r="F185" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G185" s="12" t="n">
-        <v>30003</v>
+        <v>20004</v>
       </c>
       <c r="H185" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I185" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="12" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B186" s="12" t="s">
         <v>75</v>
@@ -11836,21 +11854,21 @@
         <v>75</v>
       </c>
       <c r="F186" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G186" s="12" t="n">
-        <v>30004</v>
+        <v>20005</v>
       </c>
       <c r="H186" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I186" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="12" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B187" s="12" t="s">
         <v>75</v>
@@ -11865,21 +11883,21 @@
         <v>75</v>
       </c>
       <c r="F187" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G187" s="12" t="n">
-        <v>30005</v>
+        <v>20006</v>
       </c>
       <c r="H187" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I187" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="12" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B188" s="12" t="s">
         <v>75</v>
@@ -11894,21 +11912,21 @@
         <v>75</v>
       </c>
       <c r="F188" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G188" s="12" t="n">
-        <v>30006</v>
+        <v>20007</v>
       </c>
       <c r="H188" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I188" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="12" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B189" s="12" t="s">
         <v>75</v>
@@ -11923,21 +11941,21 @@
         <v>75</v>
       </c>
       <c r="F189" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G189" s="12" t="n">
-        <v>40001</v>
+        <v>20008</v>
       </c>
       <c r="H189" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I189" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="12" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B190" s="12" t="s">
         <v>75</v>
@@ -11952,21 +11970,21 @@
         <v>75</v>
       </c>
       <c r="F190" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G190" s="12" t="n">
-        <v>60001</v>
+        <v>30001</v>
       </c>
       <c r="H190" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I190" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="12" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B191" s="12" t="s">
         <v>75</v>
@@ -11981,21 +11999,21 @@
         <v>75</v>
       </c>
       <c r="F191" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G191" s="12" t="n">
-        <v>60002</v>
+        <v>30002</v>
       </c>
       <c r="H191" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I191" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="12" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B192" s="12" t="s">
         <v>75</v>
@@ -12010,21 +12028,21 @@
         <v>75</v>
       </c>
       <c r="F192" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G192" s="12" t="n">
-        <v>60003</v>
+        <v>30003</v>
       </c>
       <c r="H192" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I192" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B193" s="12" t="s">
         <v>75</v>
@@ -12039,21 +12057,21 @@
         <v>75</v>
       </c>
       <c r="F193" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G193" s="12" t="n">
-        <v>60004</v>
+        <v>30004</v>
       </c>
       <c r="H193" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I193" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B194" s="12" t="s">
         <v>75</v>
@@ -12068,21 +12086,21 @@
         <v>75</v>
       </c>
       <c r="F194" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G194" s="12" t="n">
-        <v>60005</v>
+        <v>30005</v>
       </c>
       <c r="H194" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I194" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="12" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B195" s="12" t="s">
         <v>75</v>
@@ -12097,21 +12115,21 @@
         <v>75</v>
       </c>
       <c r="F195" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G195" s="12" t="n">
-        <v>60006</v>
+        <v>30006</v>
       </c>
       <c r="H195" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I195" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="12" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B196" s="12" t="s">
         <v>75</v>
@@ -12126,21 +12144,21 @@
         <v>75</v>
       </c>
       <c r="F196" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G196" s="12" t="n">
-        <v>60007</v>
+        <v>40001</v>
       </c>
       <c r="H196" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I196" s="12" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="12" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B197" s="12" t="s">
         <v>75</v>
@@ -12155,287 +12173,287 @@
         <v>75</v>
       </c>
       <c r="F197" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G197" s="12" t="n">
+        <v>60001</v>
+      </c>
+      <c r="H197" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I197" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A198" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="B198" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C198" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D198" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E198" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F198" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G198" s="12" t="n">
+        <v>60002</v>
+      </c>
+      <c r="H198" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I198" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A199" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="B199" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C199" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D199" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E199" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F199" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G199" s="12" t="n">
+        <v>60003</v>
+      </c>
+      <c r="H199" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I199" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A200" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="B200" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C200" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D200" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E200" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F200" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G200" s="12" t="n">
+        <v>60004</v>
+      </c>
+      <c r="H200" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I200" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A201" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="B201" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C201" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D201" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E201" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F201" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G201" s="12" t="n">
+        <v>60005</v>
+      </c>
+      <c r="H201" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I201" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A202" s="12" t="s">
+        <v>352</v>
+      </c>
+      <c r="B202" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C202" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D202" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E202" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F202" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G202" s="12" t="n">
+        <v>60006</v>
+      </c>
+      <c r="H202" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I202" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A203" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="B203" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C203" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D203" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E203" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F203" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G203" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H203" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I203" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A204" s="12" t="s">
+        <v>354</v>
+      </c>
+      <c r="B204" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C204" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D204" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E204" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F204" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G204" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H197" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I197" s="12" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A198" s="3" t="s">
+      <c r="H204" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I204" s="12" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="205" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A205" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B198" s="4" t="s">
+      <c r="B205" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C198" s="4" t="s">
+      <c r="C205" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D198" s="3" t="s">
+      <c r="D205" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E198" s="4" t="s">
+      <c r="E205" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F198" s="3" t="s">
+      <c r="F205" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G198" s="4" t="s">
+      <c r="G205" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H198" s="4" t="s">
+      <c r="H205" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I198" s="3" t="s">
+      <c r="I205" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A199" s="3"/>
-      <c r="B199" s="4" t="s">
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A206" s="3"/>
+      <c r="B206" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C199" s="4" t="s">
+      <c r="C206" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D199" s="3"/>
-      <c r="E199" s="4" t="s">
+      <c r="D206" s="3"/>
+      <c r="E206" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F199" s="3"/>
-      <c r="G199" s="4" t="s">
+      <c r="F206" s="3"/>
+      <c r="G206" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H199" s="4" t="s">
+      <c r="H206" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I199" s="3"/>
-    </row>
-    <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A200" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="B200" s="5"/>
-      <c r="C200" s="5"/>
-      <c r="D200" s="5"/>
-      <c r="E200" s="5"/>
-      <c r="F200" s="5"/>
-      <c r="G200" s="5"/>
-      <c r="H200" s="5"/>
-      <c r="I200" s="5"/>
-    </row>
-    <row r="201" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A201" s="12" t="s">
-        <v>331</v>
-      </c>
-      <c r="B201" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C201" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D201" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E201" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F201" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G201" s="12" t="n">
-        <v>30001</v>
-      </c>
-      <c r="H201" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I201" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="202" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A202" s="12" t="s">
-        <v>332</v>
-      </c>
-      <c r="B202" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C202" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D202" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E202" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F202" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G202" s="12" t="n">
-        <v>30002</v>
-      </c>
-      <c r="H202" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I202" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="203" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A203" s="12" t="s">
-        <v>333</v>
-      </c>
-      <c r="B203" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C203" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D203" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E203" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F203" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G203" s="12" t="n">
-        <v>30003</v>
-      </c>
-      <c r="H203" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I203" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="204" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A204" s="12" t="s">
-        <v>334</v>
-      </c>
-      <c r="B204" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C204" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D204" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E204" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F204" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G204" s="12" t="n">
-        <v>30004</v>
-      </c>
-      <c r="H204" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I204" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="205" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A205" s="12" t="s">
-        <v>335</v>
-      </c>
-      <c r="B205" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C205" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D205" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E205" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F205" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G205" s="12" t="n">
-        <v>30005</v>
-      </c>
-      <c r="H205" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I205" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="206" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A206" s="12" t="s">
-        <v>336</v>
-      </c>
-      <c r="B206" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C206" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D206" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E206" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F206" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G206" s="12" t="n">
-        <v>30006</v>
-      </c>
-      <c r="H206" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I206" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A207" s="12" t="s">
-        <v>337</v>
-      </c>
-      <c r="B207" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C207" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="D207" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E207" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F207" s="12" t="s">
-        <v>322</v>
-      </c>
-      <c r="G207" s="12" t="n">
-        <v>40001</v>
-      </c>
-      <c r="H207" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I207" s="12" t="s">
-        <v>323</v>
-      </c>
+      <c r="I206" s="3"/>
+    </row>
+    <row r="207" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A207" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="B207" s="5"/>
+      <c r="C207" s="5"/>
+      <c r="D207" s="5"/>
+      <c r="E207" s="5"/>
+      <c r="F207" s="5"/>
+      <c r="G207" s="5"/>
+      <c r="H207" s="5"/>
+      <c r="I207" s="5"/>
     </row>
     <row r="208" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="12" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="B208" s="12" t="s">
         <v>75</v>
@@ -12450,21 +12468,21 @@
         <v>75</v>
       </c>
       <c r="F208" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G208" s="12" t="n">
-        <v>45001</v>
+        <v>30001</v>
       </c>
       <c r="H208" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I208" s="12" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="12" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B209" s="12" t="s">
         <v>75</v>
@@ -12479,21 +12497,21 @@
         <v>75</v>
       </c>
       <c r="F209" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G209" s="12" t="n">
-        <v>60001</v>
+        <v>30002</v>
       </c>
       <c r="H209" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I209" s="12" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="12" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B210" s="12" t="s">
         <v>75</v>
@@ -12508,21 +12526,21 @@
         <v>75</v>
       </c>
       <c r="F210" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G210" s="12" t="n">
-        <v>60002</v>
+        <v>30003</v>
       </c>
       <c r="H210" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I210" s="12" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="12" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B211" s="12" t="s">
         <v>75</v>
@@ -12537,21 +12555,21 @@
         <v>75</v>
       </c>
       <c r="F211" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G211" s="12" t="n">
-        <v>60003</v>
+        <v>30004</v>
       </c>
       <c r="H211" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I211" s="12" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="12" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B212" s="12" t="s">
         <v>75</v>
@@ -12566,21 +12584,21 @@
         <v>75</v>
       </c>
       <c r="F212" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G212" s="12" t="n">
-        <v>60004</v>
+        <v>30005</v>
       </c>
       <c r="H212" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I212" s="12" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="12" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B213" s="12" t="s">
         <v>75</v>
@@ -12595,21 +12613,21 @@
         <v>75</v>
       </c>
       <c r="F213" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G213" s="12" t="n">
-        <v>60005</v>
+        <v>30006</v>
       </c>
       <c r="H213" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I213" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="214" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="12" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B214" s="12" t="s">
         <v>75</v>
@@ -12624,21 +12642,21 @@
         <v>75</v>
       </c>
       <c r="F214" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G214" s="12" t="n">
-        <v>60006</v>
+        <v>40001</v>
       </c>
       <c r="H214" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I214" s="12" t="s">
-        <v>347</v>
+        <v>332</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="12" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
       <c r="B215" s="12" t="s">
         <v>75</v>
@@ -12653,21 +12671,21 @@
         <v>75</v>
       </c>
       <c r="F215" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G215" s="12" t="n">
-        <v>60007</v>
+        <v>45001</v>
       </c>
       <c r="H215" s="12" t="n">
         <v>1</v>
       </c>
       <c r="I215" s="12" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="12" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B216" s="12" t="s">
         <v>75</v>
@@ -12682,277 +12700,287 @@
         <v>75</v>
       </c>
       <c r="F216" s="12" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
       <c r="G216" s="12" t="n">
+        <v>60001</v>
+      </c>
+      <c r="H216" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I216" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="B217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C217" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E217" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F217" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G217" s="12" t="n">
+        <v>60002</v>
+      </c>
+      <c r="H217" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I217" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="B218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C218" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E218" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F218" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G218" s="12" t="n">
+        <v>60003</v>
+      </c>
+      <c r="H218" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I218" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="B219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C219" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E219" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F219" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G219" s="12" t="n">
+        <v>60004</v>
+      </c>
+      <c r="H219" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I219" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="12" t="s">
+        <v>351</v>
+      </c>
+      <c r="B220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C220" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E220" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F220" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G220" s="12" t="n">
+        <v>60005</v>
+      </c>
+      <c r="H220" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I220" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="12" t="s">
+        <v>352</v>
+      </c>
+      <c r="B221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C221" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E221" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F221" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G221" s="12" t="n">
+        <v>60006</v>
+      </c>
+      <c r="H221" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I221" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="B222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C222" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E222" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F222" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G222" s="12" t="n">
+        <v>60007</v>
+      </c>
+      <c r="H222" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I222" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="19.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="12" t="s">
+        <v>354</v>
+      </c>
+      <c r="B223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C223" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E223" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F223" s="12" t="s">
+        <v>331</v>
+      </c>
+      <c r="G223" s="12" t="n">
         <v>60008</v>
       </c>
-      <c r="H216" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I216" s="12" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A217" s="3" t="s">
+      <c r="H223" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I223" s="12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A224" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B217" s="4" t="s">
+      <c r="B224" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C217" s="4" t="s">
+      <c r="C224" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D217" s="3" t="s">
+      <c r="D224" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E217" s="4" t="s">
+      <c r="E224" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F217" s="3" t="s">
+      <c r="F224" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G217" s="4" t="s">
+      <c r="G224" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H217" s="4" t="s">
+      <c r="H224" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I217" s="3" t="s">
+      <c r="I224" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A218" s="3"/>
-      <c r="B218" s="4" t="s">
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="3"/>
+      <c r="B225" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C218" s="4" t="s">
+      <c r="C225" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D218" s="3"/>
-      <c r="E218" s="4" t="s">
+      <c r="D225" s="3"/>
+      <c r="E225" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F218" s="3"/>
-      <c r="G218" s="4" t="s">
+      <c r="F225" s="3"/>
+      <c r="G225" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H218" s="4" t="s">
+      <c r="H225" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="I218" s="3"/>
-    </row>
-    <row r="219" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A219" s="5" t="s">
+      <c r="I225" s="3"/>
+    </row>
+    <row r="226" customFormat="false" ht="10.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A226" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="B219" s="5"/>
-      <c r="C219" s="5"/>
-      <c r="D219" s="5"/>
-      <c r="E219" s="5"/>
-      <c r="F219" s="5"/>
-      <c r="G219" s="5"/>
-      <c r="H219" s="5"/>
-      <c r="I219" s="5"/>
-    </row>
-    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A220" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B220" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C220" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D220" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E220" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F220" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G220" s="10" t="s">
-        <v>303</v>
-      </c>
-      <c r="H220" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I220" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A221" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="B221" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C221" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D221" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E221" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F221" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G221" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="H221" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I221" s="7" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A222" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="B222" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C222" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D222" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E222" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F222" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G222" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="H222" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I222" s="7"/>
-    </row>
-    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A223" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="B223" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C223" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D223" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E223" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F223" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G223" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="H223" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I223" s="7"/>
-    </row>
-    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A224" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="B224" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C224" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D224" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E224" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F224" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G224" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="H224" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I224" s="7"/>
-    </row>
-    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A225" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="B225" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C225" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D225" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E225" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F225" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G225" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="H225" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I225" s="7"/>
-    </row>
-    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A226" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="B226" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C226" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D226" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="E226" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F226" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="G226" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="H226" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I226" s="7"/>
+      <c r="B226" s="5"/>
+      <c r="C226" s="5"/>
+      <c r="D226" s="5"/>
+      <c r="E226" s="5"/>
+      <c r="F226" s="5"/>
+      <c r="G226" s="5"/>
+      <c r="H226" s="5"/>
+      <c r="I226" s="5"/>
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="9" t="s">
-        <v>207</v>
+        <v>108</v>
       </c>
       <c r="B227" s="7" t="s">
         <v>109</v>
@@ -12970,19 +12998,21 @@
         <v>26</v>
       </c>
       <c r="G227" s="10" t="s">
-        <v>208</v>
+        <v>303</v>
       </c>
       <c r="H227" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I227" s="7"/>
+      <c r="I227" s="7" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="9" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="B228" s="7" t="s">
-        <v>24</v>
+        <v>109</v>
       </c>
       <c r="C228" s="7" t="s">
         <v>110</v>
@@ -12997,16 +13027,18 @@
         <v>26</v>
       </c>
       <c r="G228" s="10" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="H228" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I228" s="7"/>
+      <c r="I228" s="7" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="9" t="s">
-        <v>211</v>
+        <v>197</v>
       </c>
       <c r="B229" s="7" t="s">
         <v>24</v>
@@ -13024,7 +13056,7 @@
         <v>26</v>
       </c>
       <c r="G229" s="10" t="s">
-        <v>212</v>
+        <v>198</v>
       </c>
       <c r="H229" s="7" t="n">
         <v>2</v>
@@ -13033,7 +13065,7 @@
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="9" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="B230" s="7" t="s">
         <v>24</v>
@@ -13051,7 +13083,7 @@
         <v>26</v>
       </c>
       <c r="G230" s="10" t="s">
-        <v>214</v>
+        <v>200</v>
       </c>
       <c r="H230" s="7" t="n">
         <v>2</v>
@@ -13060,7 +13092,7 @@
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="9" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="B231" s="7" t="s">
         <v>24</v>
@@ -13078,7 +13110,7 @@
         <v>26</v>
       </c>
       <c r="G231" s="10" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
       <c r="H231" s="7" t="n">
         <v>2</v>
@@ -13087,10 +13119,10 @@
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="9" t="s">
-        <v>217</v>
+        <v>203</v>
       </c>
       <c r="B232" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C232" s="7" t="s">
         <v>110</v>
@@ -13105,7 +13137,7 @@
         <v>26</v>
       </c>
       <c r="G232" s="10" t="s">
-        <v>218</v>
+        <v>204</v>
       </c>
       <c r="H232" s="7" t="n">
         <v>2</v>
@@ -13114,7 +13146,7 @@
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="9" t="s">
-        <v>219</v>
+        <v>205</v>
       </c>
       <c r="B233" s="7" t="s">
         <v>109</v>
@@ -13132,7 +13164,7 @@
         <v>26</v>
       </c>
       <c r="G233" s="10" t="s">
-        <v>220</v>
+        <v>206</v>
       </c>
       <c r="H233" s="7" t="n">
         <v>2</v>
@@ -13141,10 +13173,10 @@
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="9" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="B234" s="7" t="s">
-        <v>222</v>
+        <v>109</v>
       </c>
       <c r="C234" s="7" t="s">
         <v>110</v>
@@ -13159,7 +13191,7 @@
         <v>26</v>
       </c>
       <c r="G234" s="10" t="s">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="H234" s="7" t="n">
         <v>2</v>
@@ -13168,10 +13200,10 @@
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="9" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="B235" s="7" t="s">
-        <v>222</v>
+        <v>24</v>
       </c>
       <c r="C235" s="7" t="s">
         <v>110</v>
@@ -13186,7 +13218,7 @@
         <v>26</v>
       </c>
       <c r="G235" s="10" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="H235" s="7" t="n">
         <v>2</v>
@@ -13195,10 +13227,10 @@
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="9" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="B236" s="7" t="s">
-        <v>195</v>
+        <v>24</v>
       </c>
       <c r="C236" s="7" t="s">
         <v>110</v>
@@ -13213,7 +13245,7 @@
         <v>26</v>
       </c>
       <c r="G236" s="10" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="H236" s="7" t="n">
         <v>2</v>
@@ -13222,10 +13254,10 @@
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="9" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="B237" s="7" t="s">
-        <v>195</v>
+        <v>24</v>
       </c>
       <c r="C237" s="7" t="s">
         <v>110</v>
@@ -13240,7 +13272,7 @@
         <v>26</v>
       </c>
       <c r="G237" s="10" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="H237" s="7" t="n">
         <v>2</v>
@@ -13249,10 +13281,10 @@
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="9" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="B238" s="7" t="s">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="C238" s="7" t="s">
         <v>110</v>
@@ -13267,7 +13299,7 @@
         <v>26</v>
       </c>
       <c r="G238" s="10" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="H238" s="7" t="n">
         <v>2</v>
@@ -13276,7 +13308,7 @@
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="9" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="B239" s="7" t="s">
         <v>109</v>
@@ -13294,7 +13326,7 @@
         <v>26</v>
       </c>
       <c r="G239" s="10" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="H239" s="7" t="n">
         <v>2</v>
@@ -13302,11 +13334,11 @@
       <c r="I239" s="7"/>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A240" s="7" t="s">
-        <v>304</v>
+      <c r="A240" s="9" t="s">
+        <v>219</v>
       </c>
       <c r="B240" s="7" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="C240" s="7" t="s">
         <v>110</v>
@@ -13321,21 +13353,19 @@
         <v>26</v>
       </c>
       <c r="G240" s="10" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="H240" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="I240" s="7" t="s">
-        <v>236</v>
-      </c>
+      <c r="I240" s="7"/>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A241" s="7" t="s">
-        <v>237</v>
+      <c r="A241" s="9" t="s">
+        <v>221</v>
       </c>
       <c r="B241" s="7" t="s">
-        <v>75</v>
+        <v>222</v>
       </c>
       <c r="C241" s="7" t="s">
         <v>110</v>
@@ -13350,197 +13380,409 @@
         <v>26</v>
       </c>
       <c r="G241" s="10" t="s">
+        <v>223</v>
+      </c>
+      <c r="H241" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I241" s="7"/>
+    </row>
+    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A242" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="B242" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="C242" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D242" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E242" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F242" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G242" s="10" t="s">
+        <v>225</v>
+      </c>
+      <c r="H242" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I242" s="7"/>
+    </row>
+    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A243" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="B243" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C243" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D243" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E243" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F243" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G243" s="10" t="s">
+        <v>227</v>
+      </c>
+      <c r="H243" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I243" s="7"/>
+    </row>
+    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A244" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="B244" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="C244" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D244" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E244" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F244" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G244" s="10" t="s">
+        <v>229</v>
+      </c>
+      <c r="H244" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I244" s="7"/>
+    </row>
+    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A245" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B245" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C245" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D245" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E245" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F245" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G245" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="H245" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I245" s="7"/>
+    </row>
+    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A246" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="B246" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C246" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D246" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E246" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F246" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G246" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="H246" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I246" s="7"/>
+    </row>
+    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A247" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="B247" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C247" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D247" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E247" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F247" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G247" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="H247" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I247" s="7" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A248" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="B248" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C248" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D248" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E248" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F248" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G248" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="H241" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="I241" s="7" t="s">
+      <c r="H248" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I248" s="7" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A242" s="12" t="s">
+    <row r="249" customFormat="false" ht="29.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A249" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="B249" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C249" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D249" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E249" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F249" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G249" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="H249" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I249" s="7" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="250" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A250" s="12" t="s">
         <v>240</v>
       </c>
-      <c r="B242" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C242" s="12" t="s">
+      <c r="B250" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C250" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D242" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E242" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F242" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G242" s="12" t="s">
+      <c r="D250" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E250" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F250" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G250" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="H242" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I242" s="12" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="243" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A243" s="12" t="s">
+      <c r="H250" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I250" s="12" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="251" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A251" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="B243" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C243" s="12" t="s">
+      <c r="B251" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C251" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D243" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E243" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F243" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G243" s="12" t="s">
+      <c r="D251" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E251" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F251" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G251" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="H243" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I243" s="12" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="244" customFormat="false" ht="45.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A244" s="11" t="s">
-        <v>308</v>
-      </c>
-      <c r="B244" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C244" s="12" t="s">
+      <c r="H251" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I251" s="12" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="252" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A252" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="B252" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C252" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D244" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E244" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F244" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G244" s="13" t="s">
-        <v>309</v>
-      </c>
-      <c r="H244" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I244" s="12" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="245" customFormat="false" ht="36.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A245" s="11" t="s">
-        <v>311</v>
-      </c>
-      <c r="B245" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C245" s="12" t="s">
+      <c r="D252" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E252" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F252" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G252" s="13" t="s">
+        <v>312</v>
+      </c>
+      <c r="H252" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I252" s="12" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="253" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A253" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="B253" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C253" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D245" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E245" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F245" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G245" s="13" t="s">
-        <v>312</v>
-      </c>
-      <c r="H245" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I245" s="12" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="246" customFormat="false" ht="27.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A246" s="11" t="s">
-        <v>353</v>
-      </c>
-      <c r="B246" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C246" s="12" t="s">
+      <c r="D253" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E253" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F253" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G253" s="13" t="s">
+        <v>315</v>
+      </c>
+      <c r="H253" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I253" s="12" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="254" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A254" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="B254" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C254" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D246" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E246" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F246" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G246" s="13" t="s">
-        <v>315</v>
-      </c>
-      <c r="H246" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I246" s="12" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="247" customFormat="false" ht="28.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A247" s="11" t="s">
-        <v>317</v>
-      </c>
-      <c r="B247" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="C247" s="12" t="s">
+      <c r="D254" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E254" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F254" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G254" s="13" t="s">
+        <v>318</v>
+      </c>
+      <c r="H254" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I254" s="12" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="255" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A255" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="B255" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C255" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D247" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E247" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F247" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="G247" s="13" t="s">
-        <v>318</v>
-      </c>
-      <c r="H247" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="I247" s="12" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="1048558" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048559" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048560" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048561" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048562" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048563" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="D255" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E255" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F255" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G255" s="13" t="s">
+        <v>321</v>
+      </c>
+      <c r="H255" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I255" s="12" t="s">
+        <v>322</v>
+      </c>
+    </row>
     <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -13559,26 +13801,26 @@
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="A8:I8"/>
-    <mergeCell ref="A116:A117"/>
-    <mergeCell ref="D116:D117"/>
-    <mergeCell ref="F116:F117"/>
-    <mergeCell ref="I116:I117"/>
-    <mergeCell ref="A118:I118"/>
-    <mergeCell ref="A172:A173"/>
-    <mergeCell ref="D172:D173"/>
-    <mergeCell ref="F172:F173"/>
-    <mergeCell ref="I172:I173"/>
-    <mergeCell ref="A174:I174"/>
-    <mergeCell ref="A198:A199"/>
-    <mergeCell ref="D198:D199"/>
-    <mergeCell ref="F198:F199"/>
-    <mergeCell ref="I198:I199"/>
-    <mergeCell ref="A200:I200"/>
-    <mergeCell ref="A217:A218"/>
-    <mergeCell ref="D217:D218"/>
-    <mergeCell ref="F217:F218"/>
-    <mergeCell ref="I217:I218"/>
-    <mergeCell ref="A219:I219"/>
+    <mergeCell ref="A117:A118"/>
+    <mergeCell ref="D117:D118"/>
+    <mergeCell ref="F117:F118"/>
+    <mergeCell ref="I117:I118"/>
+    <mergeCell ref="A119:I119"/>
+    <mergeCell ref="A179:A180"/>
+    <mergeCell ref="D179:D180"/>
+    <mergeCell ref="F179:F180"/>
+    <mergeCell ref="I179:I180"/>
+    <mergeCell ref="A181:I181"/>
+    <mergeCell ref="A205:A206"/>
+    <mergeCell ref="D205:D206"/>
+    <mergeCell ref="F205:F206"/>
+    <mergeCell ref="I205:I206"/>
+    <mergeCell ref="A207:I207"/>
+    <mergeCell ref="A224:A225"/>
+    <mergeCell ref="D224:D225"/>
+    <mergeCell ref="F224:F225"/>
+    <mergeCell ref="I224:I225"/>
+    <mergeCell ref="A226:I226"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -13614,7 +13856,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>355</v>
+        <v>365</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13622,7 +13864,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>356</v>
+        <v>366</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13643,10 +13885,10 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>357</v>
+        <v>367</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>358</v>
+        <v>368</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13701,7 +13943,7 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>359</v>
+        <v>369</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="16"/>
@@ -13714,7 +13956,7 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>360</v>
+        <v>370</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>195</v>
@@ -13732,18 +13974,18 @@
         <v>26</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>361</v>
+        <v>371</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>362</v>
+        <v>372</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>363</v>
+        <v>373</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>195</v>
@@ -13761,18 +14003,18 @@
         <v>26</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>364</v>
+        <v>374</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>365</v>
+        <v>375</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>366</v>
+        <v>376</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>24</v>
@@ -13790,18 +14032,18 @@
         <v>26</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>367</v>
+        <v>377</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>368</v>
+        <v>378</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>369</v>
+        <v>379</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>75</v>
@@ -13819,18 +14061,18 @@
         <v>26</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>370</v>
+        <v>380</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>371</v>
+        <v>381</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>75</v>
@@ -13848,18 +14090,18 @@
         <v>26</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>372</v>
+        <v>382</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>75</v>
@@ -13877,18 +14119,18 @@
         <v>26</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>374</v>
+        <v>384</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>75</v>
@@ -13906,18 +14148,18 @@
         <v>26</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>375</v>
+        <v>385</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="B17" s="7" t="s">
         <v>75</v>
@@ -13935,18 +14177,18 @@
         <v>26</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>376</v>
+        <v>386</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>2</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>373</v>
+        <v>383</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>377</v>
+        <v>387</v>
       </c>
       <c r="B20" s="16"/>
       <c r="C20" s="16"/>
@@ -13959,7 +14201,7 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>378</v>
+        <v>388</v>
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -13972,7 +14214,7 @@
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>379</v>
+        <v>389</v>
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>
@@ -13985,7 +14227,7 @@
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>380</v>
+        <v>390</v>
       </c>
       <c r="B23" s="17"/>
       <c r="C23" s="17"/>
@@ -13998,7 +14240,7 @@
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>381</v>
+        <v>391</v>
       </c>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>
@@ -14011,7 +14253,7 @@
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -14024,7 +14266,7 @@
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>383</v>
+        <v>393</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
@@ -14037,7 +14279,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>384</v>
+        <v>394</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -14050,7 +14292,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -14063,7 +14305,7 @@
     </row>
     <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>386</v>
+        <v>396</v>
       </c>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>

</xml_diff>

<commit_message>
SOCO: Improv: Add 100A calibration
Added calibration at 100A also, the highest current point.
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -8054,6 +8054,7 @@
     <mergeCell ref="D174:D175"/>
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="F174:F175"/>
+    <mergeCell ref="A6:A7"/>
     <mergeCell ref="I174:I175"/>
     <mergeCell ref="D112:D113"/>
     <mergeCell ref="I6:I7"/>
@@ -8062,9 +8063,8 @@
     <mergeCell ref="A8:I8"/>
     <mergeCell ref="A176:I176"/>
     <mergeCell ref="A114:I114"/>
+    <mergeCell ref="A112:A113"/>
     <mergeCell ref="F6:F7"/>
-    <mergeCell ref="A112:A113"/>
-    <mergeCell ref="A6:A7"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -12274,14 +12274,16 @@
         <is>
           <t>Internal Only. Not visible to customer. 
 Indicates the state machine of calibration
-0: Calibration Not Initiated. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 20A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
-17,18,19,20: High Point Calibration In Progress
-21: High Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
-22,23,24: Mid Point Calibration In Progress
-25: Mid Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 0.4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
-26,27,28: Low Point Calibration In Progress
-29: Low Point Calibration Done. Set Fan 1 Current and Fan 2 Current to 0.1A each. And then set Advance Calibration Flag.
-30: Fan Calibration In Progress
+0: Calibration Not Initiated. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 100A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
+17,18,19,20: Extra-High Point Calibration In Progress (V/I + PF at 100A)
+21: Extra-High Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 20A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
+22,23,24: High Point Calibration In Progress
+25: High Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
+26,27,28: Mid Point Calibration In Progress
+29: Mid Point Calibration Done. Set Grid R/Y/B and Solar R/Y/B Voltages to 240V. Set Grid R/Y/B and Solar R/Y/B current to 0.4A. Set Grid R/Y/B and Solar R/Y/B Power Factor to 0.5. And then set Advance Calibration Flag.
+30,31,32: Low Point Calibration In Progress
+33: Low Point Calibration Done. Set Fan 1 Current and Fan 2 Current to 0.1A each. And then set Advance Calibration Flag.
+34: Fan Calibration In Progress
 127: Calibration Completed Successfully
 126: Error occured during calibration. Please restart controller</t>
         </is>

</xml_diff>

<commit_message>
SOCO: Improv: Minor improv/fix in Modbus Excel Sheet
Also note, the current v2.17 code has been sent to one sample in UP
Jio live ite (Site installed).
</commit_message>
<xml_diff>
--- a/Document/SOCOModbusTable.xlsx
+++ b/Document/SOCOModbusTable.xlsx
@@ -4403,7 +4403,7 @@
     <row r="106" ht="15" customHeight="1" s="19">
       <c r="A106" s="27" t="inlineStr">
         <is>
-          <t>DG Detection Disable Setting</t>
+          <t>DG Detection Enable/Disable Setting</t>
         </is>
       </c>
       <c r="B106" s="27" t="inlineStr">
@@ -11872,7 +11872,7 @@
     <row r="106" ht="15" customHeight="1" s="19">
       <c r="A106" s="27" t="inlineStr">
         <is>
-          <t>DG Detection Disable Setting</t>
+          <t>DG Detection Enable/Disable Setting</t>
         </is>
       </c>
       <c r="B106" s="27" t="inlineStr">

</xml_diff>